<commit_message>
Excel actualizado automáticamente — 23/06/2026 11:55
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javo\APESTUDIO Dropbox\Carpeta del equipo APESTUDIO\999_PM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E71E38E-320B-4130-9462-66CDD9FC0033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EC9656-3F09-4A00-AC94-1D4F022C8453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Resumen Alejandra" sheetId="1" r:id="rId1"/>
@@ -1810,9 +1810,6 @@
     <t>Nela</t>
   </si>
   <si>
-    <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo)</t>
-  </si>
-  <si>
     <t>Montesquinza: cerrar entrega Consultores · Hermosilla: presionar Raumplan presupuesto · ⚠ No coge vacaciones agosto — disponible</t>
   </si>
   <si>
@@ -2066,6 +2063,9 @@
   </si>
   <si>
     <t>☐ Si hay hitos en agosto: verificado que no chocan con vacaciones Challan (1-15 ago)</t>
+  </si>
+  <si>
+    <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo), Alcala 58</t>
   </si>
 </sst>
 </file>
@@ -3338,20 +3338,41 @@
     <xf numFmtId="0" fontId="62" fillId="60" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="39" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="38" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3372,71 +3393,50 @@
     <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="48" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="39" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="49" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="58" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="48" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="49" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="56" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="59" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="59" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="59" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="59" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3461,6 +3461,12 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="43" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="31" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3473,18 +3479,19 @@
     <xf numFmtId="0" fontId="48" fillId="53" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="43" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="45" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="45" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3506,13 +3513,6 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="45" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="45" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="46" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3558,26 +3558,26 @@
     <xf numFmtId="0" fontId="36" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="56" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="57" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="58" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="56" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="54" fillId="58" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="56" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="56" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="57" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3890,7 +3890,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="194" t="s">
+      <c r="A1" s="200" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="195"/>
@@ -3898,7 +3898,7 @@
       <c r="D1" s="196"/>
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="201" t="s">
+      <c r="A2" s="202" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="176"/>
@@ -3906,7 +3906,7 @@
       <c r="D2" s="176"/>
     </row>
     <row r="4" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="203" t="s">
+      <c r="A4" s="197" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="195"/>
@@ -4405,7 +4405,7 @@
       <c r="A43" s="145" t="s">
         <v>109</v>
       </c>
-      <c r="B43" s="202" t="s">
+      <c r="B43" s="203" t="s">
         <v>110</v>
       </c>
       <c r="C43" s="195"/>
@@ -4415,7 +4415,7 @@
       <c r="A44" s="158" t="s">
         <v>111</v>
       </c>
-      <c r="B44" s="199" t="s">
+      <c r="B44" s="198" t="s">
         <v>112</v>
       </c>
       <c r="C44" s="195"/>
@@ -4425,7 +4425,7 @@
       <c r="A45" s="159" t="s">
         <v>113</v>
       </c>
-      <c r="B45" s="197" t="s">
+      <c r="B45" s="201" t="s">
         <v>114</v>
       </c>
       <c r="C45" s="195"/>
@@ -4435,7 +4435,7 @@
       <c r="A46" s="158" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="199" t="s">
+      <c r="B46" s="198" t="s">
         <v>115</v>
       </c>
       <c r="C46" s="195"/>
@@ -4445,7 +4445,7 @@
       <c r="A47" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B47" s="198" t="s">
+      <c r="B47" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C47" s="195"/>
@@ -4455,7 +4455,7 @@
       <c r="A48" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B48" s="198" t="s">
+      <c r="B48" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C48" s="195"/>
@@ -4465,14 +4465,14 @@
       <c r="A49" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B49" s="198" t="s">
+      <c r="B49" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C49" s="195"/>
       <c r="D49" s="196"/>
     </row>
     <row r="50" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="200" t="s">
+      <c r="A50" s="199" t="s">
         <v>116</v>
       </c>
       <c r="B50" s="195"/>
@@ -4483,7 +4483,7 @@
       <c r="A51" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B51" s="198" t="s">
+      <c r="B51" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C51" s="195"/>
@@ -4493,7 +4493,7 @@
       <c r="A52" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B52" s="198" t="s">
+      <c r="B52" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C52" s="195"/>
@@ -4503,7 +4503,7 @@
       <c r="A53" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B53" s="198" t="s">
+      <c r="B53" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C53" s="195"/>
@@ -4513,7 +4513,7 @@
       <c r="A54" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B54" s="198" t="s">
+      <c r="B54" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C54" s="195"/>
@@ -4523,7 +4523,7 @@
       <c r="A55" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B55" s="198" t="s">
+      <c r="B55" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C55" s="195"/>
@@ -4533,7 +4533,7 @@
       <c r="A56" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B56" s="198" t="s">
+      <c r="B56" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C56" s="195"/>
@@ -4543,7 +4543,7 @@
       <c r="A57" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B57" s="198" t="s">
+      <c r="B57" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C57" s="195"/>
@@ -4553,14 +4553,14 @@
       <c r="A58" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B58" s="198" t="s">
+      <c r="B58" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C58" s="195"/>
       <c r="D58" s="196"/>
     </row>
     <row r="59" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="200" t="s">
+      <c r="A59" s="199" t="s">
         <v>116</v>
       </c>
       <c r="B59" s="195"/>
@@ -4571,7 +4571,7 @@
       <c r="A60" s="158" t="s">
         <v>116</v>
       </c>
-      <c r="B60" s="198" t="s">
+      <c r="B60" s="194" t="s">
         <v>117</v>
       </c>
       <c r="C60" s="195"/>
@@ -4692,6 +4692,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="B60:D60"/>
     <mergeCell ref="B57:D57"/>
     <mergeCell ref="A4:D4"/>
@@ -4704,18 +4716,6 @@
     <mergeCell ref="B51:D51"/>
     <mergeCell ref="B56:D56"/>
     <mergeCell ref="B58:D58"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4741,7 +4741,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="204" t="s">
+      <c r="A1" s="209" t="s">
         <v>139</v>
       </c>
       <c r="B1" s="176"/>
@@ -6368,18 +6368,18 @@
       <c r="C50" s="167" t="s">
         <v>5</v>
       </c>
-      <c r="D50" s="209" t="s">
+      <c r="D50" s="206" t="s">
         <v>375</v>
       </c>
-      <c r="E50" s="209" t="s">
+      <c r="E50" s="206" t="s">
         <v>376</v>
       </c>
-      <c r="F50" s="209"/>
-      <c r="G50" s="209"/>
-      <c r="H50" s="209"/>
-      <c r="I50" s="209"/>
-      <c r="J50" s="209"/>
-      <c r="K50" s="209"/>
+      <c r="F50" s="206"/>
+      <c r="G50" s="206"/>
+      <c r="H50" s="206"/>
+      <c r="I50" s="206"/>
+      <c r="J50" s="206"/>
+      <c r="K50" s="206"/>
     </row>
     <row r="51" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="168" t="s">
@@ -6391,7 +6391,7 @@
       <c r="C51" s="169" t="s">
         <v>233</v>
       </c>
-      <c r="D51" s="208" t="s">
+      <c r="D51" s="205" t="s">
         <v>378</v>
       </c>
       <c r="E51" s="195"/>
@@ -6399,7 +6399,7 @@
       <c r="G51" s="195"/>
       <c r="H51" s="195"/>
       <c r="I51" s="196"/>
-      <c r="J51" s="206" t="s">
+      <c r="J51" s="204" t="s">
         <v>351</v>
       </c>
       <c r="K51" s="196"/>
@@ -6422,7 +6422,7 @@
       <c r="G52" s="195"/>
       <c r="H52" s="195"/>
       <c r="I52" s="196"/>
-      <c r="J52" s="205" t="s">
+      <c r="J52" s="208" t="s">
         <v>351</v>
       </c>
       <c r="K52" s="196"/>
@@ -6437,7 +6437,7 @@
       <c r="C53" s="169" t="s">
         <v>30</v>
       </c>
-      <c r="D53" s="208" t="s">
+      <c r="D53" s="205" t="s">
         <v>382</v>
       </c>
       <c r="E53" s="195"/>
@@ -6445,7 +6445,7 @@
       <c r="G53" s="195"/>
       <c r="H53" s="195"/>
       <c r="I53" s="196"/>
-      <c r="J53" s="206" t="s">
+      <c r="J53" s="204" t="s">
         <v>313</v>
       </c>
       <c r="K53" s="196"/>
@@ -6468,7 +6468,7 @@
       <c r="G54" s="195"/>
       <c r="H54" s="195"/>
       <c r="I54" s="196"/>
-      <c r="J54" s="205" t="s">
+      <c r="J54" s="208" t="s">
         <v>313</v>
       </c>
       <c r="K54" s="196"/>
@@ -6483,7 +6483,7 @@
       <c r="C55" s="169" t="s">
         <v>47</v>
       </c>
-      <c r="D55" s="208" t="s">
+      <c r="D55" s="205" t="s">
         <v>385</v>
       </c>
       <c r="E55" s="195"/>
@@ -6491,7 +6491,7 @@
       <c r="G55" s="195"/>
       <c r="H55" s="195"/>
       <c r="I55" s="196"/>
-      <c r="J55" s="206" t="s">
+      <c r="J55" s="204" t="s">
         <v>351</v>
       </c>
       <c r="K55" s="196"/>
@@ -6514,7 +6514,7 @@
       <c r="G56" s="195"/>
       <c r="H56" s="195"/>
       <c r="I56" s="196"/>
-      <c r="J56" s="205" t="s">
+      <c r="J56" s="208" t="s">
         <v>351</v>
       </c>
       <c r="K56" s="196"/>
@@ -6529,7 +6529,7 @@
       <c r="C57" s="169" t="s">
         <v>389</v>
       </c>
-      <c r="D57" s="208" t="s">
+      <c r="D57" s="205" t="s">
         <v>390</v>
       </c>
       <c r="E57" s="195"/>
@@ -6537,7 +6537,7 @@
       <c r="G57" s="195"/>
       <c r="H57" s="195"/>
       <c r="I57" s="196"/>
-      <c r="J57" s="206" t="s">
+      <c r="J57" s="204" t="s">
         <v>391</v>
       </c>
       <c r="K57" s="196"/>
@@ -6560,7 +6560,7 @@
       <c r="G58" s="195"/>
       <c r="H58" s="195"/>
       <c r="I58" s="196"/>
-      <c r="J58" s="205" t="s">
+      <c r="J58" s="208" t="s">
         <v>351</v>
       </c>
       <c r="K58" s="196"/>
@@ -6575,7 +6575,7 @@
       <c r="C59" s="169" t="s">
         <v>305</v>
       </c>
-      <c r="D59" s="208" t="s">
+      <c r="D59" s="205" t="s">
         <v>395</v>
       </c>
       <c r="E59" s="195"/>
@@ -6583,7 +6583,7 @@
       <c r="G59" s="195"/>
       <c r="H59" s="195"/>
       <c r="I59" s="196"/>
-      <c r="J59" s="206" t="s">
+      <c r="J59" s="204" t="s">
         <v>351</v>
       </c>
       <c r="K59" s="196"/>
@@ -6606,7 +6606,7 @@
       <c r="G60" s="195"/>
       <c r="H60" s="195"/>
       <c r="I60" s="196"/>
-      <c r="J60" s="205" t="s">
+      <c r="J60" s="208" t="s">
         <v>351</v>
       </c>
       <c r="K60" s="196"/>
@@ -6621,7 +6621,7 @@
       <c r="C61" s="169" t="s">
         <v>305</v>
       </c>
-      <c r="D61" s="208" t="s">
+      <c r="D61" s="205" t="s">
         <v>398</v>
       </c>
       <c r="E61" s="195"/>
@@ -6629,7 +6629,7 @@
       <c r="G61" s="195"/>
       <c r="H61" s="195"/>
       <c r="I61" s="196"/>
-      <c r="J61" s="206" t="s">
+      <c r="J61" s="204" t="s">
         <v>351</v>
       </c>
       <c r="K61" s="196"/>
@@ -6652,7 +6652,7 @@
       <c r="G62" s="195"/>
       <c r="H62" s="195"/>
       <c r="I62" s="196"/>
-      <c r="J62" s="205" t="s">
+      <c r="J62" s="208" t="s">
         <v>351</v>
       </c>
       <c r="K62" s="196"/>
@@ -6667,7 +6667,7 @@
       <c r="C63" s="169" t="s">
         <v>305</v>
       </c>
-      <c r="D63" s="208" t="s">
+      <c r="D63" s="205" t="s">
         <v>402</v>
       </c>
       <c r="E63" s="195"/>
@@ -6675,7 +6675,7 @@
       <c r="G63" s="195"/>
       <c r="H63" s="195"/>
       <c r="I63" s="196"/>
-      <c r="J63" s="206" t="s">
+      <c r="J63" s="204" t="s">
         <v>351</v>
       </c>
       <c r="K63" s="196"/>
@@ -6705,6 +6705,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="J62:K62"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="J61:K61"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="D52:I52"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A48:L48"/>
+    <mergeCell ref="D57:I57"/>
+    <mergeCell ref="D61:I61"/>
+    <mergeCell ref="J57:K57"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="D53:I53"/>
+    <mergeCell ref="J60:K60"/>
     <mergeCell ref="J63:K63"/>
     <mergeCell ref="D59:I59"/>
     <mergeCell ref="D50:I50"/>
@@ -6721,22 +6737,6 @@
     <mergeCell ref="D51:I51"/>
     <mergeCell ref="J54:K54"/>
     <mergeCell ref="D54:I54"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="J62:K62"/>
-    <mergeCell ref="J51:K51"/>
-    <mergeCell ref="J61:K61"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="D52:I52"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="D57:I57"/>
-    <mergeCell ref="D61:I61"/>
-    <mergeCell ref="J57:K57"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="D53:I53"/>
-    <mergeCell ref="J60:K60"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6755,7 +6755,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="175" t="s">
+      <c r="A1" s="185" t="s">
         <v>404</v>
       </c>
       <c r="B1" s="176"/>
@@ -6779,27 +6779,27 @@
       <c r="T1" s="176"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="182"/>
+      <c r="A2" s="189"/>
       <c r="B2" s="176"/>
-      <c r="C2" s="177" t="s">
+      <c r="C2" s="186" t="s">
         <v>405</v>
       </c>
       <c r="D2" s="176"/>
       <c r="E2" s="176"/>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="188" t="s">
         <v>406</v>
       </c>
       <c r="G2" s="176"/>
       <c r="H2" s="176"/>
       <c r="I2" s="176"/>
       <c r="J2" s="176"/>
-      <c r="K2" s="193" t="s">
+      <c r="K2" s="184" t="s">
         <v>407</v>
       </c>
       <c r="L2" s="176"/>
       <c r="M2" s="176"/>
       <c r="N2" s="176"/>
-      <c r="O2" s="190" t="s">
+      <c r="O2" s="179" t="s">
         <v>408</v>
       </c>
       <c r="P2" s="176"/>
@@ -6871,7 +6871,7 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="186" t="s">
+      <c r="A4" s="193" t="s">
         <v>425</v>
       </c>
       <c r="B4" s="176"/>
@@ -6919,7 +6919,7 @@
       <c r="T4" s="11"/>
     </row>
     <row r="5" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="187" t="s">
+      <c r="A5" s="182" t="s">
         <v>148</v>
       </c>
       <c r="B5" s="176"/>
@@ -6953,7 +6953,7 @@
       <c r="D6" s="130" t="s">
         <v>174</v>
       </c>
-      <c r="E6" s="183" t="s">
+      <c r="E6" s="190" t="s">
         <v>181</v>
       </c>
       <c r="F6" s="176"/>
@@ -7028,7 +7028,7 @@
       <c r="I8" s="128"/>
       <c r="J8" s="134"/>
       <c r="K8" s="101"/>
-      <c r="L8" s="180" t="s">
+      <c r="L8" s="181" t="s">
         <v>428</v>
       </c>
       <c r="M8" s="176"/>
@@ -7129,7 +7129,7 @@
       <c r="J11" s="134"/>
       <c r="K11" s="101"/>
       <c r="L11" s="134"/>
-      <c r="M11" s="180" t="s">
+      <c r="M11" s="181" t="s">
         <v>428</v>
       </c>
       <c r="N11" s="176"/>
@@ -7213,12 +7213,12 @@
       <c r="B14" s="12" t="s">
         <v>439</v>
       </c>
-      <c r="C14" s="185" t="s">
+      <c r="C14" s="192" t="s">
         <v>174</v>
       </c>
       <c r="D14" s="176"/>
       <c r="E14" s="176"/>
-      <c r="F14" s="192" t="s">
+      <c r="F14" s="183" t="s">
         <v>181</v>
       </c>
       <c r="G14" s="176"/>
@@ -7390,7 +7390,7 @@
       <c r="E19" s="128"/>
       <c r="F19" s="120"/>
       <c r="G19" s="128"/>
-      <c r="H19" s="185" t="s">
+      <c r="H19" s="192" t="s">
         <v>174</v>
       </c>
       <c r="I19" s="176"/>
@@ -7431,7 +7431,7 @@
       <c r="J20" s="134"/>
       <c r="K20" s="101"/>
       <c r="L20" s="134"/>
-      <c r="M20" s="180" t="s">
+      <c r="M20" s="181" t="s">
         <v>428</v>
       </c>
       <c r="N20" s="176"/>
@@ -7497,7 +7497,7 @@
       <c r="H22" s="134"/>
       <c r="I22" s="134"/>
       <c r="J22" s="134"/>
-      <c r="K22" s="179" t="s">
+      <c r="K22" s="187" t="s">
         <v>428</v>
       </c>
       <c r="L22" s="176"/>
@@ -7521,7 +7521,7 @@
       <c r="B23" s="12" t="s">
         <v>446</v>
       </c>
-      <c r="C23" s="188" t="s">
+      <c r="C23" s="177" t="s">
         <v>426</v>
       </c>
       <c r="D23" s="176"/>
@@ -7533,7 +7533,7 @@
       <c r="J23" s="134"/>
       <c r="K23" s="101"/>
       <c r="L23" s="134"/>
-      <c r="M23" s="180" t="s">
+      <c r="M23" s="181" t="s">
         <v>428</v>
       </c>
       <c r="N23" s="176"/>
@@ -7567,7 +7567,7 @@
       <c r="J24" s="134"/>
       <c r="K24" s="101"/>
       <c r="L24" s="134"/>
-      <c r="M24" s="180" t="s">
+      <c r="M24" s="181" t="s">
         <v>428</v>
       </c>
       <c r="N24" s="176"/>
@@ -7588,7 +7588,7 @@
       <c r="O25" s="99"/>
     </row>
     <row r="26" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="184" t="s">
+      <c r="A26" s="191" t="s">
         <v>448</v>
       </c>
       <c r="B26" s="176"/>
@@ -7618,7 +7618,7 @@
       <c r="B27" s="18" t="s">
         <v>233</v>
       </c>
-      <c r="C27" s="178" t="s">
+      <c r="C27" s="175" t="s">
         <v>378</v>
       </c>
       <c r="D27" s="176"/>
@@ -7646,7 +7646,7 @@
       <c r="B28" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="178" t="s">
+      <c r="C28" s="175" t="s">
         <v>449</v>
       </c>
       <c r="D28" s="176"/>
@@ -7674,7 +7674,7 @@
       <c r="B29" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="178" t="s">
+      <c r="C29" s="175" t="s">
         <v>449</v>
       </c>
       <c r="D29" s="176"/>
@@ -7702,7 +7702,7 @@
       <c r="B30" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="178" t="s">
+      <c r="C30" s="175" t="s">
         <v>385</v>
       </c>
       <c r="D30" s="176"/>
@@ -7729,7 +7729,7 @@
       <c r="O31" s="99"/>
     </row>
     <row r="32" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="191" t="s">
+      <c r="A32" s="180" t="s">
         <v>450</v>
       </c>
       <c r="B32" s="176"/>
@@ -7802,7 +7802,7 @@
       <c r="O34" s="99"/>
     </row>
     <row r="35" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="187" t="s">
+      <c r="A35" s="182" t="s">
         <v>456</v>
       </c>
       <c r="B35" s="176"/>
@@ -7826,7 +7826,7 @@
       <c r="T35" s="176"/>
     </row>
     <row r="36" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="189" t="s">
+      <c r="A36" s="178" t="s">
         <v>457</v>
       </c>
       <c r="B36" s="176"/>
@@ -7850,7 +7850,7 @@
       <c r="T36" s="176"/>
     </row>
     <row r="37" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="189" t="s">
+      <c r="A37" s="178" t="s">
         <v>458</v>
       </c>
       <c r="B37" s="176"/>
@@ -7874,7 +7874,7 @@
       <c r="T37" s="176"/>
     </row>
     <row r="38" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="189" t="s">
+      <c r="A38" s="178" t="s">
         <v>459</v>
       </c>
       <c r="B38" s="176"/>
@@ -7898,7 +7898,7 @@
       <c r="T38" s="176"/>
     </row>
     <row r="39" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="189" t="s">
+      <c r="A39" s="178" t="s">
         <v>460</v>
       </c>
       <c r="B39" s="176"/>
@@ -7928,20 +7928,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="C27:R27"/>
-    <mergeCell ref="C23:I23"/>
-    <mergeCell ref="A39:T39"/>
-    <mergeCell ref="O2:R2"/>
-    <mergeCell ref="A36:T36"/>
-    <mergeCell ref="A37:T37"/>
-    <mergeCell ref="A32:T32"/>
-    <mergeCell ref="L8:R8"/>
-    <mergeCell ref="A35:T35"/>
-    <mergeCell ref="A38:T38"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="M20:R20"/>
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C28:R28"/>
@@ -7958,6 +7944,20 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:T5"/>
     <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C27:R27"/>
+    <mergeCell ref="C23:I23"/>
+    <mergeCell ref="A39:T39"/>
+    <mergeCell ref="O2:R2"/>
+    <mergeCell ref="A36:T36"/>
+    <mergeCell ref="A37:T37"/>
+    <mergeCell ref="A32:T32"/>
+    <mergeCell ref="L8:R8"/>
+    <mergeCell ref="A35:T35"/>
+    <mergeCell ref="A38:T38"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="M20:R20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7976,7 +7976,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="222" t="s">
+      <c r="A1" s="218" t="s">
         <v>461</v>
       </c>
       <c r="B1" s="176"/>
@@ -8000,27 +8000,27 @@
       <c r="T1" s="176"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="182"/>
+      <c r="A2" s="189"/>
       <c r="B2" s="176"/>
-      <c r="C2" s="177" t="s">
+      <c r="C2" s="186" t="s">
         <v>405</v>
       </c>
       <c r="D2" s="176"/>
       <c r="E2" s="176"/>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="188" t="s">
         <v>406</v>
       </c>
       <c r="G2" s="176"/>
       <c r="H2" s="176"/>
       <c r="I2" s="176"/>
       <c r="J2" s="176"/>
-      <c r="K2" s="193" t="s">
+      <c r="K2" s="184" t="s">
         <v>407</v>
       </c>
       <c r="L2" s="176"/>
       <c r="M2" s="176"/>
       <c r="N2" s="176"/>
-      <c r="O2" s="190" t="s">
+      <c r="O2" s="179" t="s">
         <v>408</v>
       </c>
       <c r="P2" s="176"/>
@@ -8092,7 +8092,7 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="186" t="s">
+      <c r="A4" s="193" t="s">
         <v>425</v>
       </c>
       <c r="B4" s="176"/>
@@ -8140,7 +8140,7 @@
       <c r="T4" s="11"/>
     </row>
     <row r="5" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="219" t="s">
+      <c r="A5" s="221" t="s">
         <v>148</v>
       </c>
       <c r="B5" s="176"/>
@@ -8173,7 +8173,7 @@
       <c r="C6" s="129" t="s">
         <v>429</v>
       </c>
-      <c r="D6" s="220" t="s">
+      <c r="D6" s="222" t="s">
         <v>463</v>
       </c>
       <c r="E6" s="176"/>
@@ -8181,7 +8181,7 @@
       <c r="G6" s="139" t="s">
         <v>433</v>
       </c>
-      <c r="H6" s="188" t="s">
+      <c r="H6" s="177" t="s">
         <v>426</v>
       </c>
       <c r="I6" s="176"/>
@@ -8189,7 +8189,7 @@
       <c r="K6" s="101"/>
       <c r="L6" s="134"/>
       <c r="M6" s="134"/>
-      <c r="N6" s="221" t="s">
+      <c r="N6" s="223" t="s">
         <v>427</v>
       </c>
       <c r="O6" s="176"/>
@@ -8219,7 +8219,7 @@
       <c r="G7" s="128"/>
       <c r="H7" s="128"/>
       <c r="I7" s="128"/>
-      <c r="J7" s="183" t="s">
+      <c r="J7" s="190" t="s">
         <v>181</v>
       </c>
       <c r="K7" s="176"/>
@@ -8384,7 +8384,7 @@
       <c r="L12" s="134"/>
       <c r="M12" s="134"/>
       <c r="N12" s="134"/>
-      <c r="O12" s="223" t="s">
+      <c r="O12" s="219" t="s">
         <v>426</v>
       </c>
       <c r="P12" s="176"/>
@@ -8583,7 +8583,7 @@
       <c r="O19" s="99"/>
     </row>
     <row r="20" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="184" t="s">
+      <c r="A20" s="191" t="s">
         <v>448</v>
       </c>
       <c r="B20" s="176"/>
@@ -8613,7 +8613,7 @@
       <c r="B21" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="C21" s="178" t="s">
+      <c r="C21" s="175" t="s">
         <v>467</v>
       </c>
       <c r="D21" s="176"/>
@@ -8641,7 +8641,7 @@
       <c r="B22" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="C22" s="178" t="s">
+      <c r="C22" s="175" t="s">
         <v>395</v>
       </c>
       <c r="D22" s="176"/>
@@ -8669,7 +8669,7 @@
       <c r="B23" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="C23" s="178" t="s">
+      <c r="C23" s="175" t="s">
         <v>395</v>
       </c>
       <c r="D23" s="176"/>
@@ -8697,7 +8697,7 @@
       <c r="B24" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="C24" s="178" t="s">
+      <c r="C24" s="175" t="s">
         <v>468</v>
       </c>
       <c r="D24" s="176"/>
@@ -8724,7 +8724,7 @@
       <c r="O25" s="99"/>
     </row>
     <row r="26" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="191" t="s">
+      <c r="A26" s="180" t="s">
         <v>450</v>
       </c>
       <c r="B26" s="176"/>
@@ -8797,7 +8797,7 @@
       <c r="O28" s="99"/>
     </row>
     <row r="29" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="219" t="s">
+      <c r="A29" s="221" t="s">
         <v>456</v>
       </c>
       <c r="B29" s="176"/>
@@ -8821,7 +8821,7 @@
       <c r="T29" s="176"/>
     </row>
     <row r="30" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="218" t="s">
+      <c r="A30" s="220" t="s">
         <v>469</v>
       </c>
       <c r="B30" s="176"/>
@@ -8845,7 +8845,7 @@
       <c r="T30" s="176"/>
     </row>
     <row r="31" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="218" t="s">
+      <c r="A31" s="220" t="s">
         <v>470</v>
       </c>
       <c r="B31" s="176"/>
@@ -8869,7 +8869,7 @@
       <c r="T31" s="176"/>
     </row>
     <row r="32" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="218" t="s">
+      <c r="A32" s="220" t="s">
         <v>471</v>
       </c>
       <c r="B32" s="176"/>
@@ -8893,7 +8893,7 @@
       <c r="T32" s="176"/>
     </row>
     <row r="33" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="218" t="s">
+      <c r="A33" s="220" t="s">
         <v>472</v>
       </c>
       <c r="B33" s="176"/>
@@ -8923,17 +8923,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="C24:R24"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="O12:R12"/>
-    <mergeCell ref="C23:R23"/>
-    <mergeCell ref="O2:R2"/>
     <mergeCell ref="A33:T33"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:T5"/>
@@ -8947,6 +8936,17 @@
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
     <mergeCell ref="A26:T26"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="C24:R24"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="O12:R12"/>
+    <mergeCell ref="C23:R23"/>
+    <mergeCell ref="O2:R2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8965,7 +8965,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="233" t="s">
+      <c r="A1" s="225" t="s">
         <v>473</v>
       </c>
       <c r="B1" s="176"/>
@@ -8989,27 +8989,27 @@
       <c r="T1" s="176"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="182"/>
+      <c r="A2" s="189"/>
       <c r="B2" s="176"/>
-      <c r="C2" s="177" t="s">
+      <c r="C2" s="186" t="s">
         <v>405</v>
       </c>
       <c r="D2" s="176"/>
       <c r="E2" s="176"/>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="188" t="s">
         <v>406</v>
       </c>
       <c r="G2" s="176"/>
       <c r="H2" s="176"/>
       <c r="I2" s="176"/>
       <c r="J2" s="176"/>
-      <c r="K2" s="193" t="s">
+      <c r="K2" s="184" t="s">
         <v>407</v>
       </c>
       <c r="L2" s="176"/>
       <c r="M2" s="176"/>
       <c r="N2" s="176"/>
-      <c r="O2" s="190" t="s">
+      <c r="O2" s="179" t="s">
         <v>408</v>
       </c>
       <c r="P2" s="176"/>
@@ -9081,7 +9081,7 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="186" t="s">
+      <c r="A4" s="193" t="s">
         <v>425</v>
       </c>
       <c r="B4" s="176"/>
@@ -9129,7 +9129,7 @@
       <c r="T4" s="11"/>
     </row>
     <row r="5" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="234" t="s">
+      <c r="A5" s="226" t="s">
         <v>148</v>
       </c>
       <c r="B5" s="176"/>
@@ -9159,7 +9159,7 @@
       <c r="B6" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="C6" s="185" t="s">
+      <c r="C6" s="192" t="s">
         <v>174</v>
       </c>
       <c r="D6" s="176"/>
@@ -9168,7 +9168,7 @@
       <c r="G6" s="139" t="s">
         <v>433</v>
       </c>
-      <c r="H6" s="185" t="s">
+      <c r="H6" s="192" t="s">
         <v>174</v>
       </c>
       <c r="I6" s="176"/>
@@ -9254,13 +9254,13 @@
       <c r="I8" s="137" t="s">
         <v>436</v>
       </c>
-      <c r="J8" s="225" t="s">
+      <c r="J8" s="227" t="s">
         <v>433</v>
       </c>
       <c r="K8" s="176"/>
       <c r="L8" s="134"/>
       <c r="M8" s="134"/>
-      <c r="N8" s="221" t="s">
+      <c r="N8" s="223" t="s">
         <v>427</v>
       </c>
       <c r="O8" s="176"/>
@@ -9287,14 +9287,14 @@
       <c r="D9" s="129" t="s">
         <v>429</v>
       </c>
-      <c r="E9" s="188" t="s">
+      <c r="E9" s="177" t="s">
         <v>426</v>
       </c>
       <c r="F9" s="176"/>
       <c r="G9" s="176"/>
       <c r="H9" s="176"/>
       <c r="I9" s="176"/>
-      <c r="J9" s="225" t="s">
+      <c r="J9" s="227" t="s">
         <v>433</v>
       </c>
       <c r="K9" s="176"/>
@@ -9325,7 +9325,7 @@
       <c r="D10" s="134"/>
       <c r="E10" s="134"/>
       <c r="F10" s="101"/>
-      <c r="G10" s="183" t="s">
+      <c r="G10" s="190" t="s">
         <v>181</v>
       </c>
       <c r="H10" s="176"/>
@@ -9354,7 +9354,7 @@
         <v>33</v>
       </c>
       <c r="C11" s="134"/>
-      <c r="D11" s="188" t="s">
+      <c r="D11" s="177" t="s">
         <v>426</v>
       </c>
       <c r="E11" s="176"/>
@@ -9388,7 +9388,7 @@
       <c r="C12" s="135" t="s">
         <v>428</v>
       </c>
-      <c r="D12" s="185" t="s">
+      <c r="D12" s="192" t="s">
         <v>174</v>
       </c>
       <c r="E12" s="176"/>
@@ -9451,7 +9451,7 @@
       <c r="B14" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="C14" s="183" t="s">
+      <c r="C14" s="190" t="s">
         <v>181</v>
       </c>
       <c r="D14" s="176"/>
@@ -9486,7 +9486,7 @@
       <c r="C15" s="129" t="s">
         <v>429</v>
       </c>
-      <c r="D15" s="180" t="s">
+      <c r="D15" s="181" t="s">
         <v>428</v>
       </c>
       <c r="E15" s="176"/>
@@ -9498,7 +9498,7 @@
       <c r="K15" s="101"/>
       <c r="L15" s="134"/>
       <c r="M15" s="134"/>
-      <c r="N15" s="180" t="s">
+      <c r="N15" s="181" t="s">
         <v>428</v>
       </c>
       <c r="O15" s="176"/>
@@ -9556,13 +9556,13 @@
       <c r="G17" s="134"/>
       <c r="H17" s="134"/>
       <c r="I17" s="134"/>
-      <c r="J17" s="225" t="s">
+      <c r="J17" s="227" t="s">
         <v>433</v>
       </c>
       <c r="K17" s="176"/>
       <c r="L17" s="134"/>
       <c r="M17" s="134"/>
-      <c r="N17" s="180" t="s">
+      <c r="N17" s="181" t="s">
         <v>428</v>
       </c>
       <c r="O17" s="176"/>
@@ -9582,34 +9582,34 @@
       <c r="O18" s="99"/>
     </row>
     <row r="19" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="226" t="s">
+      <c r="A19" s="229" t="s">
         <v>368</v>
       </c>
-      <c r="B19" s="227" t="s">
+      <c r="B19" s="230" t="s">
         <v>294</v>
       </c>
-      <c r="C19" s="228" t="s">
+      <c r="C19" s="231" t="s">
         <v>426</v>
       </c>
-      <c r="D19" s="229"/>
-      <c r="E19" s="229"/>
-      <c r="F19" s="229"/>
-      <c r="G19" s="229"/>
-      <c r="H19" s="229"/>
-      <c r="I19" s="229"/>
-      <c r="J19" s="229"/>
-      <c r="K19" s="230"/>
-      <c r="L19" s="230"/>
-      <c r="M19" s="230"/>
-      <c r="N19" s="230"/>
-      <c r="O19" s="230"/>
-      <c r="P19" s="230"/>
-      <c r="Q19" s="230"/>
-      <c r="R19" s="230"/>
-      <c r="S19" s="231" t="s">
+      <c r="D19" s="232"/>
+      <c r="E19" s="232"/>
+      <c r="F19" s="232"/>
+      <c r="G19" s="232"/>
+      <c r="H19" s="232"/>
+      <c r="I19" s="232"/>
+      <c r="J19" s="232"/>
+      <c r="K19" s="233"/>
+      <c r="L19" s="233"/>
+      <c r="M19" s="233"/>
+      <c r="N19" s="233"/>
+      <c r="O19" s="233"/>
+      <c r="P19" s="233"/>
+      <c r="Q19" s="233"/>
+      <c r="R19" s="233"/>
+      <c r="S19" s="234" t="s">
         <v>371</v>
       </c>
-      <c r="T19" s="232" t="s">
+      <c r="T19" s="235" t="s">
         <v>20</v>
       </c>
     </row>
@@ -9641,7 +9641,7 @@
       <c r="B21" s="18" t="s">
         <v>481</v>
       </c>
-      <c r="C21" s="178" t="s">
+      <c r="C21" s="175" t="s">
         <v>482</v>
       </c>
       <c r="D21" s="176"/>
@@ -9681,16 +9681,16 @@
       <c r="C23" s="176"/>
       <c r="D23" s="176"/>
       <c r="E23" s="176"/>
-      <c r="F23" s="235"/>
+      <c r="F23" s="224"/>
       <c r="G23" s="176"/>
       <c r="H23" s="176"/>
       <c r="I23" s="176"/>
       <c r="J23" s="176"/>
-      <c r="K23" s="235"/>
+      <c r="K23" s="224"/>
       <c r="L23" s="176"/>
       <c r="M23" s="176"/>
       <c r="N23" s="176"/>
-      <c r="O23" s="235"/>
+      <c r="O23" s="224"/>
       <c r="P23" s="176"/>
       <c r="Q23" s="176"/>
       <c r="R23" s="176"/>
@@ -9752,16 +9752,16 @@
       <c r="C26" s="176"/>
       <c r="D26" s="176"/>
       <c r="E26" s="176"/>
-      <c r="F26" s="235"/>
+      <c r="F26" s="224"/>
       <c r="G26" s="176"/>
       <c r="H26" s="176"/>
       <c r="I26" s="176"/>
       <c r="J26" s="176"/>
-      <c r="K26" s="235"/>
+      <c r="K26" s="224"/>
       <c r="L26" s="176"/>
       <c r="M26" s="176"/>
       <c r="N26" s="176"/>
-      <c r="O26" s="235"/>
+      <c r="O26" s="224"/>
       <c r="P26" s="176"/>
       <c r="Q26" s="176"/>
       <c r="R26" s="176"/>
@@ -9769,7 +9769,7 @@
       <c r="T26" s="176"/>
     </row>
     <row r="27" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="234" t="s">
+      <c r="A27" s="226" t="s">
         <v>456</v>
       </c>
       <c r="B27" s="176"/>
@@ -9793,7 +9793,7 @@
       <c r="T27" s="176"/>
     </row>
     <row r="28" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="224" t="s">
+      <c r="A28" s="228" t="s">
         <v>484</v>
       </c>
       <c r="B28" s="176"/>
@@ -9817,7 +9817,7 @@
       <c r="T28" s="176"/>
     </row>
     <row r="29" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="224" t="s">
+      <c r="A29" s="228" t="s">
         <v>485</v>
       </c>
       <c r="B29" s="176"/>
@@ -9841,7 +9841,7 @@
       <c r="T29" s="176"/>
     </row>
     <row r="30" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="224" t="s">
+      <c r="A30" s="228" t="s">
         <v>486</v>
       </c>
       <c r="B30" s="176"/>
@@ -9865,7 +9865,7 @@
       <c r="T30" s="176"/>
     </row>
     <row r="31" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="224" t="s">
+      <c r="A31" s="228" t="s">
         <v>487</v>
       </c>
       <c r="B31" s="176"/>
@@ -9889,7 +9889,7 @@
       <c r="T31" s="176"/>
     </row>
     <row r="32" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="224" t="s">
+      <c r="A32" s="228" t="s">
         <v>488</v>
       </c>
       <c r="B32" s="176"/>
@@ -9924,6 +9924,23 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="A28:T28"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="A19:T19"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D12:R12"/>
+    <mergeCell ref="C21:R21"/>
+    <mergeCell ref="D15:I15"/>
+    <mergeCell ref="A27:T27"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="A32:T32"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="N15:R15"/>
+    <mergeCell ref="A29:T29"/>
+    <mergeCell ref="A31:T31"/>
+    <mergeCell ref="A30:T30"/>
     <mergeCell ref="N17:R17"/>
     <mergeCell ref="A26:T26"/>
     <mergeCell ref="C20:R20"/>
@@ -9940,23 +9957,6 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:T5"/>
     <mergeCell ref="O2:R2"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="A32:T32"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="N15:R15"/>
-    <mergeCell ref="A29:T29"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="A28:T28"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="A19:T19"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="A31:T31"/>
-    <mergeCell ref="A30:T30"/>
-    <mergeCell ref="D12:R12"/>
-    <mergeCell ref="C21:R21"/>
-    <mergeCell ref="D15:I15"/>
-    <mergeCell ref="A27:T27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10713,10 +10713,10 @@
         <v>159</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>587</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>588</v>
       </c>
       <c r="E13" s="67" t="s">
         <v>323</v>
@@ -10730,10 +10730,10 @@
         <v>223</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>589</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>590</v>
       </c>
       <c r="E14" s="65" t="s">
         <v>20</v>
@@ -10741,16 +10741,16 @@
     </row>
     <row r="15" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B15" s="114" t="s">
         <v>563</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>592</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>593</v>
       </c>
       <c r="E15" s="64" t="s">
         <v>7</v>
@@ -10775,7 +10775,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="250" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B1" s="176"/>
       <c r="C1" s="176"/>
@@ -10811,7 +10811,7 @@
     </row>
     <row r="3" spans="1:32" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="249" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B3" s="176"/>
       <c r="C3" s="176"/>
@@ -10849,94 +10849,94 @@
         <v>560</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="F4" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="G4" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="G4" s="62" t="s">
+      <c r="H4" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="H4" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="I4" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="K4" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="L4" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="L4" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="M4" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="N4" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="N4" s="62" t="s">
+      <c r="O4" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="O4" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="P4" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="Q4" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="Q4" s="10" t="s">
+      <c r="R4" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="R4" s="10" t="s">
+      <c r="S4" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="S4" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="T4" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="U4" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="U4" s="62" t="s">
+      <c r="V4" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="V4" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="W4" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="X4" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="X4" s="10" t="s">
+      <c r="Y4" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="Y4" s="10" t="s">
+      <c r="Z4" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="Z4" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="AA4" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="AB4" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="AB4" s="62" t="s">
+      <c r="AC4" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="AC4" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="AD4" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="AE4" s="10" t="s">
         <v>596</v>
-      </c>
-      <c r="AE4" s="10" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="5" spans="1:32" ht="11" customHeight="1" x14ac:dyDescent="0.35">
@@ -11034,7 +11034,7 @@
     </row>
     <row r="6" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B6" s="26"/>
       <c r="C6" s="26"/>
@@ -11051,19 +11051,19 @@
       <c r="N6" s="27"/>
       <c r="O6" s="27"/>
       <c r="P6" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q6" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R6" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S6" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T6" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U6" s="27"/>
       <c r="V6" s="27"/>
@@ -11079,7 +11079,7 @@
     </row>
     <row r="7" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="25" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
@@ -11131,19 +11131,19 @@
       <c r="N8" s="27"/>
       <c r="O8" s="27"/>
       <c r="P8" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q8" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R8" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S8" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T8" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U8" s="27"/>
       <c r="V8" s="27"/>
@@ -11229,7 +11229,7 @@
     </row>
     <row r="11" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="25" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
@@ -11474,7 +11474,7 @@
     </row>
     <row r="18" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="25" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -11509,7 +11509,7 @@
     </row>
     <row r="19" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="25" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -11544,7 +11544,7 @@
     </row>
     <row r="21" spans="1:32" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="249" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B21" s="176"/>
       <c r="C21" s="176"/>
@@ -11583,97 +11583,97 @@
         <v>560</v>
       </c>
       <c r="B22" s="10" t="s">
+        <v>597</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="D22" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="E22" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="E22" s="62" t="s">
+      <c r="F22" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="F22" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="G22" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="H22" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="I22" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="J22" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="J22" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="K22" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="L22" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="L22" s="62" t="s">
+      <c r="M22" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="M22" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="N22" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="O22" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="O22" s="10" t="s">
+      <c r="P22" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="P22" s="10" t="s">
+      <c r="Q22" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="Q22" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="R22" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="S22" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="S22" s="62" t="s">
+      <c r="T22" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="T22" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="U22" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="V22" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="V22" s="10" t="s">
+      <c r="W22" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="W22" s="10" t="s">
+      <c r="X22" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="X22" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="Y22" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="Z22" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="Z22" s="62" t="s">
+      <c r="AA22" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="AA22" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="AB22" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="AC22" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="AC22" s="10" t="s">
+      <c r="AD22" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="AD22" s="10" t="s">
+      <c r="AE22" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="AE22" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="AF22" s="10" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="23" spans="1:32" ht="11" customHeight="1" x14ac:dyDescent="0.35">
@@ -11774,7 +11774,7 @@
     </row>
     <row r="24" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="25" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -11810,7 +11810,7 @@
     </row>
     <row r="25" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="25" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -11954,7 +11954,7 @@
     </row>
     <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="25" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B29" s="26"/>
       <c r="C29" s="26"/>
@@ -11976,40 +11976,40 @@
       <c r="S29" s="27"/>
       <c r="T29" s="27"/>
       <c r="U29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="X29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Y29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AA29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AB29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AC29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AD29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AE29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AF29" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="30" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -12130,19 +12130,19 @@
       <c r="E33" s="27"/>
       <c r="F33" s="27"/>
       <c r="G33" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H33" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I33" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J33" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K33" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L33" s="27"/>
       <c r="M33" s="27"/>
@@ -12219,66 +12219,66 @@
       <c r="L35" s="27"/>
       <c r="M35" s="27"/>
       <c r="N35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="X35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Y35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Z35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AA35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AB35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AC35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AD35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AE35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AF35" s="32" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="36" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="25" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B36" s="26"/>
       <c r="C36" s="26"/>
@@ -12294,63 +12294,63 @@
       <c r="M36" s="27"/>
       <c r="N36" s="26"/>
       <c r="O36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="X36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Y36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Z36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AA36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AB36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AC36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AD36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AE36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AF36" s="33" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="37" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="25" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B37" s="26"/>
       <c r="C37" s="26"/>
@@ -12386,7 +12386,7 @@
     </row>
     <row r="39" spans="1:32" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="249" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B39" s="176"/>
       <c r="C39" s="176"/>
@@ -12425,97 +12425,97 @@
         <v>560</v>
       </c>
       <c r="B40" s="62" t="s">
+        <v>600</v>
+      </c>
+      <c r="C40" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="C40" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="D40" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="E40" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="F40" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="F40" s="10" t="s">
+      <c r="G40" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="G40" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="H40" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="I40" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="I40" s="62" t="s">
+      <c r="J40" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="J40" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="K40" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="L40" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="L40" s="10" t="s">
+      <c r="M40" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="M40" s="10" t="s">
+      <c r="N40" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="N40" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="O40" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="P40" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="P40" s="62" t="s">
+      <c r="Q40" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="Q40" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="R40" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="S40" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="S40" s="10" t="s">
+      <c r="T40" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="T40" s="10" t="s">
+      <c r="U40" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="U40" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="V40" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="W40" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="W40" s="62" t="s">
+      <c r="X40" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="X40" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="Y40" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="Z40" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="Z40" s="10" t="s">
+      <c r="AA40" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="AA40" s="10" t="s">
+      <c r="AB40" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="AB40" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="AC40" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="AD40" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="AD40" s="62" t="s">
+      <c r="AE40" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="AE40" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="AF40" s="10" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="41" spans="1:32" ht="11" customHeight="1" x14ac:dyDescent="0.35">
@@ -12616,66 +12616,66 @@
     </row>
     <row r="42" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="25" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B42" s="27"/>
       <c r="C42" s="27"/>
       <c r="D42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V42" s="28" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W42" s="27"/>
       <c r="X42" s="27"/>
@@ -12690,66 +12690,66 @@
     </row>
     <row r="43" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="25" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B43" s="27"/>
       <c r="C43" s="27"/>
       <c r="D43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V43" s="34" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W43" s="27"/>
       <c r="X43" s="27"/>
@@ -12769,61 +12769,61 @@
       <c r="B44" s="27"/>
       <c r="C44" s="27"/>
       <c r="D44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V44" s="29" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W44" s="27"/>
       <c r="X44" s="27"/>
@@ -12843,61 +12843,61 @@
       <c r="B45" s="27"/>
       <c r="C45" s="27"/>
       <c r="D45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V45" s="35" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W45" s="27"/>
       <c r="X45" s="27"/>
@@ -12924,40 +12924,40 @@
       <c r="I46" s="27"/>
       <c r="J46" s="27"/>
       <c r="K46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V46" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W46" s="27"/>
       <c r="X46" s="27"/>
@@ -12972,37 +12972,37 @@
     </row>
     <row r="47" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="C47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K47" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L47" s="26"/>
       <c r="M47" s="26"/>
@@ -13047,40 +13047,40 @@
       <c r="P48" s="27"/>
       <c r="Q48" s="27"/>
       <c r="R48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="X48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Y48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Z48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AA48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AB48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AC48" s="37" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AD48" s="27"/>
       <c r="AE48" s="27"/>
@@ -13100,49 +13100,49 @@
       <c r="I49" s="27"/>
       <c r="J49" s="27"/>
       <c r="K49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Q49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="X49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Y49" s="38" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Z49" s="26"/>
       <c r="AA49" s="26"/>
@@ -13159,40 +13159,40 @@
       <c r="B50" s="27"/>
       <c r="C50" s="27"/>
       <c r="D50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="O50" s="39" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="P50" s="27"/>
       <c r="Q50" s="27"/>
@@ -13233,19 +13233,19 @@
       <c r="P51" s="27"/>
       <c r="Q51" s="27"/>
       <c r="R51" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="S51" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="T51" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="U51" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="V51" s="31" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="W51" s="27"/>
       <c r="X51" s="27"/>
@@ -13265,19 +13265,19 @@
       <c r="B52" s="27"/>
       <c r="C52" s="27"/>
       <c r="D52" s="40" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E52" s="40" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F52" s="40" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G52" s="40" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H52" s="40" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I52" s="27"/>
       <c r="J52" s="27"/>
@@ -13342,7 +13342,7 @@
     </row>
     <row r="54" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="25" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B54" s="27"/>
       <c r="C54" s="27"/>
@@ -13378,7 +13378,7 @@
     </row>
     <row r="55" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="25" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B55" s="27"/>
       <c r="C55" s="27"/>
@@ -13414,7 +13414,7 @@
     </row>
     <row r="57" spans="1:32" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="249" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B57" s="176"/>
       <c r="C57" s="176"/>
@@ -13452,94 +13452,94 @@
         <v>560</v>
       </c>
       <c r="B58" s="10" t="s">
+        <v>596</v>
+      </c>
+      <c r="C58" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="D58" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="D58" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="E58" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="F58" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="F58" s="62" t="s">
+      <c r="G58" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="G58" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="H58" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="I58" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="I58" s="10" t="s">
+      <c r="J58" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="J58" s="10" t="s">
+      <c r="K58" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="K58" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="L58" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="M58" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="M58" s="62" t="s">
+      <c r="N58" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="N58" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="O58" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="P58" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="P58" s="10" t="s">
+      <c r="Q58" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="Q58" s="10" t="s">
+      <c r="R58" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="R58" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="S58" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="T58" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="T58" s="62" t="s">
+      <c r="U58" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="U58" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="V58" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="W58" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="W58" s="10" t="s">
+      <c r="X58" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="X58" s="10" t="s">
+      <c r="Y58" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="Y58" s="10" t="s">
-        <v>599</v>
-      </c>
       <c r="Z58" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="AA58" s="62" t="s">
         <v>600</v>
       </c>
-      <c r="AA58" s="62" t="s">
+      <c r="AB58" s="62" t="s">
         <v>601</v>
       </c>
-      <c r="AB58" s="62" t="s">
-        <v>602</v>
-      </c>
       <c r="AC58" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="AD58" s="10" t="s">
         <v>596</v>
       </c>
-      <c r="AD58" s="10" t="s">
+      <c r="AE58" s="10" t="s">
         <v>597</v>
-      </c>
-      <c r="AE58" s="10" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="59" spans="1:32" ht="11" customHeight="1" x14ac:dyDescent="0.35">
@@ -13637,7 +13637,7 @@
     </row>
     <row r="60" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="25" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B60" s="26"/>
       <c r="C60" s="26"/>
@@ -13672,7 +13672,7 @@
     </row>
     <row r="61" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="25" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B61" s="26"/>
       <c r="C61" s="26"/>
@@ -13783,28 +13783,28 @@
       <c r="C64" s="26"/>
       <c r="D64" s="26"/>
       <c r="E64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="J64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L64" s="36" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M64" s="27"/>
       <c r="N64" s="27"/>
@@ -13828,7 +13828,7 @@
     </row>
     <row r="65" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="25" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B65" s="26"/>
       <c r="C65" s="26"/>
@@ -14073,7 +14073,7 @@
     </row>
     <row r="72" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="25" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B72" s="26"/>
       <c r="C72" s="26"/>
@@ -14108,7 +14108,7 @@
     </row>
     <row r="73" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="25" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B73" s="26"/>
       <c r="C73" s="26"/>
@@ -14143,7 +14143,7 @@
     </row>
     <row r="75" spans="1:31" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="248" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B75" s="176"/>
       <c r="C75" s="176"/>
@@ -14199,8 +14199,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="256" t="s">
-        <v>612</v>
+      <c r="A1" s="251" t="s">
+        <v>611</v>
       </c>
       <c r="B1" s="176"/>
       <c r="C1" s="176"/>
@@ -14217,8 +14217,8 @@
       <c r="N1" s="176"/>
     </row>
     <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="257" t="s">
-        <v>613</v>
+      <c r="A2" s="252" t="s">
+        <v>612</v>
       </c>
       <c r="B2" s="176"/>
       <c r="C2" s="176"/>
@@ -14235,8 +14235,8 @@
       <c r="N2" s="176"/>
     </row>
     <row r="4" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="254" t="s">
-        <v>614</v>
+      <c r="A4" s="253" t="s">
+        <v>613</v>
       </c>
       <c r="B4" s="176"/>
       <c r="C4" s="176"/>
@@ -14254,55 +14254,55 @@
     </row>
     <row r="5" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>615</v>
-      </c>
-      <c r="B5" s="199"/>
+        <v>614</v>
+      </c>
+      <c r="B5" s="198"/>
       <c r="C5" s="195"/>
       <c r="D5" s="196"/>
     </row>
     <row r="6" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="B6" s="199"/>
+        <v>615</v>
+      </c>
+      <c r="B6" s="198"/>
       <c r="C6" s="195"/>
       <c r="D6" s="196"/>
     </row>
     <row r="7" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="B7" s="199"/>
+        <v>616</v>
+      </c>
+      <c r="B7" s="198"/>
       <c r="C7" s="195"/>
       <c r="D7" s="196"/>
     </row>
     <row r="8" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="B8" s="199"/>
+        <v>617</v>
+      </c>
+      <c r="B8" s="198"/>
       <c r="C8" s="195"/>
       <c r="D8" s="196"/>
     </row>
     <row r="9" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>619</v>
-      </c>
-      <c r="B9" s="199"/>
+        <v>618</v>
+      </c>
+      <c r="B9" s="198"/>
       <c r="C9" s="195"/>
       <c r="D9" s="196"/>
     </row>
     <row r="10" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="B10" s="199"/>
+        <v>619</v>
+      </c>
+      <c r="B10" s="198"/>
       <c r="C10" s="195"/>
       <c r="D10" s="196"/>
     </row>
     <row r="12" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="254" t="s">
-        <v>621</v>
+      <c r="A12" s="253" t="s">
+        <v>620</v>
       </c>
       <c r="B12" s="176"/>
       <c r="C12" s="176"/>
@@ -14320,47 +14320,47 @@
     </row>
     <row r="13" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="124" t="s">
-        <v>622</v>
-      </c>
-      <c r="B13" s="199"/>
+        <v>621</v>
+      </c>
+      <c r="B13" s="198"/>
       <c r="C13" s="195"/>
       <c r="D13" s="196"/>
     </row>
     <row r="14" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="124" t="s">
-        <v>623</v>
-      </c>
-      <c r="B14" s="199"/>
+        <v>622</v>
+      </c>
+      <c r="B14" s="198"/>
       <c r="C14" s="195"/>
       <c r="D14" s="196"/>
     </row>
     <row r="15" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="124" t="s">
-        <v>624</v>
-      </c>
-      <c r="B15" s="199"/>
+        <v>623</v>
+      </c>
+      <c r="B15" s="198"/>
       <c r="C15" s="195"/>
       <c r="D15" s="196"/>
     </row>
     <row r="16" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="124" t="s">
-        <v>625</v>
-      </c>
-      <c r="B16" s="199"/>
+        <v>624</v>
+      </c>
+      <c r="B16" s="198"/>
       <c r="C16" s="195"/>
       <c r="D16" s="196"/>
     </row>
     <row r="17" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="124" t="s">
-        <v>626</v>
-      </c>
-      <c r="B17" s="199"/>
+        <v>625</v>
+      </c>
+      <c r="B17" s="198"/>
       <c r="C17" s="195"/>
       <c r="D17" s="196"/>
     </row>
     <row r="19" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="254" t="s">
-        <v>627</v>
+      <c r="A19" s="253" t="s">
+        <v>626</v>
       </c>
       <c r="B19" s="176"/>
       <c r="C19" s="176"/>
@@ -14378,55 +14378,55 @@
     </row>
     <row r="20" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="113" t="s">
-        <v>628</v>
-      </c>
-      <c r="B20" s="199"/>
+        <v>627</v>
+      </c>
+      <c r="B20" s="198"/>
       <c r="C20" s="195"/>
       <c r="D20" s="196"/>
     </row>
     <row r="21" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="113" t="s">
-        <v>629</v>
-      </c>
-      <c r="B21" s="199"/>
+        <v>628</v>
+      </c>
+      <c r="B21" s="198"/>
       <c r="C21" s="195"/>
       <c r="D21" s="196"/>
     </row>
     <row r="22" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="113" t="s">
-        <v>630</v>
-      </c>
-      <c r="B22" s="199"/>
+        <v>629</v>
+      </c>
+      <c r="B22" s="198"/>
       <c r="C22" s="195"/>
       <c r="D22" s="196"/>
     </row>
     <row r="23" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="113" t="s">
-        <v>631</v>
-      </c>
-      <c r="B23" s="199"/>
+        <v>630</v>
+      </c>
+      <c r="B23" s="198"/>
       <c r="C23" s="195"/>
       <c r="D23" s="196"/>
     </row>
     <row r="24" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="113" t="s">
-        <v>632</v>
-      </c>
-      <c r="B24" s="199"/>
+        <v>631</v>
+      </c>
+      <c r="B24" s="198"/>
       <c r="C24" s="195"/>
       <c r="D24" s="196"/>
     </row>
     <row r="25" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="113" t="s">
-        <v>633</v>
-      </c>
-      <c r="B25" s="199"/>
+        <v>632</v>
+      </c>
+      <c r="B25" s="198"/>
       <c r="C25" s="195"/>
       <c r="D25" s="196"/>
     </row>
     <row r="27" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="254" t="s">
-        <v>634</v>
+      <c r="A27" s="253" t="s">
+        <v>633</v>
       </c>
       <c r="B27" s="176"/>
       <c r="C27" s="176"/>
@@ -14444,47 +14444,47 @@
     </row>
     <row r="28" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="125" t="s">
-        <v>635</v>
-      </c>
-      <c r="B28" s="199"/>
+        <v>634</v>
+      </c>
+      <c r="B28" s="198"/>
       <c r="C28" s="195"/>
       <c r="D28" s="196"/>
     </row>
     <row r="29" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="125" t="s">
-        <v>636</v>
-      </c>
-      <c r="B29" s="199"/>
+        <v>635</v>
+      </c>
+      <c r="B29" s="198"/>
       <c r="C29" s="195"/>
       <c r="D29" s="196"/>
     </row>
     <row r="30" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="125" t="s">
-        <v>637</v>
-      </c>
-      <c r="B30" s="199"/>
+        <v>636</v>
+      </c>
+      <c r="B30" s="198"/>
       <c r="C30" s="195"/>
       <c r="D30" s="196"/>
     </row>
     <row r="31" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="125" t="s">
-        <v>638</v>
-      </c>
-      <c r="B31" s="199"/>
+        <v>637</v>
+      </c>
+      <c r="B31" s="198"/>
       <c r="C31" s="195"/>
       <c r="D31" s="196"/>
     </row>
     <row r="32" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="125" t="s">
-        <v>639</v>
-      </c>
-      <c r="B32" s="199"/>
+        <v>638</v>
+      </c>
+      <c r="B32" s="198"/>
       <c r="C32" s="195"/>
       <c r="D32" s="196"/>
     </row>
     <row r="34" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="255" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B34" s="176"/>
       <c r="C34" s="176"/>
@@ -14501,8 +14501,8 @@
       <c r="N34" s="176"/>
     </row>
     <row r="35" spans="1:14" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="252" t="s">
-        <v>641</v>
+      <c r="A35" s="257" t="s">
+        <v>640</v>
       </c>
       <c r="B35" s="176"/>
       <c r="C35" s="176"/>
@@ -14523,19 +14523,19 @@
         <v>146</v>
       </c>
       <c r="B36" s="70" t="s">
+        <v>641</v>
+      </c>
+      <c r="C36" s="70" t="s">
         <v>642</v>
       </c>
-      <c r="C36" s="70" t="s">
+      <c r="D36" s="70" t="s">
         <v>643</v>
-      </c>
-      <c r="D36" s="70" t="s">
-        <v>644</v>
       </c>
       <c r="E36" s="70" t="s">
         <v>5</v>
       </c>
       <c r="F36" s="70" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -14543,10 +14543,10 @@
         <v>426</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>646</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>647</v>
       </c>
       <c r="D37" s="126">
         <f>C37-B37+1</f>
@@ -14560,10 +14560,10 @@
         <v>427</v>
       </c>
       <c r="B38" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>648</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>649</v>
       </c>
       <c r="D38" s="127">
         <f>C38-B38+1</f>
@@ -14574,13 +14574,13 @@
     </row>
     <row r="39" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>650</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="C39" s="3" t="s">
         <v>651</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>652</v>
       </c>
       <c r="D39" s="126">
         <f>C39-B39+1</f>
@@ -14594,10 +14594,10 @@
         <v>164</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>653</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>654</v>
       </c>
       <c r="D40" s="127">
         <f>C40-B40+1</f>
@@ -14611,10 +14611,10 @@
         <v>428</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>655</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>656</v>
       </c>
       <c r="D41" s="126">
         <f>C41-B41+1</f>
@@ -14625,38 +14625,38 @@
     </row>
     <row r="42" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
       <c r="E42" s="7"/>
       <c r="F42" s="7" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -14664,10 +14664,10 @@
         <v>174</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D45" s="126">
         <f>C45-B45+1</f>
@@ -14681,10 +14681,10 @@
         <v>181</v>
       </c>
       <c r="B46" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>663</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>664</v>
       </c>
       <c r="D46" s="127">
         <f>C46-B46+1</f>
@@ -14698,10 +14698,10 @@
         <v>248</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D47" s="126">
         <f>C47-B47+1</f>
@@ -14712,7 +14712,7 @@
     </row>
     <row r="50" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="255" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B50" s="176"/>
       <c r="C50" s="176"/>
@@ -14729,8 +14729,8 @@
       <c r="N50" s="176"/>
     </row>
     <row r="51" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="251" t="s">
-        <v>666</v>
+      <c r="A51" s="254" t="s">
+        <v>665</v>
       </c>
       <c r="B51" s="195"/>
       <c r="C51" s="195"/>
@@ -14747,8 +14747,8 @@
       <c r="N51" s="196"/>
     </row>
     <row r="52" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="253" t="s">
-        <v>667</v>
+      <c r="A52" s="256" t="s">
+        <v>666</v>
       </c>
       <c r="B52" s="195"/>
       <c r="C52" s="195"/>
@@ -14765,8 +14765,8 @@
       <c r="N52" s="196"/>
     </row>
     <row r="53" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="251" t="s">
-        <v>668</v>
+      <c r="A53" s="254" t="s">
+        <v>667</v>
       </c>
       <c r="B53" s="195"/>
       <c r="C53" s="195"/>
@@ -14783,8 +14783,8 @@
       <c r="N53" s="196"/>
     </row>
     <row r="54" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="253" t="s">
-        <v>669</v>
+      <c r="A54" s="256" t="s">
+        <v>668</v>
       </c>
       <c r="B54" s="195"/>
       <c r="C54" s="195"/>
@@ -14801,8 +14801,8 @@
       <c r="N54" s="196"/>
     </row>
     <row r="55" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="251" t="s">
-        <v>670</v>
+      <c r="A55" s="254" t="s">
+        <v>669</v>
       </c>
       <c r="B55" s="195"/>
       <c r="C55" s="195"/>
@@ -14819,8 +14819,8 @@
       <c r="N55" s="196"/>
     </row>
     <row r="56" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="253" t="s">
-        <v>671</v>
+      <c r="A56" s="256" t="s">
+        <v>670</v>
       </c>
       <c r="B56" s="195"/>
       <c r="C56" s="195"/>
@@ -14837,8 +14837,8 @@
       <c r="N56" s="196"/>
     </row>
     <row r="57" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="251" t="s">
-        <v>672</v>
+      <c r="A57" s="254" t="s">
+        <v>671</v>
       </c>
       <c r="B57" s="195"/>
       <c r="C57" s="195"/>
@@ -14856,31 +14856,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A55:N55"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A50:N50"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="A54:N54"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="A51:N51"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="A34:N34"/>
     <mergeCell ref="A57:N57"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B25:D25"/>
@@ -14894,6 +14869,31 @@
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="A56:N56"/>
     <mergeCell ref="A27:N27"/>
+    <mergeCell ref="A55:N55"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A50:N50"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="A54:N54"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="A51:N51"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="A34:N34"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel actualizado automáticamente — 24/06/2026 14:04
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -3306,6 +3306,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="587" t="inlineStr">
         <is>
@@ -4335,6 +4336,7 @@
       <c r="C63" s="251" t="n"/>
       <c r="D63" s="252" t="n"/>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="604" t="inlineStr">
         <is>
@@ -4367,7 +4369,7 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>HOY 22 jun: Lagos105+Pedro(PM) · ALTHEON Barcelona(Laia+Alejandra) · Tepeyac mié24 · PSN primera reunión mié 1jul · Ibiza visita obra(Sara) · Paula vacaciones desde hoy</t>
+          <t>HOY 22 jun: Lagos105+Pedro(PM) · ALTHEON Barcelona(Laia+Alejandra) · Tepeyac mié24 · PSN primera reunión mié 1jul · Ibiza visita obra(Sara) · Paula vacaciones desde mañana 25 jun</t>
         </is>
       </c>
       <c r="C67" s="251" t="n"/>
@@ -4443,6 +4445,7 @@
       <c r="C72" s="251" t="n"/>
       <c r="D72" s="252" t="n"/>
     </row>
+    <row r="73"/>
     <row r="74">
       <c r="A74" s="537" t="inlineStr">
         <is>
@@ -11741,12 +11744,12 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Tepeyac: reunión cliente mié 24 jun (antes de irse o delegada?)</t>
-        </is>
-      </c>
-      <c r="E6" s="165" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
+          <t>🏖 VACACIONES desde mañana 25 jun hasta 21 ago · TEPEYAC: ✅ cliente aprueba distribución · reunión presupuesto sem29jun con Raúl+Alejandra+PM (Paula ya de vacaciones — confirmar si asiste o se ajusta fecha)</t>
+        </is>
+      </c>
+      <c r="E6" s="487" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel actualizado automáticamente — 24/06/2026 14:07
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -4369,7 +4369,7 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>HOY 22 jun: Lagos105+Pedro(PM) · ALTHEON Barcelona(Laia+Alejandra) · Tepeyac mié24 · PSN primera reunión mié 1jul · Ibiza visita obra(Sara) · Paula vacaciones desde mañana 25 jun</t>
+          <t>HOY 22 jun: Lagos105+Pedro(PM) · ALTHEON Barcelona(Laia+Alejandra) · Tepeyac mié24 · PSN primera reunión mié 1jul · Ibiza visita obra(Sara) · Paula vacaciones 3-21 ago</t>
         </is>
       </c>
       <c r="C67" s="251" t="n"/>
@@ -11744,12 +11744,12 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>🏖 VACACIONES desde mañana 25 jun hasta 21 ago · TEPEYAC: ✅ cliente aprueba distribución · reunión presupuesto sem29jun con Raúl+Alejandra+PM (Paula ya de vacaciones — confirmar si asiste o se ajusta fecha)</t>
-        </is>
-      </c>
-      <c r="E6" s="487" t="inlineStr">
-        <is>
-          <t>VACACIONES</t>
+          <t>TEPEYAC: ✅ cliente aprueba distribución · reunión presupuesto sem29jun con Raúl+Alejandra+PM · Demolición prevista agosto · 🏖 Vacaciones 3-21 ago</t>
+        </is>
+      </c>
+      <c r="E6" s="165" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 26/06/2026 12:31
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javo\APESTUDIO Dropbox\Carpeta del equipo APESTUDIO\999_PM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6793C1-0DAC-4092-87E4-6C10184964DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFB5268-727C-4DD1-9FCC-E3279604408C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1385" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="641">
   <si>
     <t>RESUMEN SEMANAL · PARA ALEJANDRA</t>
   </si>
@@ -1869,9 +1869,6 @@
     <t>Nombre del proyecto</t>
   </si>
   <si>
-    <t>Cliente</t>
-  </si>
-  <si>
     <t>Departamento (VIV/HOT/REST)</t>
   </si>
   <si>
@@ -1881,9 +1878,6 @@
     <t>Fecha de entrada</t>
   </si>
   <si>
-    <t>PM externo del cliente</t>
-  </si>
-  <si>
     <t>2 · TIPO DE PROYECTO</t>
   </si>
   <si>
@@ -1896,9 +1890,6 @@
     <t>¿Incluye obra? (Sí/No)</t>
   </si>
   <si>
-    <t>¿Incluye montaje? (Sí/No · quién ejecuta)</t>
-  </si>
-  <si>
     <t>¿Constructora definida?</t>
   </si>
   <si>
@@ -1939,6 +1930,27 @@
   </si>
   <si>
     <t>⚠ 4 semanas antes del montaje: visita obra + planning constructora</t>
+  </si>
+  <si>
+    <t>Cliente/Perfil</t>
+  </si>
+  <si>
+    <t>Dirección</t>
+  </si>
+  <si>
+    <t>Persona de confianza</t>
+  </si>
+  <si>
+    <t>Equipo externo</t>
+  </si>
+  <si>
+    <t>Ubicación obra (Madrid, extrarradio, nacional, internacional)</t>
+  </si>
+  <si>
+    <t>Expectativa</t>
+  </si>
+  <si>
+    <t>Realidad</t>
   </si>
 </sst>
 </file>
@@ -2518,7 +2530,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -2567,11 +2579,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3060,8 +3098,23 @@
     <xf numFmtId="0" fontId="15" fillId="44" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="44" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9995,7 +10048,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
@@ -10033,193 +10086,211 @@
     </row>
     <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="90" t="s">
-        <v>613</v>
-      </c>
-      <c r="B6" s="167"/>
-      <c r="C6" s="168"/>
+        <v>634</v>
+      </c>
+      <c r="B6" s="174"/>
+      <c r="C6" s="175"/>
     </row>
     <row r="7" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="90" t="s">
-        <v>614</v>
-      </c>
-      <c r="B7" s="167"/>
-      <c r="C7" s="168"/>
+        <v>635</v>
+      </c>
+      <c r="B7" s="172"/>
+      <c r="C7" s="173"/>
     </row>
     <row r="8" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="90" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B8" s="167"/>
       <c r="C8" s="168"/>
     </row>
     <row r="9" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="90" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B9" s="167"/>
       <c r="C9" s="168"/>
     </row>
     <row r="10" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="90" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B10" s="167"/>
       <c r="C10" s="168"/>
     </row>
-    <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="90" t="s">
+        <v>636</v>
+      </c>
+      <c r="B11" s="167"/>
+      <c r="C11" s="168"/>
+    </row>
     <row r="12" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="157" t="s">
-        <v>618</v>
-      </c>
-      <c r="B12" s="165"/>
-      <c r="C12" s="94"/>
-    </row>
-    <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="91" t="s">
-        <v>619</v>
-      </c>
-      <c r="B13" s="169"/>
-      <c r="C13" s="170"/>
-    </row>
+      <c r="A12" s="90" t="s">
+        <v>637</v>
+      </c>
+      <c r="B12" s="167"/>
+      <c r="C12" s="168"/>
+    </row>
+    <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="91" t="s">
-        <v>620</v>
-      </c>
-      <c r="B14" s="169"/>
-      <c r="C14" s="170"/>
+      <c r="A14" s="157" t="s">
+        <v>616</v>
+      </c>
+      <c r="B14" s="165"/>
+      <c r="C14" s="94"/>
     </row>
     <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="91" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="B15" s="169"/>
       <c r="C15" s="170"/>
     </row>
     <row r="16" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="91" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="B16" s="169"/>
       <c r="C16" s="170"/>
     </row>
     <row r="17" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="91" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="B17" s="169"/>
       <c r="C17" s="170"/>
     </row>
-    <row r="18" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="91" t="s">
+        <v>638</v>
+      </c>
+      <c r="B18" s="169"/>
+      <c r="C18" s="170"/>
+    </row>
     <row r="19" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="171" t="s">
-        <v>624</v>
-      </c>
-      <c r="B19" s="172"/>
-      <c r="C19" s="172"/>
-    </row>
-    <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
-        <v>625</v>
-      </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-    </row>
+      <c r="A19" s="91" t="s">
+        <v>620</v>
+      </c>
+      <c r="B19" s="169"/>
+      <c r="C19" s="170"/>
+    </row>
+    <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
-        <v>626</v>
-      </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
+      <c r="A21" s="171" t="s">
+        <v>621</v>
+      </c>
+      <c r="B21" s="176" t="s">
+        <v>639</v>
+      </c>
+      <c r="C21" s="177" t="s">
+        <v>640</v>
+      </c>
     </row>
     <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
     </row>
     <row r="23" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
     </row>
     <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
     </row>
-    <row r="25" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+    </row>
     <row r="26" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="158" t="s">
-        <v>630</v>
-      </c>
-      <c r="B26" s="166"/>
-      <c r="C26" s="94"/>
-    </row>
-    <row r="27" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="92" t="s">
-        <v>631</v>
-      </c>
-      <c r="B27" s="92"/>
-      <c r="C27" s="5"/>
-    </row>
+      <c r="A26" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+    </row>
+    <row r="27" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="92" t="s">
-        <v>632</v>
-      </c>
-      <c r="B28" s="92"/>
-      <c r="C28" s="5"/>
-    </row>
-    <row r="29" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="158" t="s">
+        <v>627</v>
+      </c>
+      <c r="B28" s="166"/>
+      <c r="C28" s="94"/>
+    </row>
+    <row r="29" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="92" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="B29" s="92"/>
       <c r="C29" s="5"/>
     </row>
     <row r="30" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="92" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="B30" s="92"/>
       <c r="C30" s="5"/>
     </row>
     <row r="31" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="92" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="B31" s="92"/>
       <c r="C31" s="5"/>
     </row>
-    <row r="32" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="92" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="B32" s="92"/>
       <c r="C32" s="5"/>
+    </row>
+    <row r="33" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="92" t="s">
+        <v>632</v>
+      </c>
+      <c r="B33" s="92"/>
+      <c r="C33" s="5"/>
+    </row>
+    <row r="34" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="92" t="s">
+        <v>633</v>
+      </c>
+      <c r="B34" s="92"/>
+      <c r="C34" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A28:C28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 26/06/2026 12:38
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javo\APESTUDIO Dropbox\Carpeta del equipo APESTUDIO\999_PM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFB5268-727C-4DD1-9FCC-E3279604408C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FF013-5A94-4E4C-9B93-C4D0CF34530A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="642">
   <si>
     <t>RESUMEN SEMANAL · PARA ALEJANDRA</t>
   </si>
@@ -1914,21 +1914,6 @@
     <t>4 · CHECKLIST ANTES DE COMPROMETER FECHAS</t>
   </si>
   <si>
-    <t>¿Cuántos proyectos activos tiene Challan? (máx 2-3)</t>
-  </si>
-  <si>
-    <t>¿Constructora disponible?</t>
-  </si>
-  <si>
-    <t>¿Responsable tiene hueco?</t>
-  </si>
-  <si>
-    <t>¿Vacaciones del equipo afectan hitos?</t>
-  </si>
-  <si>
-    <t>¿Hitos caen en agosto (Challan vac 1-15ago)?</t>
-  </si>
-  <si>
     <t>⚠ 4 semanas antes del montaje: visita obra + planning constructora</t>
   </si>
   <si>
@@ -1941,9 +1926,6 @@
     <t>Persona de confianza</t>
   </si>
   <si>
-    <t>Equipo externo</t>
-  </si>
-  <si>
     <t>Ubicación obra (Madrid, extrarradio, nacional, internacional)</t>
   </si>
   <si>
@@ -1951,6 +1933,27 @@
   </si>
   <si>
     <t>Realidad</t>
+  </si>
+  <si>
+    <t>Equipo externo (PM, arquitecto, constructora, paisajista)</t>
+  </si>
+  <si>
+    <t>Hitos clave reflejados en Planing de departamento?</t>
+  </si>
+  <si>
+    <t>Proyecto añadido al Master Global con fases?</t>
+  </si>
+  <si>
+    <t>Responsable añadido a Foco por Persona?</t>
+  </si>
+  <si>
+    <t>Se ha comprobado disponibilidad de renderista?</t>
+  </si>
+  <si>
+    <t>Se han cruzado vacaciones del equipo?</t>
+  </si>
+  <si>
+    <t>PRESUPUESTO ESTIMADO (OBRA/DECO)</t>
   </si>
 </sst>
 </file>
@@ -2609,7 +2612,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="180">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3110,11 +3113,22 @@
     <xf numFmtId="0" fontId="6" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="44" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3131,6 +3145,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10048,7 +10079,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
@@ -10086,14 +10117,14 @@
     </row>
     <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="90" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="B6" s="174"/>
       <c r="C6" s="175"/>
     </row>
     <row r="7" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="90" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="B7" s="172"/>
       <c r="C7" s="173"/>
@@ -10121,157 +10152,176 @@
     </row>
     <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="90" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="B11" s="167"/>
       <c r="C11" s="168"/>
     </row>
     <row r="12" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="90" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B12" s="167"/>
       <c r="C12" s="168"/>
     </row>
-    <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="157" t="s">
+    <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="176" t="s">
+        <v>641</v>
+      </c>
+      <c r="B13" s="174"/>
+      <c r="C13" s="175"/>
+    </row>
+    <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="157" t="s">
         <v>616</v>
       </c>
-      <c r="B14" s="165"/>
-      <c r="C14" s="94"/>
-    </row>
-    <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="91" t="s">
-        <v>617</v>
-      </c>
-      <c r="B15" s="169"/>
-      <c r="C15" s="170"/>
+      <c r="B15" s="165"/>
+      <c r="C15" s="94"/>
     </row>
     <row r="16" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="91" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B16" s="169"/>
       <c r="C16" s="170"/>
     </row>
     <row r="17" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="91" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B17" s="169"/>
       <c r="C17" s="170"/>
     </row>
     <row r="18" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="91" t="s">
-        <v>638</v>
+        <v>619</v>
       </c>
       <c r="B18" s="169"/>
       <c r="C18" s="170"/>
     </row>
     <row r="19" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="91" t="s">
-        <v>620</v>
+        <v>632</v>
       </c>
       <c r="B19" s="169"/>
       <c r="C19" s="170"/>
     </row>
-    <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="171" t="s">
+    <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="91" t="s">
+        <v>620</v>
+      </c>
+      <c r="B20" s="169"/>
+      <c r="C20" s="170"/>
+    </row>
+    <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="171" t="s">
         <v>621</v>
       </c>
-      <c r="B21" s="176" t="s">
-        <v>639</v>
-      </c>
-      <c r="C21" s="177" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
+      <c r="B22" s="177" t="s">
+        <v>633</v>
+      </c>
+      <c r="C22" s="178" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="23" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
     </row>
     <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
     </row>
     <row r="25" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
     </row>
     <row r="26" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
     </row>
-    <row r="27" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="158" t="s">
+    <row r="27" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+    </row>
+    <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="158" t="s">
         <v>627</v>
       </c>
-      <c r="B28" s="166"/>
-      <c r="C28" s="94"/>
-    </row>
-    <row r="29" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="92" t="s">
-        <v>628</v>
-      </c>
-      <c r="B29" s="92"/>
-      <c r="C29" s="5"/>
-    </row>
-    <row r="30" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="166"/>
+      <c r="C29" s="94"/>
+    </row>
+    <row r="30" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="92" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
       <c r="B30" s="92"/>
-      <c r="C30" s="5"/>
+      <c r="C30" s="179" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="92" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="B31" s="92"/>
-      <c r="C31" s="5"/>
+      <c r="C31" s="179" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="92" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="B32" s="92"/>
-      <c r="C32" s="5"/>
+      <c r="C32" s="179" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="92" t="s">
-        <v>632</v>
+        <v>639</v>
       </c>
       <c r="B33" s="92"/>
-      <c r="C33" s="5"/>
-    </row>
-    <row r="34" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C33" s="179" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="92" t="s">
-        <v>633</v>
+        <v>640</v>
       </c>
       <c r="B34" s="92"/>
-      <c r="C34" s="5"/>
+      <c r="C34" s="179" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="92" t="s">
+        <v>628</v>
+      </c>
+      <c r="B35" s="92"/>
+      <c r="C35" s="179" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -10280,17 +10330,17 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 26/06/2026 12:39
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javo\APESTUDIO Dropbox\Carpeta del equipo APESTUDIO\999_PM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FF013-5A94-4E4C-9B93-C4D0CF34530A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBED7B9-1AE9-4EBC-B61F-A3552457963D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1914,9 +1914,6 @@
     <t>4 · CHECKLIST ANTES DE COMPROMETER FECHAS</t>
   </si>
   <si>
-    <t>⚠ 4 semanas antes del montaje: visita obra + planning constructora</t>
-  </si>
-  <si>
     <t>Cliente/Perfil</t>
   </si>
   <si>
@@ -1954,13 +1951,16 @@
   </si>
   <si>
     <t>PRESUPUESTO ESTIMADO (OBRA/DECO)</t>
+  </si>
+  <si>
+    <t>Posibles comisiones proveedores</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="57" x14ac:knownFonts="1">
+  <fonts count="58" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2299,6 +2299,14 @@
       <color rgb="FFE67E22"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF1C1C1C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="47">
     <fill>
@@ -3113,9 +3121,6 @@
     <xf numFmtId="0" fontId="6" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3129,6 +3134,9 @@
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10117,14 +10125,14 @@
     </row>
     <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="90" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B6" s="174"/>
       <c r="C6" s="175"/>
     </row>
     <row r="7" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="90" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B7" s="172"/>
       <c r="C7" s="173"/>
@@ -10152,174 +10160,172 @@
     </row>
     <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="90" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B11" s="167"/>
       <c r="C11" s="168"/>
     </row>
     <row r="12" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="90" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B12" s="167"/>
       <c r="C12" s="168"/>
     </row>
     <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="176" t="s">
-        <v>641</v>
+      <c r="A13" s="179" t="s">
+        <v>640</v>
       </c>
       <c r="B13" s="174"/>
       <c r="C13" s="175"/>
     </row>
-    <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="157" t="s">
+    <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="90" t="s">
+        <v>641</v>
+      </c>
+      <c r="B14" s="174"/>
+      <c r="C14" s="175"/>
+    </row>
+    <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="157" t="s">
         <v>616</v>
       </c>
-      <c r="B15" s="165"/>
-      <c r="C15" s="94"/>
-    </row>
-    <row r="16" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="91" t="s">
-        <v>617</v>
-      </c>
-      <c r="B16" s="169"/>
-      <c r="C16" s="170"/>
+      <c r="B16" s="165"/>
+      <c r="C16" s="94"/>
     </row>
     <row r="17" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="91" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B17" s="169"/>
       <c r="C17" s="170"/>
     </row>
     <row r="18" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="91" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B18" s="169"/>
       <c r="C18" s="170"/>
     </row>
     <row r="19" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="91" t="s">
-        <v>632</v>
+        <v>619</v>
       </c>
       <c r="B19" s="169"/>
       <c r="C19" s="170"/>
     </row>
     <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="91" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="B20" s="169"/>
       <c r="C20" s="170"/>
     </row>
-    <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="171" t="s">
+    <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="91" t="s">
+        <v>620</v>
+      </c>
+      <c r="B21" s="169"/>
+      <c r="C21" s="170"/>
+    </row>
+    <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="23" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="171" t="s">
         <v>621</v>
       </c>
-      <c r="B22" s="177" t="s">
+      <c r="B23" s="176" t="s">
+        <v>632</v>
+      </c>
+      <c r="C23" s="177" t="s">
         <v>633</v>
       </c>
-      <c r="C22" s="178" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
     </row>
     <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
     </row>
     <row r="25" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
     </row>
     <row r="26" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
     </row>
     <row r="27" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
     </row>
-    <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="29" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="158" t="s">
+    <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+    </row>
+    <row r="29" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="158" t="s">
         <v>627</v>
       </c>
-      <c r="B29" s="166"/>
-      <c r="C29" s="94"/>
-    </row>
-    <row r="30" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="92" t="s">
-        <v>637</v>
-      </c>
-      <c r="B30" s="92"/>
-      <c r="C30" s="179" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="166"/>
+      <c r="C30" s="94"/>
+    </row>
+    <row r="31" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="92" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B31" s="92"/>
-      <c r="C31" s="179" t="b">
+      <c r="C31" s="178" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="92" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B32" s="92"/>
-      <c r="C32" s="179" t="b">
+      <c r="C32" s="178" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="92" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="B33" s="92"/>
-      <c r="C33" s="179" t="b">
+      <c r="C33" s="178" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="92" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B34" s="92"/>
-      <c r="C34" s="179" t="b">
+      <c r="C34" s="178" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="92" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="B35" s="92"/>
-      <c r="C35" s="179" t="b">
+      <c r="C35" s="178" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10330,17 +10336,17 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B21:C21"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A30:C30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 30/06/2026 11:31
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javo\APESTUDIO Dropbox\Carpeta del equipo APESTUDIO\999_PM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{816E9427-1538-4AE8-9B6F-066478FDBD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9F3538-C559-4980-9FD9-EDEA88B77AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Resumen Alejandra" sheetId="1" r:id="rId1"/>
@@ -2793,11 +2793,91 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="51" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="54" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="44" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2807,126 +2887,65 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="53" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="49" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="43" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2934,28 +2953,9 @@
     <xf numFmtId="0" fontId="31" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="43" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="44" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="43" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2971,44 +2971,44 @@
     <xf numFmtId="0" fontId="4" fillId="45" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="57" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="60" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="59" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3322,28 +3322,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="117" t="s">
+      <c r="A2" s="125" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
-      <c r="C2" s="108"/>
-      <c r="D2" s="108"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
     </row>
     <row r="4" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="105" t="s">
+      <c r="A4" s="133" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="101"/>
-      <c r="C4" s="101"/>
-      <c r="D4" s="102"/>
+      <c r="B4" s="104"/>
+      <c r="C4" s="104"/>
+      <c r="D4" s="105"/>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -3472,12 +3472,12 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="112" t="s">
+      <c r="A15" s="134" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="101"/>
-      <c r="C15" s="101"/>
-      <c r="D15" s="102"/>
+      <c r="B15" s="104"/>
+      <c r="C15" s="104"/>
+      <c r="D15" s="105"/>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
@@ -3610,12 +3610,12 @@
       <c r="D26" s="96"/>
     </row>
     <row r="27" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="116" t="s">
+      <c r="A27" s="124" t="s">
         <v>59</v>
       </c>
-      <c r="B27" s="101"/>
-      <c r="C27" s="101"/>
-      <c r="D27" s="102"/>
+      <c r="B27" s="104"/>
+      <c r="C27" s="104"/>
+      <c r="D27" s="105"/>
     </row>
     <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
@@ -3758,229 +3758,219 @@
       </c>
     </row>
     <row r="39" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="111" t="s">
+      <c r="A39" s="128" t="s">
         <v>95</v>
       </c>
-      <c r="B39" s="101"/>
-      <c r="C39" s="101"/>
-      <c r="D39" s="102"/>
+      <c r="B39" s="104"/>
+      <c r="C39" s="104"/>
+      <c r="D39" s="105"/>
     </row>
     <row r="40" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="109" t="s">
+      <c r="A40" s="127" t="s">
         <v>96</v>
       </c>
-      <c r="B40" s="108"/>
-      <c r="C40" s="108"/>
-      <c r="D40" s="108"/>
+      <c r="B40" s="101"/>
+      <c r="C40" s="101"/>
+      <c r="D40" s="101"/>
     </row>
     <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="B41" s="114" t="s">
+      <c r="B41" s="122" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="101"/>
-      <c r="D41" s="102"/>
+      <c r="C41" s="104"/>
+      <c r="D41" s="105"/>
     </row>
     <row r="42" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="B42" s="100" t="s">
+      <c r="B42" s="123" t="s">
         <v>100</v>
       </c>
-      <c r="C42" s="101"/>
-      <c r="D42" s="102"/>
+      <c r="C42" s="104"/>
+      <c r="D42" s="105"/>
     </row>
     <row r="43" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="110" t="s">
+      <c r="B43" s="121" t="s">
         <v>101</v>
       </c>
-      <c r="C43" s="101"/>
-      <c r="D43" s="102"/>
+      <c r="C43" s="104"/>
+      <c r="D43" s="105"/>
     </row>
     <row r="44" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B44" s="100" t="s">
+      <c r="B44" s="123" t="s">
         <v>102</v>
       </c>
-      <c r="C44" s="101"/>
-      <c r="D44" s="102"/>
+      <c r="C44" s="104"/>
+      <c r="D44" s="105"/>
     </row>
     <row r="45" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="110" t="s">
+      <c r="B45" s="121" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="101"/>
-      <c r="D45" s="102"/>
+      <c r="C45" s="104"/>
+      <c r="D45" s="105"/>
     </row>
     <row r="46" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="B46" s="100" t="s">
+      <c r="B46" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="C46" s="101"/>
-      <c r="D46" s="102"/>
+      <c r="C46" s="104"/>
+      <c r="D46" s="105"/>
     </row>
     <row r="47" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="110" t="s">
+      <c r="B47" s="121" t="s">
         <v>105</v>
       </c>
-      <c r="C47" s="101"/>
-      <c r="D47" s="102"/>
+      <c r="C47" s="104"/>
+      <c r="D47" s="105"/>
     </row>
     <row r="48" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="100" t="s">
+      <c r="B48" s="123" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="101"/>
-      <c r="D48" s="102"/>
+      <c r="C48" s="104"/>
+      <c r="D48" s="105"/>
     </row>
     <row r="49" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="B49" s="110" t="s">
+      <c r="B49" s="121" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="101"/>
-      <c r="D49" s="102"/>
+      <c r="C49" s="104"/>
+      <c r="D49" s="105"/>
     </row>
     <row r="50" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B50" s="100" t="s">
+      <c r="B50" s="123" t="s">
         <v>109</v>
       </c>
-      <c r="C50" s="101"/>
-      <c r="D50" s="102"/>
+      <c r="C50" s="104"/>
+      <c r="D50" s="105"/>
     </row>
     <row r="51" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B51" s="110" t="s">
+      <c r="B51" s="121" t="s">
         <v>111</v>
       </c>
-      <c r="C51" s="101"/>
-      <c r="D51" s="102"/>
+      <c r="C51" s="104"/>
+      <c r="D51" s="105"/>
     </row>
     <row r="53" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="104" t="s">
+      <c r="A53" s="132" t="s">
         <v>112</v>
       </c>
-      <c r="B53" s="101"/>
-      <c r="C53" s="101"/>
-      <c r="D53" s="102"/>
+      <c r="B53" s="104"/>
+      <c r="C53" s="104"/>
+      <c r="D53" s="105"/>
     </row>
     <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B54" s="115" t="s">
+      <c r="B54" s="130" t="s">
         <v>114</v>
       </c>
-      <c r="C54" s="101"/>
-      <c r="D54" s="102"/>
+      <c r="C54" s="104"/>
+      <c r="D54" s="105"/>
     </row>
     <row r="55" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B55" s="106" t="s">
+      <c r="B55" s="129" t="s">
         <v>116</v>
       </c>
-      <c r="C55" s="101"/>
-      <c r="D55" s="102"/>
+      <c r="C55" s="104"/>
+      <c r="D55" s="105"/>
     </row>
     <row r="56" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="B56" s="103" t="s">
+      <c r="B56" s="131" t="s">
         <v>118</v>
       </c>
-      <c r="C56" s="101"/>
-      <c r="D56" s="102"/>
+      <c r="C56" s="104"/>
+      <c r="D56" s="105"/>
     </row>
     <row r="57" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="B57" s="106" t="s">
+      <c r="B57" s="129" t="s">
         <v>120</v>
       </c>
-      <c r="C57" s="101"/>
-      <c r="D57" s="102"/>
+      <c r="C57" s="104"/>
+      <c r="D57" s="105"/>
     </row>
     <row r="58" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="B58" s="103" t="s">
+      <c r="B58" s="131" t="s">
         <v>122</v>
       </c>
-      <c r="C58" s="101"/>
-      <c r="D58" s="102"/>
+      <c r="C58" s="104"/>
+      <c r="D58" s="105"/>
     </row>
     <row r="59" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="B59" s="106" t="s">
+      <c r="B59" s="129" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="101"/>
-      <c r="D59" s="102"/>
+      <c r="C59" s="104"/>
+      <c r="D59" s="105"/>
     </row>
     <row r="60" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B60" s="103" t="s">
+      <c r="B60" s="131" t="s">
         <v>125</v>
       </c>
-      <c r="C60" s="101"/>
-      <c r="D60" s="102"/>
+      <c r="C60" s="104"/>
+      <c r="D60" s="105"/>
     </row>
     <row r="62" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="107" t="s">
+      <c r="A62" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="B62" s="108"/>
-      <c r="C62" s="108"/>
-      <c r="D62" s="108"/>
+      <c r="B62" s="101"/>
+      <c r="C62" s="101"/>
+      <c r="D62" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B48:D48"/>
     <mergeCell ref="A62:D62"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="A40:D40"/>
@@ -3995,8 +3985,18 @@
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B60:D60"/>
     <mergeCell ref="A53:D53"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B48:D48"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="B57:D57"/>
     <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4013,7 +4013,7 @@
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="44" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="6" max="6" width="24.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
@@ -4022,36 +4022,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="135" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="102"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="105"/>
     </row>
     <row r="2" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="121" t="s">
+      <c r="A2" s="142" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="102"/>
+      <c r="B2" s="104"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="104"/>
+      <c r="K2" s="104"/>
+      <c r="L2" s="105"/>
     </row>
     <row r="3" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="22" t="s">
@@ -4064,7 +4064,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>131</v>
@@ -4089,20 +4089,20 @@
       </c>
     </row>
     <row r="4" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="123" t="s">
+      <c r="A4" s="139" t="s">
         <v>136</v>
       </c>
-      <c r="B4" s="108"/>
-      <c r="C4" s="108"/>
-      <c r="D4" s="108"/>
-      <c r="E4" s="108"/>
-      <c r="F4" s="108"/>
-      <c r="G4" s="108"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="108"/>
-      <c r="J4" s="108"/>
-      <c r="K4" s="108"/>
-      <c r="L4" s="108"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="101"/>
+      <c r="D4" s="101"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="101"/>
+      <c r="J4" s="101"/>
+      <c r="K4" s="101"/>
+      <c r="L4" s="101"/>
     </row>
     <row r="5" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
@@ -5581,28 +5581,28 @@
       </c>
     </row>
     <row r="49" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="124" t="s">
+      <c r="A49" s="141" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="124" t="s">
+      <c r="B49" s="141" t="s">
         <v>129</v>
       </c>
-      <c r="C49" s="124" t="s">
+      <c r="C49" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="D49" s="124" t="s">
+      <c r="D49" s="141" t="s">
         <v>361</v>
       </c>
-      <c r="E49" s="124" t="s">
+      <c r="E49" s="141" t="s">
         <v>362</v>
       </c>
-      <c r="F49" s="124"/>
-      <c r="G49" s="124"/>
-      <c r="H49" s="124"/>
-      <c r="I49" s="124"/>
-      <c r="J49" s="124"/>
-      <c r="K49" s="124"/>
-      <c r="L49" s="108"/>
+      <c r="F49" s="141"/>
+      <c r="G49" s="141"/>
+      <c r="H49" s="141"/>
+      <c r="I49" s="141"/>
+      <c r="J49" s="141"/>
+      <c r="K49" s="141"/>
+      <c r="L49" s="101"/>
     </row>
     <row r="50" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="46" t="s">
@@ -5637,18 +5637,18 @@
       <c r="C51" s="51" t="s">
         <v>142</v>
       </c>
-      <c r="D51" s="118" t="s">
+      <c r="D51" s="140" t="s">
         <v>366</v>
       </c>
-      <c r="E51" s="101"/>
-      <c r="F51" s="101"/>
-      <c r="G51" s="101"/>
-      <c r="H51" s="101"/>
-      <c r="I51" s="102"/>
-      <c r="J51" s="120" t="s">
+      <c r="E51" s="104"/>
+      <c r="F51" s="104"/>
+      <c r="G51" s="104"/>
+      <c r="H51" s="104"/>
+      <c r="I51" s="105"/>
+      <c r="J51" s="137" t="s">
         <v>227</v>
       </c>
-      <c r="K51" s="102"/>
+      <c r="K51" s="105"/>
     </row>
     <row r="52" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="46" t="s">
@@ -5660,18 +5660,18 @@
       <c r="C52" s="47" t="s">
         <v>312</v>
       </c>
-      <c r="D52" s="122" t="s">
+      <c r="D52" s="138" t="s">
         <v>368</v>
       </c>
-      <c r="E52" s="101"/>
-      <c r="F52" s="101"/>
-      <c r="G52" s="101"/>
-      <c r="H52" s="101"/>
-      <c r="I52" s="102"/>
-      <c r="J52" s="119" t="s">
+      <c r="E52" s="104"/>
+      <c r="F52" s="104"/>
+      <c r="G52" s="104"/>
+      <c r="H52" s="104"/>
+      <c r="I52" s="105"/>
+      <c r="J52" s="136" t="s">
         <v>274</v>
       </c>
-      <c r="K52" s="102"/>
+      <c r="K52" s="105"/>
     </row>
     <row r="53" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="50" t="s">
@@ -5683,18 +5683,18 @@
       <c r="C53" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="D53" s="118" t="s">
+      <c r="D53" s="140" t="s">
         <v>368</v>
       </c>
-      <c r="E53" s="101"/>
-      <c r="F53" s="101"/>
-      <c r="G53" s="101"/>
-      <c r="H53" s="101"/>
-      <c r="I53" s="102"/>
-      <c r="J53" s="120" t="s">
+      <c r="E53" s="104"/>
+      <c r="F53" s="104"/>
+      <c r="G53" s="104"/>
+      <c r="H53" s="104"/>
+      <c r="I53" s="105"/>
+      <c r="J53" s="137" t="s">
         <v>274</v>
       </c>
-      <c r="K53" s="102"/>
+      <c r="K53" s="105"/>
     </row>
     <row r="54" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="46" t="s">
@@ -5706,18 +5706,18 @@
       <c r="C54" s="47" t="s">
         <v>351</v>
       </c>
-      <c r="D54" s="122" t="s">
+      <c r="D54" s="138" t="s">
         <v>371</v>
       </c>
-      <c r="E54" s="101"/>
-      <c r="F54" s="101"/>
-      <c r="G54" s="101"/>
-      <c r="H54" s="101"/>
-      <c r="I54" s="102"/>
-      <c r="J54" s="119" t="s">
+      <c r="E54" s="104"/>
+      <c r="F54" s="104"/>
+      <c r="G54" s="104"/>
+      <c r="H54" s="104"/>
+      <c r="I54" s="105"/>
+      <c r="J54" s="136" t="s">
         <v>227</v>
       </c>
-      <c r="K54" s="102"/>
+      <c r="K54" s="105"/>
     </row>
     <row r="55" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="50" t="s">
@@ -5729,18 +5729,18 @@
       <c r="C55" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="D55" s="118" t="s">
+      <c r="D55" s="140" t="s">
         <v>373</v>
       </c>
-      <c r="E55" s="101"/>
-      <c r="F55" s="101"/>
-      <c r="G55" s="101"/>
-      <c r="H55" s="101"/>
-      <c r="I55" s="102"/>
-      <c r="J55" s="120" t="s">
+      <c r="E55" s="104"/>
+      <c r="F55" s="104"/>
+      <c r="G55" s="104"/>
+      <c r="H55" s="104"/>
+      <c r="I55" s="105"/>
+      <c r="J55" s="137" t="s">
         <v>227</v>
       </c>
-      <c r="K55" s="102"/>
+      <c r="K55" s="105"/>
     </row>
     <row r="56" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="46" t="s">
@@ -5752,18 +5752,18 @@
       <c r="C56" s="47" t="s">
         <v>328</v>
       </c>
-      <c r="D56" s="122" t="s">
+      <c r="D56" s="138" t="s">
         <v>374</v>
       </c>
-      <c r="E56" s="101"/>
-      <c r="F56" s="101"/>
-      <c r="G56" s="101"/>
-      <c r="H56" s="101"/>
-      <c r="I56" s="102"/>
-      <c r="J56" s="119" t="s">
+      <c r="E56" s="104"/>
+      <c r="F56" s="104"/>
+      <c r="G56" s="104"/>
+      <c r="H56" s="104"/>
+      <c r="I56" s="105"/>
+      <c r="J56" s="136" t="s">
         <v>331</v>
       </c>
-      <c r="K56" s="102"/>
+      <c r="K56" s="105"/>
     </row>
     <row r="57" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="50" t="s">
@@ -5775,18 +5775,18 @@
       <c r="C57" s="51" t="s">
         <v>266</v>
       </c>
-      <c r="D57" s="118" t="s">
+      <c r="D57" s="140" t="s">
         <v>376</v>
       </c>
-      <c r="E57" s="101"/>
-      <c r="F57" s="101"/>
-      <c r="G57" s="101"/>
-      <c r="H57" s="101"/>
-      <c r="I57" s="102"/>
-      <c r="J57" s="120" t="s">
+      <c r="E57" s="104"/>
+      <c r="F57" s="104"/>
+      <c r="G57" s="104"/>
+      <c r="H57" s="104"/>
+      <c r="I57" s="105"/>
+      <c r="J57" s="137" t="s">
         <v>227</v>
       </c>
-      <c r="K57" s="102"/>
+      <c r="K57" s="105"/>
     </row>
     <row r="58" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="46" t="s">
@@ -5798,18 +5798,18 @@
       <c r="C58" s="47" t="s">
         <v>266</v>
       </c>
-      <c r="D58" s="122" t="s">
+      <c r="D58" s="138" t="s">
         <v>378</v>
       </c>
-      <c r="E58" s="101"/>
-      <c r="F58" s="101"/>
-      <c r="G58" s="101"/>
-      <c r="H58" s="101"/>
-      <c r="I58" s="102"/>
-      <c r="J58" s="119" t="s">
+      <c r="E58" s="104"/>
+      <c r="F58" s="104"/>
+      <c r="G58" s="104"/>
+      <c r="H58" s="104"/>
+      <c r="I58" s="105"/>
+      <c r="J58" s="136" t="s">
         <v>227</v>
       </c>
-      <c r="K58" s="102"/>
+      <c r="K58" s="105"/>
     </row>
     <row r="59" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="50" t="s">
@@ -5821,18 +5821,18 @@
       <c r="C59" s="51" t="s">
         <v>266</v>
       </c>
-      <c r="D59" s="118" t="s">
+      <c r="D59" s="140" t="s">
         <v>378</v>
       </c>
-      <c r="E59" s="101"/>
-      <c r="F59" s="101"/>
-      <c r="G59" s="101"/>
-      <c r="H59" s="101"/>
-      <c r="I59" s="102"/>
-      <c r="J59" s="120" t="s">
+      <c r="E59" s="104"/>
+      <c r="F59" s="104"/>
+      <c r="G59" s="104"/>
+      <c r="H59" s="104"/>
+      <c r="I59" s="105"/>
+      <c r="J59" s="137" t="s">
         <v>227</v>
       </c>
-      <c r="K59" s="102"/>
+      <c r="K59" s="105"/>
     </row>
     <row r="60" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="46" t="s">
@@ -5844,18 +5844,18 @@
       <c r="C60" s="47" t="s">
         <v>266</v>
       </c>
-      <c r="D60" s="122" t="s">
+      <c r="D60" s="138" t="s">
         <v>381</v>
       </c>
-      <c r="E60" s="101"/>
-      <c r="F60" s="101"/>
-      <c r="G60" s="101"/>
-      <c r="H60" s="101"/>
-      <c r="I60" s="102"/>
-      <c r="J60" s="119" t="s">
+      <c r="E60" s="104"/>
+      <c r="F60" s="104"/>
+      <c r="G60" s="104"/>
+      <c r="H60" s="104"/>
+      <c r="I60" s="105"/>
+      <c r="J60" s="136" t="s">
         <v>227</v>
       </c>
-      <c r="K60" s="102"/>
+      <c r="K60" s="105"/>
     </row>
     <row r="61" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="50" t="s">
@@ -5867,18 +5867,18 @@
       <c r="C61" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="D61" s="118" t="s">
+      <c r="D61" s="140" t="s">
         <v>383</v>
       </c>
-      <c r="E61" s="101"/>
-      <c r="F61" s="101"/>
-      <c r="G61" s="101"/>
-      <c r="H61" s="101"/>
-      <c r="I61" s="102"/>
-      <c r="J61" s="120" t="s">
+      <c r="E61" s="104"/>
+      <c r="F61" s="104"/>
+      <c r="G61" s="104"/>
+      <c r="H61" s="104"/>
+      <c r="I61" s="105"/>
+      <c r="J61" s="137" t="s">
         <v>227</v>
       </c>
-      <c r="K61" s="102"/>
+      <c r="K61" s="105"/>
     </row>
     <row r="62" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="46" t="s">
@@ -5890,18 +5890,18 @@
       <c r="C62" s="47" t="s">
         <v>266</v>
       </c>
-      <c r="D62" s="122" t="s">
+      <c r="D62" s="138" t="s">
         <v>385</v>
       </c>
-      <c r="E62" s="101"/>
-      <c r="F62" s="101"/>
-      <c r="G62" s="101"/>
-      <c r="H62" s="101"/>
-      <c r="I62" s="102"/>
-      <c r="J62" s="119" t="s">
+      <c r="E62" s="104"/>
+      <c r="F62" s="104"/>
+      <c r="G62" s="104"/>
+      <c r="H62" s="104"/>
+      <c r="I62" s="105"/>
+      <c r="J62" s="136" t="s">
         <v>227</v>
       </c>
-      <c r="K62" s="102"/>
+      <c r="K62" s="105"/>
     </row>
     <row r="63" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="50" t="s">
@@ -5913,18 +5913,18 @@
       <c r="C63" s="51" t="s">
         <v>266</v>
       </c>
-      <c r="D63" s="118" t="s">
+      <c r="D63" s="140" t="s">
         <v>385</v>
       </c>
-      <c r="E63" s="101"/>
-      <c r="F63" s="101"/>
-      <c r="G63" s="101"/>
-      <c r="H63" s="101"/>
-      <c r="I63" s="102"/>
-      <c r="J63" s="120" t="s">
+      <c r="E63" s="104"/>
+      <c r="F63" s="104"/>
+      <c r="G63" s="104"/>
+      <c r="H63" s="104"/>
+      <c r="I63" s="105"/>
+      <c r="J63" s="137" t="s">
         <v>227</v>
       </c>
-      <c r="K63" s="102"/>
+      <c r="K63" s="105"/>
     </row>
     <row r="64" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="46" t="s">
@@ -5936,31 +5936,49 @@
       <c r="C64" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="D64" s="122" t="s">
+      <c r="D64" s="138" t="s">
         <v>387</v>
       </c>
-      <c r="E64" s="101"/>
-      <c r="F64" s="101"/>
-      <c r="G64" s="101"/>
-      <c r="H64" s="101"/>
-      <c r="I64" s="102"/>
-      <c r="J64" s="119" t="s">
+      <c r="E64" s="104"/>
+      <c r="F64" s="104"/>
+      <c r="G64" s="104"/>
+      <c r="H64" s="104"/>
+      <c r="I64" s="105"/>
+      <c r="J64" s="136" t="s">
         <v>227</v>
       </c>
-      <c r="K64" s="102"/>
+      <c r="K64" s="105"/>
     </row>
     <row r="65" spans="4:11" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D65" s="108"/>
-      <c r="E65" s="108"/>
-      <c r="F65" s="108"/>
-      <c r="G65" s="108"/>
-      <c r="H65" s="108"/>
-      <c r="I65" s="108"/>
-      <c r="J65" s="108"/>
-      <c r="K65" s="108"/>
+      <c r="D65" s="101"/>
+      <c r="E65" s="101"/>
+      <c r="F65" s="101"/>
+      <c r="G65" s="101"/>
+      <c r="H65" s="101"/>
+      <c r="I65" s="101"/>
+      <c r="J65" s="101"/>
+      <c r="K65" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="J64:K64"/>
+    <mergeCell ref="D61:I61"/>
+    <mergeCell ref="J57:K57"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="D53:I53"/>
+    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="D62:I62"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="D56:I56"/>
+    <mergeCell ref="D58:I58"/>
+    <mergeCell ref="D57:I57"/>
+    <mergeCell ref="J63:K63"/>
+    <mergeCell ref="D59:I59"/>
+    <mergeCell ref="D60:I60"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="D63:I63"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="J62:K62"/>
     <mergeCell ref="J51:K51"/>
@@ -5977,24 +5995,6 @@
     <mergeCell ref="D51:I51"/>
     <mergeCell ref="J54:K54"/>
     <mergeCell ref="D54:I54"/>
-    <mergeCell ref="J63:K63"/>
-    <mergeCell ref="D59:I59"/>
-    <mergeCell ref="D60:I60"/>
-    <mergeCell ref="J56:K56"/>
-    <mergeCell ref="D63:I63"/>
-    <mergeCell ref="A49:L49"/>
-    <mergeCell ref="D53:I53"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="D62:I62"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="D56:I56"/>
-    <mergeCell ref="D58:I58"/>
-    <mergeCell ref="D57:I57"/>
-    <mergeCell ref="J64:K64"/>
-    <mergeCell ref="D61:I61"/>
-    <mergeCell ref="J57:K57"/>
-    <mergeCell ref="J59:K59"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6013,14 +6013,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="135" t="s">
         <v>443</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="102"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="105"/>
     </row>
     <row r="2" spans="1:6" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="22" t="s">
@@ -6295,14 +6295,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="146" t="s">
+      <c r="A18" s="143" t="s">
         <v>481</v>
       </c>
-      <c r="B18" s="108"/>
-      <c r="C18" s="108"/>
-      <c r="D18" s="108"/>
-      <c r="E18" s="108"/>
-      <c r="F18" s="108"/>
+      <c r="B18" s="101"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
     </row>
     <row r="19" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="88" t="s">
@@ -6343,56 +6343,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="150" t="s">
         <v>388</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="101"/>
-      <c r="T1" s="102"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
+      <c r="O1" s="104"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
+      <c r="S1" s="104"/>
+      <c r="T1" s="105"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="138"/>
-      <c r="B2" s="102"/>
-      <c r="C2" s="133" t="s">
+      <c r="A2" s="145"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="110" t="s">
         <v>389</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="102"/>
-      <c r="F2" s="136" t="s">
+      <c r="D2" s="104"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="113" t="s">
         <v>390</v>
       </c>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="145" t="s">
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="103" t="s">
         <v>391</v>
       </c>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="130" t="s">
+      <c r="L2" s="104"/>
+      <c r="M2" s="104"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="108" t="s">
         <v>392</v>
       </c>
-      <c r="P2" s="101"/>
-      <c r="Q2" s="101"/>
-      <c r="R2" s="102"/>
+      <c r="P2" s="104"/>
+      <c r="Q2" s="104"/>
+      <c r="R2" s="105"/>
       <c r="S2" s="52"/>
       <c r="T2" s="52"/>
     </row>
@@ -6459,10 +6459,10 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="141" t="s">
+      <c r="A4" s="148" t="s">
         <v>408</v>
       </c>
-      <c r="B4" s="102"/>
+      <c r="B4" s="105"/>
       <c r="C4" s="56" t="s">
         <v>409</v>
       </c>
@@ -6507,28 +6507,28 @@
       <c r="T4" s="68"/>
     </row>
     <row r="5" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="142" t="s">
+      <c r="A5" s="149" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
-      <c r="L5" s="108"/>
-      <c r="M5" s="108"/>
-      <c r="N5" s="108"/>
-      <c r="O5" s="108"/>
-      <c r="P5" s="108"/>
-      <c r="Q5" s="108"/>
-      <c r="R5" s="108"/>
-      <c r="S5" s="108"/>
-      <c r="T5" s="108"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101"/>
+      <c r="F5" s="101"/>
+      <c r="G5" s="101"/>
+      <c r="H5" s="101"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="101"/>
+      <c r="L5" s="101"/>
+      <c r="M5" s="101"/>
+      <c r="N5" s="101"/>
+      <c r="O5" s="101"/>
+      <c r="P5" s="101"/>
+      <c r="Q5" s="101"/>
+      <c r="R5" s="101"/>
+      <c r="S5" s="101"/>
+      <c r="T5" s="101"/>
     </row>
     <row r="6" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="69" t="s">
@@ -6537,14 +6537,14 @@
       <c r="B6" s="70" t="s">
         <v>157</v>
       </c>
-      <c r="C6" s="127" t="s">
+      <c r="C6" s="151" t="s">
         <v>156</v>
       </c>
-      <c r="D6" s="108"/>
-      <c r="E6" s="134" t="s">
+      <c r="D6" s="101"/>
+      <c r="E6" s="146" t="s">
         <v>163</v>
       </c>
-      <c r="F6" s="108"/>
+      <c r="F6" s="101"/>
       <c r="G6" s="71"/>
       <c r="H6" s="71"/>
       <c r="I6" s="71"/>
@@ -6616,15 +6616,15 @@
       <c r="I8" s="73"/>
       <c r="J8" s="74"/>
       <c r="K8" s="74"/>
-      <c r="L8" s="139" t="s">
+      <c r="L8" s="147" t="s">
         <v>411</v>
       </c>
-      <c r="M8" s="108"/>
-      <c r="N8" s="108"/>
-      <c r="O8" s="108"/>
-      <c r="P8" s="108"/>
-      <c r="Q8" s="108"/>
-      <c r="R8" s="108"/>
+      <c r="M8" s="101"/>
+      <c r="N8" s="101"/>
+      <c r="O8" s="101"/>
+      <c r="P8" s="101"/>
+      <c r="Q8" s="101"/>
+      <c r="R8" s="101"/>
       <c r="S8" s="75" t="s">
         <v>353</v>
       </c>
@@ -6649,14 +6649,14 @@
       <c r="J9" s="73"/>
       <c r="K9" s="73"/>
       <c r="L9" s="73"/>
-      <c r="M9" s="139" t="s">
+      <c r="M9" s="147" t="s">
         <v>411</v>
       </c>
-      <c r="N9" s="108"/>
-      <c r="O9" s="108"/>
-      <c r="P9" s="108"/>
-      <c r="Q9" s="108"/>
-      <c r="R9" s="108"/>
+      <c r="N9" s="101"/>
+      <c r="O9" s="101"/>
+      <c r="P9" s="101"/>
+      <c r="Q9" s="101"/>
+      <c r="R9" s="101"/>
       <c r="S9" s="75" t="s">
         <v>418</v>
       </c>
@@ -6671,14 +6671,14 @@
       <c r="B10" s="70" t="s">
         <v>246</v>
       </c>
-      <c r="C10" s="127" t="s">
+      <c r="C10" s="151" t="s">
         <v>156</v>
       </c>
-      <c r="D10" s="108"/>
-      <c r="E10" s="134" t="s">
+      <c r="D10" s="101"/>
+      <c r="E10" s="146" t="s">
         <v>163</v>
       </c>
-      <c r="F10" s="108"/>
+      <c r="F10" s="101"/>
       <c r="G10" s="71"/>
       <c r="H10" s="71"/>
       <c r="I10" s="71"/>
@@ -6844,15 +6844,15 @@
       <c r="I15" s="74"/>
       <c r="J15" s="74"/>
       <c r="K15" s="74"/>
-      <c r="L15" s="139" t="s">
+      <c r="L15" s="147" t="s">
         <v>411</v>
       </c>
-      <c r="M15" s="108"/>
-      <c r="N15" s="108"/>
-      <c r="O15" s="108"/>
-      <c r="P15" s="108"/>
-      <c r="Q15" s="108"/>
-      <c r="R15" s="108"/>
+      <c r="M15" s="101"/>
+      <c r="N15" s="101"/>
+      <c r="O15" s="101"/>
+      <c r="P15" s="101"/>
+      <c r="Q15" s="101"/>
+      <c r="R15" s="101"/>
       <c r="S15" s="75" t="s">
         <v>425</v>
       </c>
@@ -6942,15 +6942,15 @@
       <c r="I18" s="74"/>
       <c r="J18" s="74"/>
       <c r="K18" s="74"/>
-      <c r="L18" s="139" t="s">
+      <c r="L18" s="147" t="s">
         <v>411</v>
       </c>
-      <c r="M18" s="108"/>
-      <c r="N18" s="108"/>
-      <c r="O18" s="108"/>
-      <c r="P18" s="108"/>
-      <c r="Q18" s="108"/>
-      <c r="R18" s="108"/>
+      <c r="M18" s="101"/>
+      <c r="N18" s="101"/>
+      <c r="O18" s="101"/>
+      <c r="P18" s="101"/>
+      <c r="Q18" s="101"/>
+      <c r="R18" s="101"/>
       <c r="S18" s="75" t="s">
         <v>353</v>
       </c>
@@ -6975,16 +6975,16 @@
       <c r="H19" s="74"/>
       <c r="I19" s="74"/>
       <c r="J19" s="74"/>
-      <c r="K19" s="139" t="s">
+      <c r="K19" s="147" t="s">
         <v>411</v>
       </c>
-      <c r="L19" s="108"/>
-      <c r="M19" s="108"/>
-      <c r="N19" s="108"/>
-      <c r="O19" s="108"/>
-      <c r="P19" s="108"/>
-      <c r="Q19" s="108"/>
-      <c r="R19" s="108"/>
+      <c r="L19" s="101"/>
+      <c r="M19" s="101"/>
+      <c r="N19" s="101"/>
+      <c r="O19" s="101"/>
+      <c r="P19" s="101"/>
+      <c r="Q19" s="101"/>
+      <c r="R19" s="101"/>
       <c r="S19" s="75" t="s">
         <v>420</v>
       </c>
@@ -7042,10 +7042,10 @@
       <c r="E21" s="73"/>
       <c r="F21" s="73"/>
       <c r="G21" s="73"/>
-      <c r="H21" s="127" t="s">
+      <c r="H21" s="151" t="s">
         <v>156</v>
       </c>
-      <c r="I21" s="108"/>
+      <c r="I21" s="101"/>
       <c r="J21" s="67" t="s">
         <v>416</v>
       </c>
@@ -7117,14 +7117,14 @@
       <c r="J23" s="74"/>
       <c r="K23" s="74"/>
       <c r="L23" s="74"/>
-      <c r="M23" s="139" t="s">
+      <c r="M23" s="147" t="s">
         <v>411</v>
       </c>
-      <c r="N23" s="108"/>
-      <c r="O23" s="108"/>
-      <c r="P23" s="108"/>
-      <c r="Q23" s="108"/>
-      <c r="R23" s="108"/>
+      <c r="N23" s="101"/>
+      <c r="O23" s="101"/>
+      <c r="P23" s="101"/>
+      <c r="Q23" s="101"/>
+      <c r="R23" s="101"/>
       <c r="S23" s="75" t="s">
         <v>428</v>
       </c>
@@ -7133,28 +7133,28 @@
       </c>
     </row>
     <row r="25" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="135" t="s">
+      <c r="A25" s="102" t="s">
         <v>360</v>
       </c>
-      <c r="B25" s="108"/>
-      <c r="C25" s="108"/>
-      <c r="D25" s="108"/>
-      <c r="E25" s="108"/>
-      <c r="F25" s="108"/>
-      <c r="G25" s="108"/>
-      <c r="H25" s="108"/>
-      <c r="I25" s="108"/>
-      <c r="J25" s="108"/>
-      <c r="K25" s="108"/>
-      <c r="L25" s="108"/>
-      <c r="M25" s="108"/>
-      <c r="N25" s="108"/>
-      <c r="O25" s="108"/>
-      <c r="P25" s="108"/>
-      <c r="Q25" s="108"/>
-      <c r="R25" s="108"/>
-      <c r="S25" s="108"/>
-      <c r="T25" s="108"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="101"/>
+      <c r="E25" s="101"/>
+      <c r="F25" s="101"/>
+      <c r="G25" s="101"/>
+      <c r="H25" s="101"/>
+      <c r="I25" s="101"/>
+      <c r="J25" s="101"/>
+      <c r="K25" s="101"/>
+      <c r="L25" s="101"/>
+      <c r="M25" s="101"/>
+      <c r="N25" s="101"/>
+      <c r="O25" s="101"/>
+      <c r="P25" s="101"/>
+      <c r="Q25" s="101"/>
+      <c r="R25" s="101"/>
+      <c r="S25" s="101"/>
+      <c r="T25" s="101"/>
     </row>
     <row r="26" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="77" t="s">
@@ -7163,26 +7163,26 @@
       <c r="B26" s="78" t="s">
         <v>220</v>
       </c>
-      <c r="C26" s="126" t="s">
+      <c r="C26" s="116" t="s">
         <v>429</v>
       </c>
-      <c r="D26" s="108"/>
-      <c r="E26" s="108"/>
-      <c r="F26" s="108"/>
-      <c r="G26" s="108"/>
-      <c r="H26" s="108"/>
-      <c r="I26" s="108"/>
-      <c r="J26" s="108"/>
-      <c r="K26" s="108"/>
-      <c r="L26" s="108"/>
-      <c r="M26" s="108"/>
-      <c r="N26" s="108"/>
-      <c r="O26" s="108"/>
-      <c r="P26" s="108"/>
-      <c r="Q26" s="108"/>
-      <c r="R26" s="108"/>
-      <c r="S26" s="108"/>
-      <c r="T26" s="108"/>
+      <c r="D26" s="101"/>
+      <c r="E26" s="101"/>
+      <c r="F26" s="101"/>
+      <c r="G26" s="101"/>
+      <c r="H26" s="101"/>
+      <c r="I26" s="101"/>
+      <c r="J26" s="101"/>
+      <c r="K26" s="101"/>
+      <c r="L26" s="101"/>
+      <c r="M26" s="101"/>
+      <c r="N26" s="101"/>
+      <c r="O26" s="101"/>
+      <c r="P26" s="101"/>
+      <c r="Q26" s="101"/>
+      <c r="R26" s="101"/>
+      <c r="S26" s="101"/>
+      <c r="T26" s="101"/>
     </row>
     <row r="27" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="77" t="s">
@@ -7191,26 +7191,26 @@
       <c r="B27" s="78" t="s">
         <v>312</v>
       </c>
-      <c r="C27" s="126" t="s">
+      <c r="C27" s="116" t="s">
         <v>430</v>
       </c>
-      <c r="D27" s="108"/>
-      <c r="E27" s="108"/>
-      <c r="F27" s="108"/>
-      <c r="G27" s="108"/>
-      <c r="H27" s="108"/>
-      <c r="I27" s="108"/>
-      <c r="J27" s="108"/>
-      <c r="K27" s="108"/>
-      <c r="L27" s="108"/>
-      <c r="M27" s="108"/>
-      <c r="N27" s="108"/>
-      <c r="O27" s="108"/>
-      <c r="P27" s="108"/>
-      <c r="Q27" s="108"/>
-      <c r="R27" s="108"/>
-      <c r="S27" s="108"/>
-      <c r="T27" s="108"/>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="101"/>
+      <c r="K27" s="101"/>
+      <c r="L27" s="101"/>
+      <c r="M27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="101"/>
+      <c r="P27" s="101"/>
+      <c r="Q27" s="101"/>
+      <c r="R27" s="101"/>
+      <c r="S27" s="101"/>
+      <c r="T27" s="101"/>
     </row>
     <row r="28" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="77" t="s">
@@ -7219,26 +7219,26 @@
       <c r="B28" s="78" t="s">
         <v>312</v>
       </c>
-      <c r="C28" s="126" t="s">
+      <c r="C28" s="116" t="s">
         <v>430</v>
       </c>
-      <c r="D28" s="108"/>
-      <c r="E28" s="108"/>
-      <c r="F28" s="108"/>
-      <c r="G28" s="108"/>
-      <c r="H28" s="108"/>
-      <c r="I28" s="108"/>
-      <c r="J28" s="108"/>
-      <c r="K28" s="108"/>
-      <c r="L28" s="108"/>
-      <c r="M28" s="108"/>
-      <c r="N28" s="108"/>
-      <c r="O28" s="108"/>
-      <c r="P28" s="108"/>
-      <c r="Q28" s="108"/>
-      <c r="R28" s="108"/>
-      <c r="S28" s="108"/>
-      <c r="T28" s="108"/>
+      <c r="D28" s="101"/>
+      <c r="E28" s="101"/>
+      <c r="F28" s="101"/>
+      <c r="G28" s="101"/>
+      <c r="H28" s="101"/>
+      <c r="I28" s="101"/>
+      <c r="J28" s="101"/>
+      <c r="K28" s="101"/>
+      <c r="L28" s="101"/>
+      <c r="M28" s="101"/>
+      <c r="N28" s="101"/>
+      <c r="O28" s="101"/>
+      <c r="P28" s="101"/>
+      <c r="Q28" s="101"/>
+      <c r="R28" s="101"/>
+      <c r="S28" s="101"/>
+      <c r="T28" s="101"/>
     </row>
     <row r="29" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="77" t="s">
@@ -7247,50 +7247,50 @@
       <c r="B29" s="78" t="s">
         <v>351</v>
       </c>
-      <c r="C29" s="126" t="s">
+      <c r="C29" s="116" t="s">
         <v>371</v>
       </c>
-      <c r="D29" s="108"/>
-      <c r="E29" s="108"/>
-      <c r="F29" s="108"/>
-      <c r="G29" s="108"/>
-      <c r="H29" s="108"/>
-      <c r="I29" s="108"/>
-      <c r="J29" s="108"/>
-      <c r="K29" s="108"/>
-      <c r="L29" s="108"/>
-      <c r="M29" s="108"/>
-      <c r="N29" s="108"/>
-      <c r="O29" s="108"/>
-      <c r="P29" s="108"/>
-      <c r="Q29" s="108"/>
-      <c r="R29" s="108"/>
-      <c r="S29" s="108"/>
-      <c r="T29" s="108"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
+      <c r="G29" s="101"/>
+      <c r="H29" s="101"/>
+      <c r="I29" s="101"/>
+      <c r="J29" s="101"/>
+      <c r="K29" s="101"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="101"/>
+      <c r="N29" s="101"/>
+      <c r="O29" s="101"/>
+      <c r="P29" s="101"/>
+      <c r="Q29" s="101"/>
+      <c r="R29" s="101"/>
+      <c r="S29" s="101"/>
+      <c r="T29" s="101"/>
     </row>
     <row r="31" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="128" t="s">
+      <c r="A31" s="112" t="s">
         <v>431</v>
       </c>
-      <c r="B31" s="108"/>
-      <c r="C31" s="108"/>
-      <c r="D31" s="108"/>
-      <c r="E31" s="108"/>
-      <c r="F31" s="108"/>
-      <c r="G31" s="108"/>
-      <c r="H31" s="108"/>
-      <c r="I31" s="108"/>
-      <c r="J31" s="108"/>
-      <c r="K31" s="108"/>
-      <c r="L31" s="108"/>
-      <c r="M31" s="108"/>
-      <c r="N31" s="108"/>
-      <c r="O31" s="108"/>
-      <c r="P31" s="108"/>
-      <c r="Q31" s="108"/>
-      <c r="R31" s="108"/>
-      <c r="S31" s="108"/>
-      <c r="T31" s="108"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="101"/>
+      <c r="E31" s="101"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="101"/>
+      <c r="H31" s="101"/>
+      <c r="I31" s="101"/>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="101"/>
+      <c r="O31" s="101"/>
+      <c r="P31" s="101"/>
+      <c r="Q31" s="101"/>
+      <c r="R31" s="101"/>
+      <c r="S31" s="101"/>
+      <c r="T31" s="101"/>
     </row>
     <row r="32" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="79" t="s">
@@ -7335,151 +7335,166 @@
       <c r="T32" s="83"/>
     </row>
     <row r="33" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="140" t="s">
+      <c r="A33" s="114" t="s">
         <v>437</v>
       </c>
-      <c r="B33" s="108"/>
-      <c r="C33" s="108"/>
-      <c r="D33" s="108"/>
-      <c r="E33" s="108"/>
-      <c r="F33" s="108"/>
-      <c r="G33" s="108"/>
-      <c r="H33" s="108"/>
-      <c r="I33" s="108"/>
-      <c r="J33" s="108"/>
-      <c r="K33" s="108"/>
-      <c r="L33" s="108"/>
-      <c r="M33" s="108"/>
-      <c r="N33" s="108"/>
-      <c r="O33" s="108"/>
-      <c r="P33" s="108"/>
-      <c r="Q33" s="108"/>
-      <c r="R33" s="108"/>
-      <c r="S33" s="108"/>
-      <c r="T33" s="108"/>
+      <c r="B33" s="101"/>
+      <c r="C33" s="101"/>
+      <c r="D33" s="101"/>
+      <c r="E33" s="101"/>
+      <c r="F33" s="101"/>
+      <c r="G33" s="101"/>
+      <c r="H33" s="101"/>
+      <c r="I33" s="101"/>
+      <c r="J33" s="101"/>
+      <c r="K33" s="101"/>
+      <c r="L33" s="101"/>
+      <c r="M33" s="101"/>
+      <c r="N33" s="101"/>
+      <c r="O33" s="101"/>
+      <c r="P33" s="101"/>
+      <c r="Q33" s="101"/>
+      <c r="R33" s="101"/>
+      <c r="S33" s="101"/>
+      <c r="T33" s="101"/>
     </row>
     <row r="34" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="129" t="s">
+      <c r="A34" s="152" t="s">
         <v>438</v>
       </c>
-      <c r="B34" s="108"/>
-      <c r="C34" s="108"/>
-      <c r="D34" s="108"/>
-      <c r="E34" s="108"/>
-      <c r="F34" s="108"/>
-      <c r="G34" s="108"/>
-      <c r="H34" s="108"/>
-      <c r="I34" s="108"/>
-      <c r="J34" s="108"/>
-      <c r="K34" s="108"/>
-      <c r="L34" s="108"/>
-      <c r="M34" s="108"/>
-      <c r="N34" s="108"/>
-      <c r="O34" s="108"/>
-      <c r="P34" s="108"/>
-      <c r="Q34" s="108"/>
-      <c r="R34" s="108"/>
-      <c r="S34" s="108"/>
-      <c r="T34" s="108"/>
+      <c r="B34" s="101"/>
+      <c r="C34" s="101"/>
+      <c r="D34" s="101"/>
+      <c r="E34" s="101"/>
+      <c r="F34" s="101"/>
+      <c r="G34" s="101"/>
+      <c r="H34" s="101"/>
+      <c r="I34" s="101"/>
+      <c r="J34" s="101"/>
+      <c r="K34" s="101"/>
+      <c r="L34" s="101"/>
+      <c r="M34" s="101"/>
+      <c r="N34" s="101"/>
+      <c r="O34" s="101"/>
+      <c r="P34" s="101"/>
+      <c r="Q34" s="101"/>
+      <c r="R34" s="101"/>
+      <c r="S34" s="101"/>
+      <c r="T34" s="101"/>
     </row>
     <row r="35" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="143" t="s">
+      <c r="A35" s="117" t="s">
         <v>439</v>
       </c>
-      <c r="B35" s="108"/>
-      <c r="C35" s="108"/>
-      <c r="D35" s="108"/>
-      <c r="E35" s="108"/>
-      <c r="F35" s="108"/>
-      <c r="G35" s="108"/>
-      <c r="H35" s="108"/>
-      <c r="I35" s="108"/>
-      <c r="J35" s="108"/>
-      <c r="K35" s="108"/>
-      <c r="L35" s="108"/>
-      <c r="M35" s="108"/>
-      <c r="N35" s="108"/>
-      <c r="O35" s="108"/>
-      <c r="P35" s="108"/>
-      <c r="Q35" s="108"/>
-      <c r="R35" s="108"/>
-      <c r="S35" s="108"/>
-      <c r="T35" s="108"/>
+      <c r="B35" s="101"/>
+      <c r="C35" s="101"/>
+      <c r="D35" s="101"/>
+      <c r="E35" s="101"/>
+      <c r="F35" s="101"/>
+      <c r="G35" s="101"/>
+      <c r="H35" s="101"/>
+      <c r="I35" s="101"/>
+      <c r="J35" s="101"/>
+      <c r="K35" s="101"/>
+      <c r="L35" s="101"/>
+      <c r="M35" s="101"/>
+      <c r="N35" s="101"/>
+      <c r="O35" s="101"/>
+      <c r="P35" s="101"/>
+      <c r="Q35" s="101"/>
+      <c r="R35" s="101"/>
+      <c r="S35" s="101"/>
+      <c r="T35" s="101"/>
     </row>
     <row r="36" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="131" t="s">
+      <c r="A36" s="100" t="s">
         <v>440</v>
       </c>
-      <c r="B36" s="108"/>
-      <c r="C36" s="108"/>
-      <c r="D36" s="108"/>
-      <c r="E36" s="108"/>
-      <c r="F36" s="108"/>
-      <c r="G36" s="108"/>
-      <c r="H36" s="108"/>
-      <c r="I36" s="108"/>
-      <c r="J36" s="108"/>
-      <c r="K36" s="108"/>
-      <c r="L36" s="108"/>
-      <c r="M36" s="108"/>
-      <c r="N36" s="108"/>
-      <c r="O36" s="108"/>
-      <c r="P36" s="108"/>
-      <c r="Q36" s="108"/>
-      <c r="R36" s="108"/>
-      <c r="S36" s="108"/>
-      <c r="T36" s="108"/>
+      <c r="B36" s="101"/>
+      <c r="C36" s="101"/>
+      <c r="D36" s="101"/>
+      <c r="E36" s="101"/>
+      <c r="F36" s="101"/>
+      <c r="G36" s="101"/>
+      <c r="H36" s="101"/>
+      <c r="I36" s="101"/>
+      <c r="J36" s="101"/>
+      <c r="K36" s="101"/>
+      <c r="L36" s="101"/>
+      <c r="M36" s="101"/>
+      <c r="N36" s="101"/>
+      <c r="O36" s="101"/>
+      <c r="P36" s="101"/>
+      <c r="Q36" s="101"/>
+      <c r="R36" s="101"/>
+      <c r="S36" s="101"/>
+      <c r="T36" s="101"/>
     </row>
     <row r="37" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="137" t="s">
+      <c r="A37" s="107" t="s">
         <v>441</v>
       </c>
-      <c r="B37" s="108"/>
-      <c r="C37" s="108"/>
-      <c r="D37" s="108"/>
-      <c r="E37" s="108"/>
-      <c r="F37" s="108"/>
-      <c r="G37" s="108"/>
-      <c r="H37" s="108"/>
-      <c r="I37" s="108"/>
-      <c r="J37" s="108"/>
-      <c r="K37" s="108"/>
-      <c r="L37" s="108"/>
-      <c r="M37" s="108"/>
-      <c r="N37" s="108"/>
-      <c r="O37" s="108"/>
-      <c r="P37" s="108"/>
-      <c r="Q37" s="108"/>
-      <c r="R37" s="108"/>
-      <c r="S37" s="108"/>
-      <c r="T37" s="108"/>
+      <c r="B37" s="101"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="101"/>
+      <c r="E37" s="101"/>
+      <c r="F37" s="101"/>
+      <c r="G37" s="101"/>
+      <c r="H37" s="101"/>
+      <c r="I37" s="101"/>
+      <c r="J37" s="101"/>
+      <c r="K37" s="101"/>
+      <c r="L37" s="101"/>
+      <c r="M37" s="101"/>
+      <c r="N37" s="101"/>
+      <c r="O37" s="101"/>
+      <c r="P37" s="101"/>
+      <c r="Q37" s="101"/>
+      <c r="R37" s="101"/>
+      <c r="S37" s="101"/>
+      <c r="T37" s="101"/>
     </row>
     <row r="38" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="144" t="s">
         <v>442</v>
       </c>
-      <c r="B38" s="108"/>
-      <c r="C38" s="108"/>
-      <c r="D38" s="108"/>
-      <c r="E38" s="108"/>
-      <c r="F38" s="108"/>
-      <c r="G38" s="108"/>
-      <c r="H38" s="108"/>
-      <c r="I38" s="108"/>
-      <c r="J38" s="108"/>
-      <c r="K38" s="108"/>
-      <c r="L38" s="108"/>
-      <c r="M38" s="108"/>
-      <c r="N38" s="108"/>
-      <c r="O38" s="108"/>
-      <c r="P38" s="108"/>
-      <c r="Q38" s="108"/>
-      <c r="R38" s="108"/>
-      <c r="S38" s="108"/>
-      <c r="T38" s="108"/>
+      <c r="B38" s="101"/>
+      <c r="C38" s="101"/>
+      <c r="D38" s="101"/>
+      <c r="E38" s="101"/>
+      <c r="F38" s="101"/>
+      <c r="G38" s="101"/>
+      <c r="H38" s="101"/>
+      <c r="I38" s="101"/>
+      <c r="J38" s="101"/>
+      <c r="K38" s="101"/>
+      <c r="L38" s="101"/>
+      <c r="M38" s="101"/>
+      <c r="N38" s="101"/>
+      <c r="O38" s="101"/>
+      <c r="P38" s="101"/>
+      <c r="Q38" s="101"/>
+      <c r="R38" s="101"/>
+      <c r="S38" s="101"/>
+      <c r="T38" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="O2:R2"/>
+    <mergeCell ref="A36:T36"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="C27:T27"/>
+    <mergeCell ref="A25:T25"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="C26:T26"/>
+    <mergeCell ref="C29:T29"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A31:T31"/>
+    <mergeCell ref="A34:T34"/>
     <mergeCell ref="A38:T38"/>
     <mergeCell ref="K2:N2"/>
     <mergeCell ref="A37:T37"/>
@@ -7496,21 +7511,6 @@
     <mergeCell ref="M9:R9"/>
     <mergeCell ref="A35:T35"/>
     <mergeCell ref="K19:R19"/>
-    <mergeCell ref="O2:R2"/>
-    <mergeCell ref="A36:T36"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="C27:T27"/>
-    <mergeCell ref="A25:T25"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="C26:T26"/>
-    <mergeCell ref="C29:T29"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A31:T31"/>
-    <mergeCell ref="A34:T34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7529,56 +7529,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="147" t="s">
+      <c r="A1" s="154" t="s">
         <v>486</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="101"/>
-      <c r="T1" s="102"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
+      <c r="O1" s="104"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
+      <c r="S1" s="104"/>
+      <c r="T1" s="105"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="149"/>
-      <c r="B2" s="102"/>
-      <c r="C2" s="133" t="s">
+      <c r="A2" s="115"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="110" t="s">
         <v>389</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="102"/>
-      <c r="F2" s="136" t="s">
+      <c r="D2" s="104"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="113" t="s">
         <v>390</v>
       </c>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="145" t="s">
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="103" t="s">
         <v>391</v>
       </c>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="130" t="s">
+      <c r="L2" s="104"/>
+      <c r="M2" s="104"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="108" t="s">
         <v>392</v>
       </c>
-      <c r="P2" s="101"/>
-      <c r="Q2" s="101"/>
-      <c r="R2" s="102"/>
+      <c r="P2" s="104"/>
+      <c r="Q2" s="104"/>
+      <c r="R2" s="105"/>
       <c r="S2" s="52"/>
       <c r="T2" s="52"/>
     </row>
@@ -7645,32 +7645,32 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="150"/>
-      <c r="B4" s="108"/>
+      <c r="A4" s="118"/>
+      <c r="B4" s="101"/>
     </row>
     <row r="5" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="151" t="s">
+      <c r="A5" s="156" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
-      <c r="L5" s="108"/>
-      <c r="M5" s="108"/>
-      <c r="N5" s="108"/>
-      <c r="O5" s="108"/>
-      <c r="P5" s="108"/>
-      <c r="Q5" s="108"/>
-      <c r="R5" s="108"/>
-      <c r="S5" s="108"/>
-      <c r="T5" s="108"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101"/>
+      <c r="F5" s="101"/>
+      <c r="G5" s="101"/>
+      <c r="H5" s="101"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="101"/>
+      <c r="L5" s="101"/>
+      <c r="M5" s="101"/>
+      <c r="N5" s="101"/>
+      <c r="O5" s="101"/>
+      <c r="P5" s="101"/>
+      <c r="Q5" s="101"/>
+      <c r="R5" s="101"/>
+      <c r="S5" s="101"/>
+      <c r="T5" s="101"/>
     </row>
     <row r="6" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="84" t="s">
@@ -7685,28 +7685,28 @@
       <c r="D6" s="62" t="s">
         <v>412</v>
       </c>
-      <c r="E6" s="148" t="s">
+      <c r="E6" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="F6" s="108"/>
+      <c r="F6" s="101"/>
       <c r="G6" s="67" t="s">
         <v>416</v>
       </c>
-      <c r="H6" s="148" t="s">
+      <c r="H6" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="I6" s="108"/>
+      <c r="I6" s="101"/>
       <c r="J6" s="74"/>
       <c r="K6" s="74"/>
       <c r="L6" s="74"/>
       <c r="M6" s="74"/>
-      <c r="N6" s="152" t="s">
+      <c r="N6" s="153" t="s">
         <v>410</v>
       </c>
-      <c r="O6" s="108"/>
-      <c r="P6" s="108"/>
-      <c r="Q6" s="108"/>
-      <c r="R6" s="108"/>
+      <c r="O6" s="101"/>
+      <c r="P6" s="101"/>
+      <c r="Q6" s="101"/>
+      <c r="R6" s="101"/>
       <c r="S6" s="75" t="s">
         <v>427</v>
       </c>
@@ -7730,10 +7730,10 @@
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
       <c r="I7" s="73"/>
-      <c r="J7" s="134" t="s">
+      <c r="J7" s="146" t="s">
         <v>163</v>
       </c>
-      <c r="K7" s="108"/>
+      <c r="K7" s="101"/>
       <c r="L7" s="63" t="s">
         <v>224</v>
       </c>
@@ -7837,12 +7837,12 @@
       <c r="L10" s="74"/>
       <c r="M10" s="74"/>
       <c r="N10" s="74"/>
-      <c r="O10" s="148" t="s">
+      <c r="O10" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="P10" s="108"/>
-      <c r="Q10" s="108"/>
-      <c r="R10" s="108"/>
+      <c r="P10" s="101"/>
+      <c r="Q10" s="101"/>
+      <c r="R10" s="101"/>
       <c r="S10" s="75" t="s">
         <v>420</v>
       </c>
@@ -8037,363 +8037,357 @@
       </c>
     </row>
     <row r="18" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="135" t="s">
+      <c r="A18" s="102" t="s">
         <v>490</v>
       </c>
-      <c r="B18" s="108"/>
-      <c r="C18" s="108"/>
-      <c r="D18" s="108"/>
-      <c r="E18" s="108"/>
-      <c r="F18" s="108"/>
-      <c r="G18" s="108"/>
-      <c r="H18" s="108"/>
-      <c r="I18" s="108"/>
-      <c r="J18" s="108"/>
-      <c r="K18" s="108"/>
-      <c r="L18" s="108"/>
-      <c r="M18" s="108"/>
-      <c r="N18" s="108"/>
-      <c r="O18" s="108"/>
-      <c r="P18" s="108"/>
-      <c r="Q18" s="108"/>
-      <c r="R18" s="108"/>
-      <c r="S18" s="108"/>
-      <c r="T18" s="108"/>
+      <c r="B18" s="101"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="101"/>
+      <c r="J18" s="101"/>
+      <c r="K18" s="101"/>
+      <c r="L18" s="101"/>
+      <c r="M18" s="101"/>
+      <c r="N18" s="101"/>
+      <c r="O18" s="101"/>
+      <c r="P18" s="101"/>
+      <c r="Q18" s="101"/>
+      <c r="R18" s="101"/>
+      <c r="S18" s="101"/>
+      <c r="T18" s="101"/>
     </row>
     <row r="19" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="77" t="s">
         <v>375</v>
       </c>
-      <c r="B19" s="126" t="s">
+      <c r="B19" s="116" t="s">
         <v>491</v>
       </c>
-      <c r="C19" s="108"/>
-      <c r="D19" s="108"/>
-      <c r="E19" s="108"/>
-      <c r="F19" s="108"/>
-      <c r="G19" s="108"/>
-      <c r="H19" s="108"/>
-      <c r="I19" s="108"/>
-      <c r="J19" s="108"/>
-      <c r="K19" s="108"/>
-      <c r="L19" s="108"/>
-      <c r="M19" s="108"/>
-      <c r="N19" s="108"/>
-      <c r="O19" s="108"/>
-      <c r="P19" s="108"/>
-      <c r="Q19" s="108"/>
-      <c r="R19" s="108"/>
-      <c r="S19" s="108"/>
-      <c r="T19" s="108"/>
+      <c r="C19" s="101"/>
+      <c r="D19" s="101"/>
+      <c r="E19" s="101"/>
+      <c r="F19" s="101"/>
+      <c r="G19" s="101"/>
+      <c r="H19" s="101"/>
+      <c r="I19" s="101"/>
+      <c r="J19" s="101"/>
+      <c r="K19" s="101"/>
+      <c r="L19" s="101"/>
+      <c r="M19" s="101"/>
+      <c r="N19" s="101"/>
+      <c r="O19" s="101"/>
+      <c r="P19" s="101"/>
+      <c r="Q19" s="101"/>
+      <c r="R19" s="101"/>
+      <c r="S19" s="101"/>
+      <c r="T19" s="101"/>
     </row>
     <row r="20" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="77" t="s">
         <v>377</v>
       </c>
-      <c r="B20" s="126" t="s">
+      <c r="B20" s="116" t="s">
         <v>378</v>
       </c>
-      <c r="C20" s="108"/>
-      <c r="D20" s="108"/>
-      <c r="E20" s="108"/>
-      <c r="F20" s="108"/>
-      <c r="G20" s="108"/>
-      <c r="H20" s="108"/>
-      <c r="I20" s="108"/>
-      <c r="J20" s="108"/>
-      <c r="K20" s="108"/>
-      <c r="L20" s="108"/>
-      <c r="M20" s="108"/>
-      <c r="N20" s="108"/>
-      <c r="O20" s="108"/>
-      <c r="P20" s="108"/>
-      <c r="Q20" s="108"/>
-      <c r="R20" s="108"/>
-      <c r="S20" s="108"/>
-      <c r="T20" s="108"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="101"/>
+      <c r="E20" s="101"/>
+      <c r="F20" s="101"/>
+      <c r="G20" s="101"/>
+      <c r="H20" s="101"/>
+      <c r="I20" s="101"/>
+      <c r="J20" s="101"/>
+      <c r="K20" s="101"/>
+      <c r="L20" s="101"/>
+      <c r="M20" s="101"/>
+      <c r="N20" s="101"/>
+      <c r="O20" s="101"/>
+      <c r="P20" s="101"/>
+      <c r="Q20" s="101"/>
+      <c r="R20" s="101"/>
+      <c r="S20" s="101"/>
+      <c r="T20" s="101"/>
     </row>
     <row r="21" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="77" t="s">
         <v>379</v>
       </c>
-      <c r="B21" s="126" t="s">
+      <c r="B21" s="116" t="s">
         <v>378</v>
       </c>
-      <c r="C21" s="108"/>
-      <c r="D21" s="108"/>
-      <c r="E21" s="108"/>
-      <c r="F21" s="108"/>
-      <c r="G21" s="108"/>
-      <c r="H21" s="108"/>
-      <c r="I21" s="108"/>
-      <c r="J21" s="108"/>
-      <c r="K21" s="108"/>
-      <c r="L21" s="108"/>
-      <c r="M21" s="108"/>
-      <c r="N21" s="108"/>
-      <c r="O21" s="108"/>
-      <c r="P21" s="108"/>
-      <c r="Q21" s="108"/>
-      <c r="R21" s="108"/>
-      <c r="S21" s="108"/>
-      <c r="T21" s="108"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
+      <c r="L21" s="101"/>
+      <c r="M21" s="101"/>
+      <c r="N21" s="101"/>
+      <c r="O21" s="101"/>
+      <c r="P21" s="101"/>
+      <c r="Q21" s="101"/>
+      <c r="R21" s="101"/>
+      <c r="S21" s="101"/>
+      <c r="T21" s="101"/>
     </row>
     <row r="22" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="77" t="s">
         <v>380</v>
       </c>
-      <c r="B22" s="126" t="s">
+      <c r="B22" s="116" t="s">
         <v>492</v>
       </c>
-      <c r="C22" s="108"/>
-      <c r="D22" s="108"/>
-      <c r="E22" s="108"/>
-      <c r="F22" s="108"/>
-      <c r="G22" s="108"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="108"/>
-      <c r="J22" s="108"/>
-      <c r="K22" s="108"/>
-      <c r="L22" s="108"/>
-      <c r="M22" s="108"/>
-      <c r="N22" s="108"/>
-      <c r="O22" s="108"/>
-      <c r="P22" s="108"/>
-      <c r="Q22" s="108"/>
-      <c r="R22" s="108"/>
-      <c r="S22" s="108"/>
-      <c r="T22" s="108"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="101"/>
+      <c r="F22" s="101"/>
+      <c r="G22" s="101"/>
+      <c r="H22" s="101"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="101"/>
+      <c r="L22" s="101"/>
+      <c r="M22" s="101"/>
+      <c r="N22" s="101"/>
+      <c r="O22" s="101"/>
+      <c r="P22" s="101"/>
+      <c r="Q22" s="101"/>
+      <c r="R22" s="101"/>
+      <c r="S22" s="101"/>
+      <c r="T22" s="101"/>
     </row>
     <row r="23" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="77" t="s">
         <v>382</v>
       </c>
-      <c r="B23" s="126" t="s">
+      <c r="B23" s="116" t="s">
         <v>493</v>
       </c>
-      <c r="C23" s="108"/>
-      <c r="D23" s="108"/>
-      <c r="E23" s="108"/>
-      <c r="F23" s="108"/>
-      <c r="G23" s="108"/>
-      <c r="H23" s="108"/>
-      <c r="I23" s="108"/>
-      <c r="J23" s="108"/>
-      <c r="K23" s="108"/>
-      <c r="L23" s="108"/>
-      <c r="M23" s="108"/>
-      <c r="N23" s="108"/>
-      <c r="O23" s="108"/>
-      <c r="P23" s="108"/>
-      <c r="Q23" s="108"/>
-      <c r="R23" s="108"/>
-      <c r="S23" s="108"/>
-      <c r="T23" s="108"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="101"/>
+      <c r="E23" s="101"/>
+      <c r="F23" s="101"/>
+      <c r="G23" s="101"/>
+      <c r="H23" s="101"/>
+      <c r="I23" s="101"/>
+      <c r="J23" s="101"/>
+      <c r="K23" s="101"/>
+      <c r="L23" s="101"/>
+      <c r="M23" s="101"/>
+      <c r="N23" s="101"/>
+      <c r="O23" s="101"/>
+      <c r="P23" s="101"/>
+      <c r="Q23" s="101"/>
+      <c r="R23" s="101"/>
+      <c r="S23" s="101"/>
+      <c r="T23" s="101"/>
     </row>
     <row r="24" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="77" t="s">
         <v>384</v>
       </c>
-      <c r="B24" s="126" t="s">
+      <c r="B24" s="116" t="s">
         <v>494</v>
       </c>
-      <c r="C24" s="108"/>
-      <c r="D24" s="108"/>
-      <c r="E24" s="108"/>
-      <c r="F24" s="108"/>
-      <c r="G24" s="108"/>
-      <c r="H24" s="108"/>
-      <c r="I24" s="108"/>
-      <c r="J24" s="108"/>
-      <c r="K24" s="108"/>
-      <c r="L24" s="108"/>
-      <c r="M24" s="108"/>
-      <c r="N24" s="108"/>
-      <c r="O24" s="108"/>
-      <c r="P24" s="108"/>
-      <c r="Q24" s="108"/>
-      <c r="R24" s="108"/>
-      <c r="S24" s="108"/>
-      <c r="T24" s="108"/>
+      <c r="C24" s="101"/>
+      <c r="D24" s="101"/>
+      <c r="E24" s="101"/>
+      <c r="F24" s="101"/>
+      <c r="G24" s="101"/>
+      <c r="H24" s="101"/>
+      <c r="I24" s="101"/>
+      <c r="J24" s="101"/>
+      <c r="K24" s="101"/>
+      <c r="L24" s="101"/>
+      <c r="M24" s="101"/>
+      <c r="N24" s="101"/>
+      <c r="O24" s="101"/>
+      <c r="P24" s="101"/>
+      <c r="Q24" s="101"/>
+      <c r="R24" s="101"/>
+      <c r="S24" s="101"/>
+      <c r="T24" s="101"/>
     </row>
     <row r="25" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="77" t="s">
         <v>386</v>
       </c>
-      <c r="B25" s="126" t="s">
+      <c r="B25" s="116" t="s">
         <v>494</v>
       </c>
-      <c r="C25" s="108"/>
-      <c r="D25" s="108"/>
-      <c r="E25" s="108"/>
-      <c r="F25" s="108"/>
-      <c r="G25" s="108"/>
-      <c r="H25" s="108"/>
-      <c r="I25" s="108"/>
-      <c r="J25" s="108"/>
-      <c r="K25" s="108"/>
-      <c r="L25" s="108"/>
-      <c r="M25" s="108"/>
-      <c r="N25" s="108"/>
-      <c r="O25" s="108"/>
-      <c r="P25" s="108"/>
-      <c r="Q25" s="108"/>
-      <c r="R25" s="108"/>
-      <c r="S25" s="108"/>
-      <c r="T25" s="108"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="101"/>
+      <c r="E25" s="101"/>
+      <c r="F25" s="101"/>
+      <c r="G25" s="101"/>
+      <c r="H25" s="101"/>
+      <c r="I25" s="101"/>
+      <c r="J25" s="101"/>
+      <c r="K25" s="101"/>
+      <c r="L25" s="101"/>
+      <c r="M25" s="101"/>
+      <c r="N25" s="101"/>
+      <c r="O25" s="101"/>
+      <c r="P25" s="101"/>
+      <c r="Q25" s="101"/>
+      <c r="R25" s="101"/>
+      <c r="S25" s="101"/>
+      <c r="T25" s="101"/>
     </row>
     <row r="27" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="128" t="s">
+      <c r="A27" s="112" t="s">
         <v>495</v>
       </c>
-      <c r="B27" s="108"/>
-      <c r="C27" s="108"/>
-      <c r="D27" s="108"/>
-      <c r="E27" s="108"/>
-      <c r="F27" s="108"/>
-      <c r="G27" s="108"/>
-      <c r="H27" s="108"/>
-      <c r="I27" s="108"/>
-      <c r="J27" s="108"/>
-      <c r="K27" s="108"/>
-      <c r="L27" s="108"/>
-      <c r="M27" s="108"/>
-      <c r="N27" s="108"/>
-      <c r="O27" s="108"/>
-      <c r="P27" s="108"/>
-      <c r="Q27" s="108"/>
-      <c r="R27" s="108"/>
-      <c r="S27" s="108"/>
-      <c r="T27" s="108"/>
+      <c r="B27" s="101"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="101"/>
+      <c r="K27" s="101"/>
+      <c r="L27" s="101"/>
+      <c r="M27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="101"/>
+      <c r="P27" s="101"/>
+      <c r="Q27" s="101"/>
+      <c r="R27" s="101"/>
+      <c r="S27" s="101"/>
+      <c r="T27" s="101"/>
     </row>
     <row r="28" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="129" t="s">
+      <c r="A28" s="152" t="s">
         <v>496</v>
       </c>
-      <c r="B28" s="108"/>
-      <c r="C28" s="108"/>
-      <c r="D28" s="108"/>
-      <c r="E28" s="108"/>
-      <c r="F28" s="108"/>
-      <c r="G28" s="108"/>
-      <c r="H28" s="108"/>
-      <c r="I28" s="108"/>
-      <c r="J28" s="108"/>
-      <c r="K28" s="108"/>
-      <c r="L28" s="108"/>
-      <c r="M28" s="108"/>
-      <c r="N28" s="108"/>
-      <c r="O28" s="108"/>
-      <c r="P28" s="108"/>
-      <c r="Q28" s="108"/>
-      <c r="R28" s="108"/>
-      <c r="S28" s="108"/>
-      <c r="T28" s="108"/>
+      <c r="B28" s="101"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="101"/>
+      <c r="E28" s="101"/>
+      <c r="F28" s="101"/>
+      <c r="G28" s="101"/>
+      <c r="H28" s="101"/>
+      <c r="I28" s="101"/>
+      <c r="J28" s="101"/>
+      <c r="K28" s="101"/>
+      <c r="L28" s="101"/>
+      <c r="M28" s="101"/>
+      <c r="N28" s="101"/>
+      <c r="O28" s="101"/>
+      <c r="P28" s="101"/>
+      <c r="Q28" s="101"/>
+      <c r="R28" s="101"/>
+      <c r="S28" s="101"/>
+      <c r="T28" s="101"/>
     </row>
     <row r="29" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="143" t="s">
+      <c r="A29" s="117" t="s">
         <v>497</v>
       </c>
-      <c r="B29" s="108"/>
-      <c r="C29" s="108"/>
-      <c r="D29" s="108"/>
-      <c r="E29" s="108"/>
-      <c r="F29" s="108"/>
-      <c r="G29" s="108"/>
-      <c r="H29" s="108"/>
-      <c r="I29" s="108"/>
-      <c r="J29" s="108"/>
-      <c r="K29" s="108"/>
-      <c r="L29" s="108"/>
-      <c r="M29" s="108"/>
-      <c r="N29" s="108"/>
-      <c r="O29" s="108"/>
-      <c r="P29" s="108"/>
-      <c r="Q29" s="108"/>
-      <c r="R29" s="108"/>
-      <c r="S29" s="108"/>
-      <c r="T29" s="108"/>
+      <c r="B29" s="101"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
+      <c r="G29" s="101"/>
+      <c r="H29" s="101"/>
+      <c r="I29" s="101"/>
+      <c r="J29" s="101"/>
+      <c r="K29" s="101"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="101"/>
+      <c r="N29" s="101"/>
+      <c r="O29" s="101"/>
+      <c r="P29" s="101"/>
+      <c r="Q29" s="101"/>
+      <c r="R29" s="101"/>
+      <c r="S29" s="101"/>
+      <c r="T29" s="101"/>
     </row>
     <row r="30" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="143" t="s">
+      <c r="A30" s="117" t="s">
         <v>498</v>
       </c>
-      <c r="B30" s="108"/>
-      <c r="C30" s="108"/>
-      <c r="D30" s="108"/>
-      <c r="E30" s="108"/>
-      <c r="F30" s="108"/>
-      <c r="G30" s="108"/>
-      <c r="H30" s="108"/>
-      <c r="I30" s="108"/>
-      <c r="J30" s="108"/>
-      <c r="K30" s="108"/>
-      <c r="L30" s="108"/>
-      <c r="M30" s="108"/>
-      <c r="N30" s="108"/>
-      <c r="O30" s="108"/>
-      <c r="P30" s="108"/>
-      <c r="Q30" s="108"/>
-      <c r="R30" s="108"/>
-      <c r="S30" s="108"/>
-      <c r="T30" s="108"/>
+      <c r="B30" s="101"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="101"/>
+      <c r="E30" s="101"/>
+      <c r="F30" s="101"/>
+      <c r="G30" s="101"/>
+      <c r="H30" s="101"/>
+      <c r="I30" s="101"/>
+      <c r="J30" s="101"/>
+      <c r="K30" s="101"/>
+      <c r="L30" s="101"/>
+      <c r="M30" s="101"/>
+      <c r="N30" s="101"/>
+      <c r="O30" s="101"/>
+      <c r="P30" s="101"/>
+      <c r="Q30" s="101"/>
+      <c r="R30" s="101"/>
+      <c r="S30" s="101"/>
+      <c r="T30" s="101"/>
     </row>
     <row r="31" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="131" t="s">
+      <c r="A31" s="100" t="s">
         <v>499</v>
       </c>
-      <c r="B31" s="108"/>
-      <c r="C31" s="108"/>
-      <c r="D31" s="108"/>
-      <c r="E31" s="108"/>
-      <c r="F31" s="108"/>
-      <c r="G31" s="108"/>
-      <c r="H31" s="108"/>
-      <c r="I31" s="108"/>
-      <c r="J31" s="108"/>
-      <c r="K31" s="108"/>
-      <c r="L31" s="108"/>
-      <c r="M31" s="108"/>
-      <c r="N31" s="108"/>
-      <c r="O31" s="108"/>
-      <c r="P31" s="108"/>
-      <c r="Q31" s="108"/>
-      <c r="R31" s="108"/>
-      <c r="S31" s="108"/>
-      <c r="T31" s="108"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="101"/>
+      <c r="E31" s="101"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="101"/>
+      <c r="H31" s="101"/>
+      <c r="I31" s="101"/>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="101"/>
+      <c r="O31" s="101"/>
+      <c r="P31" s="101"/>
+      <c r="Q31" s="101"/>
+      <c r="R31" s="101"/>
+      <c r="S31" s="101"/>
+      <c r="T31" s="101"/>
     </row>
     <row r="32" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="143" t="s">
+      <c r="A32" s="117" t="s">
         <v>500</v>
       </c>
-      <c r="B32" s="108"/>
-      <c r="C32" s="108"/>
-      <c r="D32" s="108"/>
-      <c r="E32" s="108"/>
-      <c r="F32" s="108"/>
-      <c r="G32" s="108"/>
-      <c r="H32" s="108"/>
-      <c r="I32" s="108"/>
-      <c r="J32" s="108"/>
-      <c r="K32" s="108"/>
-      <c r="L32" s="108"/>
-      <c r="M32" s="108"/>
-      <c r="N32" s="108"/>
-      <c r="O32" s="108"/>
-      <c r="P32" s="108"/>
-      <c r="Q32" s="108"/>
-      <c r="R32" s="108"/>
-      <c r="S32" s="108"/>
-      <c r="T32" s="108"/>
+      <c r="B32" s="101"/>
+      <c r="C32" s="101"/>
+      <c r="D32" s="101"/>
+      <c r="E32" s="101"/>
+      <c r="F32" s="101"/>
+      <c r="G32" s="101"/>
+      <c r="H32" s="101"/>
+      <c r="I32" s="101"/>
+      <c r="J32" s="101"/>
+      <c r="K32" s="101"/>
+      <c r="L32" s="101"/>
+      <c r="M32" s="101"/>
+      <c r="N32" s="101"/>
+      <c r="O32" s="101"/>
+      <c r="P32" s="101"/>
+      <c r="Q32" s="101"/>
+      <c r="R32" s="101"/>
+      <c r="S32" s="101"/>
+      <c r="T32" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A32:T32"/>
-    <mergeCell ref="B23:T23"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="A29:T29"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="A28:T28"/>
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="B20:T20"/>
@@ -8407,9 +8401,15 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:T5"/>
     <mergeCell ref="B19:T19"/>
+    <mergeCell ref="O2:R2"/>
+    <mergeCell ref="A32:T32"/>
+    <mergeCell ref="B23:T23"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="A29:T29"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="A28:T28"/>
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
-    <mergeCell ref="O2:R2"/>
     <mergeCell ref="B24:T24"/>
     <mergeCell ref="B25:T25"/>
     <mergeCell ref="A27:T27"/>
@@ -8433,56 +8433,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="109" t="s">
         <v>501</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="101"/>
-      <c r="T1" s="102"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
+      <c r="O1" s="104"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
+      <c r="S1" s="104"/>
+      <c r="T1" s="105"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="149"/>
-      <c r="B2" s="102"/>
-      <c r="C2" s="133" t="s">
+      <c r="A2" s="115"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="110" t="s">
         <v>389</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="102"/>
-      <c r="F2" s="136" t="s">
+      <c r="D2" s="104"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="113" t="s">
         <v>390</v>
       </c>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="145" t="s">
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="103" t="s">
         <v>391</v>
       </c>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="130" t="s">
+      <c r="L2" s="104"/>
+      <c r="M2" s="104"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="108" t="s">
         <v>392</v>
       </c>
-      <c r="P2" s="101"/>
-      <c r="Q2" s="101"/>
-      <c r="R2" s="102"/>
+      <c r="P2" s="104"/>
+      <c r="Q2" s="104"/>
+      <c r="R2" s="105"/>
       <c r="S2" s="52"/>
       <c r="T2" s="52"/>
     </row>
@@ -8549,56 +8549,56 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="150"/>
-      <c r="B4" s="108"/>
+      <c r="A4" s="118"/>
+      <c r="B4" s="101"/>
     </row>
     <row r="5" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="155" t="s">
+      <c r="A5" s="119" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
-      <c r="L5" s="108"/>
-      <c r="M5" s="108"/>
-      <c r="N5" s="108"/>
-      <c r="O5" s="108"/>
-      <c r="P5" s="108"/>
-      <c r="Q5" s="108"/>
-      <c r="R5" s="108"/>
-      <c r="S5" s="108"/>
-      <c r="T5" s="108"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101"/>
+      <c r="F5" s="101"/>
+      <c r="G5" s="101"/>
+      <c r="H5" s="101"/>
+      <c r="I5" s="101"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="101"/>
+      <c r="L5" s="101"/>
+      <c r="M5" s="101"/>
+      <c r="N5" s="101"/>
+      <c r="O5" s="101"/>
+      <c r="P5" s="101"/>
+      <c r="Q5" s="101"/>
+      <c r="R5" s="101"/>
+      <c r="S5" s="101"/>
+      <c r="T5" s="101"/>
     </row>
     <row r="6" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="154" t="s">
+      <c r="A6" s="111" t="s">
         <v>502</v>
       </c>
-      <c r="B6" s="108"/>
-      <c r="C6" s="108"/>
-      <c r="D6" s="108"/>
-      <c r="E6" s="108"/>
-      <c r="F6" s="108"/>
-      <c r="G6" s="108"/>
-      <c r="H6" s="108"/>
-      <c r="I6" s="108"/>
-      <c r="J6" s="108"/>
-      <c r="K6" s="108"/>
-      <c r="L6" s="108"/>
-      <c r="M6" s="108"/>
-      <c r="N6" s="108"/>
-      <c r="O6" s="108"/>
-      <c r="P6" s="108"/>
-      <c r="Q6" s="108"/>
-      <c r="R6" s="108"/>
-      <c r="S6" s="108"/>
-      <c r="T6" s="108"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="101"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="101"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="101"/>
+      <c r="K6" s="101"/>
+      <c r="L6" s="101"/>
+      <c r="M6" s="101"/>
+      <c r="N6" s="101"/>
+      <c r="O6" s="101"/>
+      <c r="P6" s="101"/>
+      <c r="Q6" s="101"/>
+      <c r="R6" s="101"/>
+      <c r="S6" s="101"/>
+      <c r="T6" s="101"/>
     </row>
     <row r="7" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="85" t="s">
@@ -8951,277 +8951,288 @@
       </c>
     </row>
     <row r="20" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="135" t="s">
+      <c r="A20" s="102" t="s">
         <v>490</v>
       </c>
-      <c r="B20" s="108"/>
-      <c r="C20" s="108"/>
-      <c r="D20" s="108"/>
-      <c r="E20" s="108"/>
-      <c r="F20" s="108"/>
-      <c r="G20" s="108"/>
-      <c r="H20" s="108"/>
-      <c r="I20" s="108"/>
-      <c r="J20" s="108"/>
-      <c r="K20" s="108"/>
-      <c r="L20" s="108"/>
-      <c r="M20" s="108"/>
-      <c r="N20" s="108"/>
-      <c r="O20" s="108"/>
-      <c r="P20" s="108"/>
-      <c r="Q20" s="108"/>
-      <c r="R20" s="108"/>
-      <c r="S20" s="108"/>
-      <c r="T20" s="108"/>
+      <c r="B20" s="101"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="101"/>
+      <c r="E20" s="101"/>
+      <c r="F20" s="101"/>
+      <c r="G20" s="101"/>
+      <c r="H20" s="101"/>
+      <c r="I20" s="101"/>
+      <c r="J20" s="101"/>
+      <c r="K20" s="101"/>
+      <c r="L20" s="101"/>
+      <c r="M20" s="101"/>
+      <c r="N20" s="101"/>
+      <c r="O20" s="101"/>
+      <c r="P20" s="101"/>
+      <c r="Q20" s="101"/>
+      <c r="R20" s="101"/>
+      <c r="S20" s="101"/>
+      <c r="T20" s="101"/>
     </row>
     <row r="21" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="77" t="s">
         <v>355</v>
       </c>
-      <c r="B21" s="126" t="s">
+      <c r="B21" s="116" t="s">
         <v>387</v>
       </c>
-      <c r="C21" s="108"/>
-      <c r="D21" s="108"/>
-      <c r="E21" s="108"/>
-      <c r="F21" s="108"/>
-      <c r="G21" s="108"/>
-      <c r="H21" s="108"/>
-      <c r="I21" s="108"/>
-      <c r="J21" s="108"/>
-      <c r="K21" s="108"/>
-      <c r="L21" s="108"/>
-      <c r="M21" s="108"/>
-      <c r="N21" s="108"/>
-      <c r="O21" s="108"/>
-      <c r="P21" s="108"/>
-      <c r="Q21" s="108"/>
-      <c r="R21" s="108"/>
-      <c r="S21" s="108"/>
-      <c r="T21" s="108"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
+      <c r="L21" s="101"/>
+      <c r="M21" s="101"/>
+      <c r="N21" s="101"/>
+      <c r="O21" s="101"/>
+      <c r="P21" s="101"/>
+      <c r="Q21" s="101"/>
+      <c r="R21" s="101"/>
+      <c r="S21" s="101"/>
+      <c r="T21" s="101"/>
     </row>
     <row r="22" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="77" t="s">
         <v>327</v>
       </c>
-      <c r="B22" s="126" t="s">
+      <c r="B22" s="116" t="s">
         <v>329</v>
       </c>
-      <c r="C22" s="108"/>
-      <c r="D22" s="108"/>
-      <c r="E22" s="108"/>
-      <c r="F22" s="108"/>
-      <c r="G22" s="108"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="108"/>
-      <c r="J22" s="108"/>
-      <c r="K22" s="108"/>
-      <c r="L22" s="108"/>
-      <c r="M22" s="108"/>
-      <c r="N22" s="108"/>
-      <c r="O22" s="108"/>
-      <c r="P22" s="108"/>
-      <c r="Q22" s="108"/>
-      <c r="R22" s="108"/>
-      <c r="S22" s="108"/>
-      <c r="T22" s="108"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="101"/>
+      <c r="F22" s="101"/>
+      <c r="G22" s="101"/>
+      <c r="H22" s="101"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="101"/>
+      <c r="L22" s="101"/>
+      <c r="M22" s="101"/>
+      <c r="N22" s="101"/>
+      <c r="O22" s="101"/>
+      <c r="P22" s="101"/>
+      <c r="Q22" s="101"/>
+      <c r="R22" s="101"/>
+      <c r="S22" s="101"/>
+      <c r="T22" s="101"/>
     </row>
     <row r="23" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="77" t="s">
         <v>372</v>
       </c>
-      <c r="B23" s="126" t="s">
+      <c r="B23" s="116" t="s">
         <v>512</v>
       </c>
-      <c r="C23" s="108"/>
-      <c r="D23" s="108"/>
-      <c r="E23" s="108"/>
-      <c r="F23" s="108"/>
-      <c r="G23" s="108"/>
-      <c r="H23" s="108"/>
-      <c r="I23" s="108"/>
-      <c r="J23" s="108"/>
-      <c r="K23" s="108"/>
-      <c r="L23" s="108"/>
-      <c r="M23" s="108"/>
-      <c r="N23" s="108"/>
-      <c r="O23" s="108"/>
-      <c r="P23" s="108"/>
-      <c r="Q23" s="108"/>
-      <c r="R23" s="108"/>
-      <c r="S23" s="108"/>
-      <c r="T23" s="108"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="101"/>
+      <c r="E23" s="101"/>
+      <c r="F23" s="101"/>
+      <c r="G23" s="101"/>
+      <c r="H23" s="101"/>
+      <c r="I23" s="101"/>
+      <c r="J23" s="101"/>
+      <c r="K23" s="101"/>
+      <c r="L23" s="101"/>
+      <c r="M23" s="101"/>
+      <c r="N23" s="101"/>
+      <c r="O23" s="101"/>
+      <c r="P23" s="101"/>
+      <c r="Q23" s="101"/>
+      <c r="R23" s="101"/>
+      <c r="S23" s="101"/>
+      <c r="T23" s="101"/>
     </row>
     <row r="25" spans="1:20" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="128" t="s">
+      <c r="A25" s="112" t="s">
         <v>495</v>
       </c>
-      <c r="B25" s="108"/>
-      <c r="C25" s="108"/>
-      <c r="D25" s="108"/>
-      <c r="E25" s="108"/>
-      <c r="F25" s="108"/>
-      <c r="G25" s="108"/>
-      <c r="H25" s="108"/>
-      <c r="I25" s="108"/>
-      <c r="J25" s="108"/>
-      <c r="K25" s="108"/>
-      <c r="L25" s="108"/>
-      <c r="M25" s="108"/>
-      <c r="N25" s="108"/>
-      <c r="O25" s="108"/>
-      <c r="P25" s="108"/>
-      <c r="Q25" s="108"/>
-      <c r="R25" s="108"/>
-      <c r="S25" s="108"/>
-      <c r="T25" s="108"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="101"/>
+      <c r="E25" s="101"/>
+      <c r="F25" s="101"/>
+      <c r="G25" s="101"/>
+      <c r="H25" s="101"/>
+      <c r="I25" s="101"/>
+      <c r="J25" s="101"/>
+      <c r="K25" s="101"/>
+      <c r="L25" s="101"/>
+      <c r="M25" s="101"/>
+      <c r="N25" s="101"/>
+      <c r="O25" s="101"/>
+      <c r="P25" s="101"/>
+      <c r="Q25" s="101"/>
+      <c r="R25" s="101"/>
+      <c r="S25" s="101"/>
+      <c r="T25" s="101"/>
     </row>
     <row r="26" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="143" t="s">
+      <c r="A26" s="117" t="s">
         <v>513</v>
       </c>
-      <c r="B26" s="108"/>
-      <c r="C26" s="108"/>
-      <c r="D26" s="108"/>
-      <c r="E26" s="108"/>
-      <c r="F26" s="108"/>
-      <c r="G26" s="108"/>
-      <c r="H26" s="108"/>
-      <c r="I26" s="108"/>
-      <c r="J26" s="108"/>
-      <c r="K26" s="108"/>
-      <c r="L26" s="108"/>
-      <c r="M26" s="108"/>
-      <c r="N26" s="108"/>
-      <c r="O26" s="108"/>
-      <c r="P26" s="108"/>
-      <c r="Q26" s="108"/>
-      <c r="R26" s="108"/>
-      <c r="S26" s="108"/>
-      <c r="T26" s="108"/>
+      <c r="B26" s="101"/>
+      <c r="C26" s="101"/>
+      <c r="D26" s="101"/>
+      <c r="E26" s="101"/>
+      <c r="F26" s="101"/>
+      <c r="G26" s="101"/>
+      <c r="H26" s="101"/>
+      <c r="I26" s="101"/>
+      <c r="J26" s="101"/>
+      <c r="K26" s="101"/>
+      <c r="L26" s="101"/>
+      <c r="M26" s="101"/>
+      <c r="N26" s="101"/>
+      <c r="O26" s="101"/>
+      <c r="P26" s="101"/>
+      <c r="Q26" s="101"/>
+      <c r="R26" s="101"/>
+      <c r="S26" s="101"/>
+      <c r="T26" s="101"/>
     </row>
     <row r="27" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="140" t="s">
+      <c r="A27" s="114" t="s">
         <v>514</v>
       </c>
-      <c r="B27" s="108"/>
-      <c r="C27" s="108"/>
-      <c r="D27" s="108"/>
-      <c r="E27" s="108"/>
-      <c r="F27" s="108"/>
-      <c r="G27" s="108"/>
-      <c r="H27" s="108"/>
-      <c r="I27" s="108"/>
-      <c r="J27" s="108"/>
-      <c r="K27" s="108"/>
-      <c r="L27" s="108"/>
-      <c r="M27" s="108"/>
-      <c r="N27" s="108"/>
-      <c r="O27" s="108"/>
-      <c r="P27" s="108"/>
-      <c r="Q27" s="108"/>
-      <c r="R27" s="108"/>
-      <c r="S27" s="108"/>
-      <c r="T27" s="108"/>
+      <c r="B27" s="101"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="101"/>
+      <c r="K27" s="101"/>
+      <c r="L27" s="101"/>
+      <c r="M27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="101"/>
+      <c r="P27" s="101"/>
+      <c r="Q27" s="101"/>
+      <c r="R27" s="101"/>
+      <c r="S27" s="101"/>
+      <c r="T27" s="101"/>
     </row>
     <row r="28" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="156" t="s">
+      <c r="A28" s="106" t="s">
         <v>515</v>
       </c>
-      <c r="B28" s="108"/>
-      <c r="C28" s="108"/>
-      <c r="D28" s="108"/>
-      <c r="E28" s="108"/>
-      <c r="F28" s="108"/>
-      <c r="G28" s="108"/>
-      <c r="H28" s="108"/>
-      <c r="I28" s="108"/>
-      <c r="J28" s="108"/>
-      <c r="K28" s="108"/>
-      <c r="L28" s="108"/>
-      <c r="M28" s="108"/>
-      <c r="N28" s="108"/>
-      <c r="O28" s="108"/>
-      <c r="P28" s="108"/>
-      <c r="Q28" s="108"/>
-      <c r="R28" s="108"/>
-      <c r="S28" s="108"/>
-      <c r="T28" s="108"/>
+      <c r="B28" s="101"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="101"/>
+      <c r="E28" s="101"/>
+      <c r="F28" s="101"/>
+      <c r="G28" s="101"/>
+      <c r="H28" s="101"/>
+      <c r="I28" s="101"/>
+      <c r="J28" s="101"/>
+      <c r="K28" s="101"/>
+      <c r="L28" s="101"/>
+      <c r="M28" s="101"/>
+      <c r="N28" s="101"/>
+      <c r="O28" s="101"/>
+      <c r="P28" s="101"/>
+      <c r="Q28" s="101"/>
+      <c r="R28" s="101"/>
+      <c r="S28" s="101"/>
+      <c r="T28" s="101"/>
     </row>
     <row r="29" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="131" t="s">
+      <c r="A29" s="100" t="s">
         <v>516</v>
       </c>
-      <c r="B29" s="108"/>
-      <c r="C29" s="108"/>
-      <c r="D29" s="108"/>
-      <c r="E29" s="108"/>
-      <c r="F29" s="108"/>
-      <c r="G29" s="108"/>
-      <c r="H29" s="108"/>
-      <c r="I29" s="108"/>
-      <c r="J29" s="108"/>
-      <c r="K29" s="108"/>
-      <c r="L29" s="108"/>
-      <c r="M29" s="108"/>
-      <c r="N29" s="108"/>
-      <c r="O29" s="108"/>
-      <c r="P29" s="108"/>
-      <c r="Q29" s="108"/>
-      <c r="R29" s="108"/>
-      <c r="S29" s="108"/>
-      <c r="T29" s="108"/>
+      <c r="B29" s="101"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
+      <c r="G29" s="101"/>
+      <c r="H29" s="101"/>
+      <c r="I29" s="101"/>
+      <c r="J29" s="101"/>
+      <c r="K29" s="101"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="101"/>
+      <c r="N29" s="101"/>
+      <c r="O29" s="101"/>
+      <c r="P29" s="101"/>
+      <c r="Q29" s="101"/>
+      <c r="R29" s="101"/>
+      <c r="S29" s="101"/>
+      <c r="T29" s="101"/>
     </row>
     <row r="30" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="137" t="s">
+      <c r="A30" s="107" t="s">
         <v>517</v>
       </c>
-      <c r="B30" s="108"/>
-      <c r="C30" s="108"/>
-      <c r="D30" s="108"/>
-      <c r="E30" s="108"/>
-      <c r="F30" s="108"/>
-      <c r="G30" s="108"/>
-      <c r="H30" s="108"/>
-      <c r="I30" s="108"/>
-      <c r="J30" s="108"/>
-      <c r="K30" s="108"/>
-      <c r="L30" s="108"/>
-      <c r="M30" s="108"/>
-      <c r="N30" s="108"/>
-      <c r="O30" s="108"/>
-      <c r="P30" s="108"/>
-      <c r="Q30" s="108"/>
-      <c r="R30" s="108"/>
-      <c r="S30" s="108"/>
-      <c r="T30" s="108"/>
+      <c r="B30" s="101"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="101"/>
+      <c r="E30" s="101"/>
+      <c r="F30" s="101"/>
+      <c r="G30" s="101"/>
+      <c r="H30" s="101"/>
+      <c r="I30" s="101"/>
+      <c r="J30" s="101"/>
+      <c r="K30" s="101"/>
+      <c r="L30" s="101"/>
+      <c r="M30" s="101"/>
+      <c r="N30" s="101"/>
+      <c r="O30" s="101"/>
+      <c r="P30" s="101"/>
+      <c r="Q30" s="101"/>
+      <c r="R30" s="101"/>
+      <c r="S30" s="101"/>
+      <c r="T30" s="101"/>
     </row>
     <row r="31" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="131" t="s">
+      <c r="A31" s="100" t="s">
         <v>518</v>
       </c>
-      <c r="B31" s="108"/>
-      <c r="C31" s="108"/>
-      <c r="D31" s="108"/>
-      <c r="E31" s="108"/>
-      <c r="F31" s="108"/>
-      <c r="G31" s="108"/>
-      <c r="H31" s="108"/>
-      <c r="I31" s="108"/>
-      <c r="J31" s="108"/>
-      <c r="K31" s="108"/>
-      <c r="L31" s="108"/>
-      <c r="M31" s="108"/>
-      <c r="N31" s="108"/>
-      <c r="O31" s="108"/>
-      <c r="P31" s="108"/>
-      <c r="Q31" s="108"/>
-      <c r="R31" s="108"/>
-      <c r="S31" s="108"/>
-      <c r="T31" s="108"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="101"/>
+      <c r="E31" s="101"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="101"/>
+      <c r="H31" s="101"/>
+      <c r="I31" s="101"/>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="101"/>
+      <c r="O31" s="101"/>
+      <c r="P31" s="101"/>
+      <c r="Q31" s="101"/>
+      <c r="R31" s="101"/>
+      <c r="S31" s="101"/>
+      <c r="T31" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A6:T6"/>
+    <mergeCell ref="A25:T25"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="B22:T22"/>
+    <mergeCell ref="B21:T21"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:T5"/>
+    <mergeCell ref="B23:T23"/>
     <mergeCell ref="A29:T29"/>
     <mergeCell ref="A20:T20"/>
     <mergeCell ref="K2:N2"/>
@@ -9229,19 +9240,8 @@
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
     <mergeCell ref="O2:R2"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A6:T6"/>
-    <mergeCell ref="A25:T25"/>
-    <mergeCell ref="F2:J2"/>
     <mergeCell ref="A27:T27"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B22:T22"/>
     <mergeCell ref="A26:T26"/>
-    <mergeCell ref="B21:T21"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:T5"/>
-    <mergeCell ref="B23:T23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9263,10 +9263,10 @@
       <c r="A1" s="158" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
     </row>
     <row r="2" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="97" t="s">
@@ -9289,10 +9289,10 @@
       <c r="A3" s="161" t="s">
         <v>522</v>
       </c>
-      <c r="B3" s="108"/>
-      <c r="C3" s="108"/>
-      <c r="D3" s="108"/>
-      <c r="E3" s="108"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
     </row>
     <row r="4" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
@@ -9315,10 +9315,10 @@
       <c r="A5" s="159" t="s">
         <v>527</v>
       </c>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101"/>
     </row>
     <row r="6" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="23" t="s">
@@ -9443,10 +9443,10 @@
       <c r="A13" s="160" t="s">
         <v>542</v>
       </c>
-      <c r="B13" s="108"/>
-      <c r="C13" s="108"/>
-      <c r="D13" s="108"/>
-      <c r="E13" s="108"/>
+      <c r="B13" s="101"/>
+      <c r="C13" s="101"/>
+      <c r="D13" s="101"/>
+      <c r="E13" s="101"/>
     </row>
     <row r="14" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="23" t="s">
@@ -9486,10 +9486,10 @@
       <c r="A16" s="157" t="s">
         <v>547</v>
       </c>
-      <c r="B16" s="108"/>
-      <c r="C16" s="108"/>
-      <c r="D16" s="108"/>
-      <c r="E16" s="108"/>
+      <c r="B16" s="101"/>
+      <c r="C16" s="101"/>
+      <c r="D16" s="101"/>
+      <c r="E16" s="101"/>
     </row>
     <row r="17" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="28" t="s">
@@ -9557,133 +9557,133 @@
       <c r="A1" s="158" t="s">
         <v>552</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
+      <c r="J1" s="101"/>
+      <c r="K1" s="101"/>
     </row>
     <row r="2" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="170" t="s">
+      <c r="A2" s="171" t="s">
         <v>553</v>
       </c>
-      <c r="B2" s="108"/>
-      <c r="C2" s="108"/>
-      <c r="D2" s="108"/>
-      <c r="E2" s="108"/>
-      <c r="F2" s="108"/>
-      <c r="G2" s="108"/>
-      <c r="H2" s="108"/>
-      <c r="I2" s="108"/>
-      <c r="J2" s="108"/>
-      <c r="K2" s="108"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="101"/>
+      <c r="I2" s="101"/>
+      <c r="J2" s="101"/>
+      <c r="K2" s="101"/>
     </row>
     <row r="3" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="167" t="s">
+      <c r="A3" s="169" t="s">
         <v>554</v>
       </c>
-      <c r="B3" s="108"/>
-      <c r="C3" s="108"/>
-      <c r="D3" s="108"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="108"/>
-      <c r="H3" s="108"/>
-      <c r="I3" s="108"/>
-      <c r="J3" s="108"/>
-      <c r="K3" s="108"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
     </row>
     <row r="4" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="173" t="s">
+      <c r="A4" s="166" t="s">
         <v>555</v>
       </c>
-      <c r="B4" s="108"/>
-      <c r="C4" s="108"/>
-      <c r="D4" s="108"/>
-      <c r="E4" s="108"/>
-      <c r="F4" s="108"/>
-      <c r="G4" s="108"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="108"/>
-      <c r="J4" s="108"/>
-      <c r="K4" s="108"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="101"/>
+      <c r="D4" s="101"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="101"/>
+      <c r="J4" s="101"/>
+      <c r="K4" s="101"/>
     </row>
     <row r="5" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="162" t="s">
+      <c r="A5" s="172" t="s">
         <v>556</v>
       </c>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="165" t="s">
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="174" t="s">
         <v>557</v>
       </c>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="164" t="s">
+      <c r="F5" s="101"/>
+      <c r="G5" s="101"/>
+      <c r="H5" s="101"/>
+      <c r="I5" s="173" t="s">
         <v>558</v>
       </c>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="101"/>
     </row>
     <row r="6" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="168" t="s">
+      <c r="A6" s="170" t="s">
         <v>559</v>
       </c>
-      <c r="B6" s="108"/>
-      <c r="C6" s="108"/>
-      <c r="D6" s="108"/>
-      <c r="E6" s="174" t="s">
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="101"/>
+      <c r="E6" s="167" t="s">
         <v>560</v>
       </c>
-      <c r="F6" s="108"/>
-      <c r="G6" s="108"/>
-      <c r="H6" s="108"/>
-      <c r="I6" s="172" t="s">
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="101"/>
+      <c r="I6" s="164" t="s">
         <v>561</v>
       </c>
-      <c r="J6" s="108"/>
-      <c r="K6" s="108"/>
+      <c r="J6" s="101"/>
+      <c r="K6" s="101"/>
     </row>
     <row r="7" spans="1:11" ht="52" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="163" t="s">
+      <c r="A7" s="168" t="s">
         <v>562</v>
       </c>
-      <c r="B7" s="108"/>
-      <c r="C7" s="108"/>
-      <c r="D7" s="108"/>
-      <c r="E7" s="163" t="s">
+      <c r="B7" s="101"/>
+      <c r="C7" s="101"/>
+      <c r="D7" s="101"/>
+      <c r="E7" s="168" t="s">
         <v>563</v>
       </c>
-      <c r="F7" s="108"/>
-      <c r="G7" s="108"/>
-      <c r="H7" s="108"/>
-      <c r="I7" s="163" t="s">
+      <c r="F7" s="101"/>
+      <c r="G7" s="101"/>
+      <c r="H7" s="101"/>
+      <c r="I7" s="168" t="s">
         <v>564</v>
       </c>
-      <c r="J7" s="108"/>
-      <c r="K7" s="108"/>
+      <c r="J7" s="101"/>
+      <c r="K7" s="101"/>
     </row>
     <row r="8" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="171" t="s">
+      <c r="A8" s="163" t="s">
         <v>565</v>
       </c>
-      <c r="B8" s="108"/>
-      <c r="C8" s="108"/>
-      <c r="D8" s="108"/>
-      <c r="E8" s="108"/>
-      <c r="F8" s="108"/>
-      <c r="G8" s="108"/>
-      <c r="H8" s="108"/>
-      <c r="I8" s="108"/>
-      <c r="J8" s="108"/>
-      <c r="K8" s="108"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="101"/>
+      <c r="D8" s="101"/>
+      <c r="E8" s="101"/>
+      <c r="F8" s="101"/>
+      <c r="G8" s="101"/>
+      <c r="H8" s="101"/>
+      <c r="I8" s="101"/>
+      <c r="J8" s="101"/>
+      <c r="K8" s="101"/>
     </row>
     <row r="9" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="99" t="s">
@@ -9913,112 +9913,123 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="171" t="s">
+      <c r="A17" s="163" t="s">
         <v>604</v>
       </c>
-      <c r="B17" s="108"/>
-      <c r="C17" s="108"/>
-      <c r="D17" s="108"/>
-      <c r="E17" s="108"/>
-      <c r="F17" s="108"/>
-      <c r="G17" s="108"/>
-      <c r="H17" s="108"/>
-      <c r="I17" s="108"/>
-      <c r="J17" s="108"/>
-      <c r="K17" s="108"/>
+      <c r="B17" s="101"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="101"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="101"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="101"/>
+      <c r="I17" s="101"/>
+      <c r="J17" s="101"/>
+      <c r="K17" s="101"/>
     </row>
     <row r="18" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="166" t="s">
+      <c r="A18" s="165" t="s">
         <v>605</v>
       </c>
-      <c r="B18" s="108"/>
-      <c r="C18" s="108"/>
-      <c r="D18" s="108"/>
-      <c r="E18" s="108"/>
-      <c r="F18" s="108"/>
-      <c r="G18" s="108"/>
-      <c r="H18" s="108"/>
-      <c r="I18" s="108"/>
-      <c r="J18" s="108"/>
-      <c r="K18" s="108"/>
+      <c r="B18" s="101"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="101"/>
+      <c r="J18" s="101"/>
+      <c r="K18" s="101"/>
     </row>
     <row r="19" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="169" t="s">
+      <c r="A19" s="162" t="s">
         <v>606</v>
       </c>
-      <c r="B19" s="108"/>
-      <c r="C19" s="108"/>
-      <c r="D19" s="108"/>
-      <c r="E19" s="108"/>
-      <c r="F19" s="108"/>
-      <c r="G19" s="108"/>
-      <c r="H19" s="108"/>
-      <c r="I19" s="108"/>
-      <c r="J19" s="108"/>
-      <c r="K19" s="108"/>
+      <c r="B19" s="101"/>
+      <c r="C19" s="101"/>
+      <c r="D19" s="101"/>
+      <c r="E19" s="101"/>
+      <c r="F19" s="101"/>
+      <c r="G19" s="101"/>
+      <c r="H19" s="101"/>
+      <c r="I19" s="101"/>
+      <c r="J19" s="101"/>
+      <c r="K19" s="101"/>
     </row>
     <row r="20" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="166" t="s">
+      <c r="A20" s="165" t="s">
         <v>607</v>
       </c>
-      <c r="B20" s="108"/>
-      <c r="C20" s="108"/>
-      <c r="D20" s="108"/>
-      <c r="E20" s="108"/>
-      <c r="F20" s="108"/>
-      <c r="G20" s="108"/>
-      <c r="H20" s="108"/>
-      <c r="I20" s="108"/>
-      <c r="J20" s="108"/>
-      <c r="K20" s="108"/>
+      <c r="B20" s="101"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="101"/>
+      <c r="E20" s="101"/>
+      <c r="F20" s="101"/>
+      <c r="G20" s="101"/>
+      <c r="H20" s="101"/>
+      <c r="I20" s="101"/>
+      <c r="J20" s="101"/>
+      <c r="K20" s="101"/>
     </row>
     <row r="21" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="169" t="s">
+      <c r="A21" s="162" t="s">
         <v>608</v>
       </c>
-      <c r="B21" s="108"/>
-      <c r="C21" s="108"/>
-      <c r="D21" s="108"/>
-      <c r="E21" s="108"/>
-      <c r="F21" s="108"/>
-      <c r="G21" s="108"/>
-      <c r="H21" s="108"/>
-      <c r="I21" s="108"/>
-      <c r="J21" s="108"/>
-      <c r="K21" s="108"/>
+      <c r="B21" s="101"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
     </row>
     <row r="22" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="166" t="s">
+      <c r="A22" s="165" t="s">
         <v>609</v>
       </c>
-      <c r="B22" s="108"/>
-      <c r="C22" s="108"/>
-      <c r="D22" s="108"/>
-      <c r="E22" s="108"/>
-      <c r="F22" s="108"/>
-      <c r="G22" s="108"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="108"/>
-      <c r="J22" s="108"/>
-      <c r="K22" s="108"/>
+      <c r="B22" s="101"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="101"/>
+      <c r="F22" s="101"/>
+      <c r="G22" s="101"/>
+      <c r="H22" s="101"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="101"/>
     </row>
     <row r="23" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="169" t="s">
+      <c r="A23" s="162" t="s">
         <v>610</v>
       </c>
-      <c r="B23" s="108"/>
-      <c r="C23" s="108"/>
-      <c r="D23" s="108"/>
-      <c r="E23" s="108"/>
-      <c r="F23" s="108"/>
-      <c r="G23" s="108"/>
-      <c r="H23" s="108"/>
-      <c r="I23" s="108"/>
-      <c r="J23" s="108"/>
-      <c r="K23" s="108"/>
+      <c r="B23" s="101"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="101"/>
+      <c r="E23" s="101"/>
+      <c r="F23" s="101"/>
+      <c r="G23" s="101"/>
+      <c r="H23" s="101"/>
+      <c r="I23" s="101"/>
+      <c r="J23" s="101"/>
+      <c r="K23" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E7:H7"/>
     <mergeCell ref="A23:K23"/>
     <mergeCell ref="A8:K8"/>
     <mergeCell ref="I6:K6"/>
@@ -10029,17 +10040,6 @@
     <mergeCell ref="A19:K19"/>
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A21:K21"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A17:K17"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="E5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 01/07/2026 14:16
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏨 Planning Hoteles" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🍽️ Planning Restaurantes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="👤 FOCO POR PERSONA" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎨 Renders Challan" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎨 Renders" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Vacaciones" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="67">
+  <fonts count="68">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -422,6 +422,12 @@
       <color rgb="001E8449"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="001C1C1C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="54">
     <fill>
@@ -761,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="256">
+  <cellXfs count="260">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1496,6 +1502,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1863,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1882,7 +1900,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="186" t="inlineStr">
         <is>
-          <t>Semana 29 jun - 3 jul 2026  ·  Actualizado 30 jun</t>
+          <t>Semana 29 jun - 3 jul 2026  ·  Actualizado 1 jul</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1955,7 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Naiara quedaría sola para el montaje de agosto sin 3ª persona. Fecha montaje se decide el 30 jun. Sin resolver: quién cubre el montaje.</t>
+          <t>Montaje confirmado semana del 10 ago. Naiara disponible (vacaciones 6-10jul y 17-21ago). Pendiente resolver 3ª persona de apoyo.</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1999,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>✅ Renders pabellón entregados. Siguiente: reunión ingeniería deshumectadora MAÑANA mar 1 jul + videocall Natalia sem 6-10jul (online).</t>
+          <t>HOY: llamar a Gaspar — no podemos perder más tiempo. Proponer que Dejaje cotice sótano en paralelo a Raúl (Natalia tendrá dos opciones). Equipo (Nela+Cristina+Sara): enviar planos sótano a Gaspar + paquete a Raúl + presionar AUNA + cotizar lavandería (Patricia) + mail recap Natalia. Pendiente: reunión revisión presupuestos semana del 6 jul (videocall).</t>
         </is>
       </c>
     </row>
@@ -2073,33 +2091,21 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="52" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>PSN OFICINAS</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Jesús + Alejandra</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Reunión el miércoles 1 jul. Planning: PE agosto, obra octubre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+    <row r="13" ht="52" customHeight="1"/>
+    <row r="14">
+      <c r="A14" s="188" t="inlineStr">
+        <is>
+          <t>📋  HITOS DE LA SEMANA (25-27 junio)</t>
+        </is>
+      </c>
+      <c r="B14" s="152" t="n"/>
+      <c r="C14" s="152" t="n"/>
+      <c r="D14" s="153" t="n"/>
+    </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="188" t="inlineStr">
-        <is>
-          <t>📋  HITOS DE LA SEMANA (25-27 junio)</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>CUÁNDO</t>
         </is>
       </c>
       <c r="B15" s="152" t="n"/>
@@ -2107,24 +2113,24 @@
       <c r="D15" s="153" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>CUÁNDO</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>PROYECTO</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>QUIÉN</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>QUÉ</t>
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Hoy lun 29</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Bernabéu</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Naiara</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Medir moquetas — dato clave para decidir montaje agosto</t>
         </is>
       </c>
     </row>
@@ -2134,208 +2140,196 @@
           <t>Hoy lun 29</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Bernabéu</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>Naiara</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Medir moquetas — dato clave para decidir montaje agosto</t>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Sara + Alejandra</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Visita de obra</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Hoy lun 29</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Santander</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Sara + Alejandra</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Visita de obra</t>
+          <t>Mar 1 jul</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Viuda de Aldama</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Cristina</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>HOY: llamar a Gaspar — no podemos perder más tiempo. Proponer que Dejaje cotice sótano en paralelo a Raúl (Natalia tendrá dos opciones). Equipo (Nela+Cristina+Sara): enviar planos sótano a Gaspar + paquete a Raúl + presionar AUNA + cotizar lavandería (Patricia) + mail recap Natalia. Pendiente: reunión revisión presupuestos semana del 6 jul (videocall).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Mar 1 jul</t>
+          <t>Esta semana</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Viuda de Aldama</t>
+          <t>Tepeyac</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>Cristina</t>
+          <t>Raúl + Alejandra + Paula + PM</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Reunión ingeniería deshumectadora piscina</t>
+          <t>Reunión presupuesto (confirmar día)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Mié 1 jul</t>
+          <t>Esta semana</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>PSN Oficinas</t>
+          <t>Lagos 132</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Jesús + Alejandra</t>
+          <t>Sofía</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>✅ Realizada — pendiente fecha medición</t>
+          <t>Reunión semanal miércoles con clientes</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Esta semana</t>
+          <t>2-3 jul</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Tepeyac</t>
+          <t>Ibiza</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>Raúl + Alejandra + Paula + PM</t>
+          <t>Sara + Alejandra</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Reunión presupuesto (confirmar día)</t>
+          <t>Reunión deco (primera de varias)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Esta semana</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
+          <t>Jue 2 jul</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Lagos 132</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Sofía</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Reunión semanal miércoles con clientes</t>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Alejandra+Sofía+Cliente</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Reunión especial (distinta a la semanal de PM)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2-3 jul</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Ibiza</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>Sara + Alejandra</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Reunión deco (primera de varias)</t>
+          <t>Sem 6 jul</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>La Rinconada</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Cristina</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Entregar presupuesto deco 100% — permite hacer pedidos</t>
         </is>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Jue 2 jul</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Lagos 132</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Alejandra+Sofía+Cliente</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Reunión especial (distinta a la semanal de PM)</t>
-        </is>
-      </c>
+      <c r="A24" s="157" t="n"/>
+      <c r="B24" s="157" t="n"/>
+      <c r="C24" s="157" t="n"/>
+      <c r="D24" s="157" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Sem 6 jul</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>La Rinconada</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Cristina</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Entregar presupuesto deco 100% — permite hacer pedidos</t>
-        </is>
-      </c>
+      <c r="A25" s="189" t="inlineStr">
+        <is>
+          <t>📅  MONTAJES CONFIRMADOS — JULIO / AGOSTO</t>
+        </is>
+      </c>
+      <c r="B25" s="152" t="n"/>
+      <c r="C25" s="152" t="n"/>
+      <c r="D25" s="153" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="157" t="n"/>
-      <c r="B26" s="157" t="n"/>
-      <c r="C26" s="157" t="n"/>
-      <c r="D26" s="157" t="n"/>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>FECHAS</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>EQUIPO</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>NOTAS</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="189" t="inlineStr">
-        <is>
-          <t>📅  MONTAJES CONFIRMADOS — JULIO / AGOSTO</t>
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>7-17 jul</t>
         </is>
       </c>
       <c r="B27" s="152" t="n"/>
@@ -2343,230 +2337,203 @@
       <c r="D27" s="153" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>FECHAS</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>PROYECTO</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>EQUIPO</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>NOTAS</t>
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>13-26 jul</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Gamal RD</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>Sofía(13) · Olatz(15) · Alejandra(20)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Viaje República Dominicana</t>
         </is>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>7-17 jul</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>Pedraza</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>Olatz + Paula</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Del 13 entran tapiceros y cortinas</t>
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>16-17 jul</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Zahara</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>Paula + Alejandra</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>⚠ Retrasado · Raúl tiene que confirmar</t>
         </is>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="18" t="inlineStr">
         <is>
-          <t>13-26 jul</t>
+          <t>21-24 jul</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Gamal RD</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Sofía(13) · Olatz(15) · Alejandra(20)</t>
+          <t>Sara + Andrea</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Viaje República Dominicana</t>
+          <t>Entrega oficial 27 jul con Alejandra</t>
         </is>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>16-17 jul</t>
+          <t>27 jul</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Zahara</t>
+          <t>Valencia — Entrega</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Paula + Alejandra</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>⚠ Retrasado · Raúl tiene que confirmar</t>
+          <t>Sara + Andrea + Alejandra</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Entrega oficial</t>
         </is>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="18" t="inlineStr">
-        <is>
-          <t>21-24 jul</t>
-        </is>
-      </c>
-      <c r="B32" s="19" t="inlineStr">
-        <is>
-          <t>Valencia</t>
-        </is>
-      </c>
-      <c r="C32" s="19" t="inlineStr">
-        <is>
-          <t>Sara + Andrea</t>
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>27-30 jul</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>One Shot Bilbao</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Marta</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Entrega oficial 27 jul con Alejandra</t>
+          <t>Jesús vacaciones — Marta cubre</t>
         </is>
       </c>
     </row>
     <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
-          <t>27 jul</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t>Valencia — Entrega</t>
-        </is>
-      </c>
-      <c r="C33" s="19" t="inlineStr">
-        <is>
-          <t>Sara + Andrea + Alejandra</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Entrega oficial</t>
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>Ago — sin fecha</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Bernabéu</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Naiara + 3ª persona ⚠</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Montaje confirmado semana del 10 ago. Naiara disponible (vacaciones 6-10jul y 17-21ago). Pendiente resolver 3ª persona de apoyo.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>27-30 jul</t>
-        </is>
-      </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>One Shot Bilbao</t>
-        </is>
-      </c>
-      <c r="C34" s="17" t="inlineStr">
-        <is>
-          <t>Marta</t>
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Finales ago</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Don Ramón (Sevilla)</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Marta · Alejandra puntual</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Jesús vacaciones — Marta cubre</t>
+          <t>Alejandra puede pasarse</t>
         </is>
       </c>
     </row>
     <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="20" t="inlineStr">
-        <is>
-          <t>Ago — sin fecha</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Bernabéu</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="inlineStr">
-        <is>
-          <t>Naiara + 3ª persona ⚠</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>⚠ Fecha decide 30 jun · 3ª persona sin resolver · Laia ya no estará</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="18" t="inlineStr">
-        <is>
-          <t>Finales ago</t>
-        </is>
-      </c>
-      <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>Don Ramón (Sevilla)</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="inlineStr">
-        <is>
-          <t>Marta · Alejandra puntual</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Alejandra puede pasarse</t>
-        </is>
-      </c>
-    </row>
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>~20 sep · 1-2 sem</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>Pedraza (fase exterior)</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>Olatz + Paula</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Sin becarias · pendiente confirmar Amarco · obra exterior/piscina/cuadras</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1"/>
     <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="21" t="inlineStr">
-        <is>
-          <t>~20 sep · 1-2 sem</t>
-        </is>
-      </c>
-      <c r="B37" s="22" t="inlineStr">
-        <is>
-          <t>Pedraza (fase exterior)</t>
-        </is>
-      </c>
-      <c r="C37" s="22" t="inlineStr">
-        <is>
-          <t>Olatz + Paula</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Sin becarias · pendiente confirmar Amarco · obra exterior/piscina/cuadras</t>
-        </is>
-      </c>
-    </row>
-    <row r="38"/>
+      <c r="A37" s="190" t="inlineStr">
+        <is>
+          <t>📅  TU PRESENCIA COMPROMETIDA</t>
+        </is>
+      </c>
+      <c r="B37" s="152" t="n"/>
+      <c r="C37" s="152" t="n"/>
+      <c r="D37" s="153" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="191" t="inlineStr">
+        <is>
+          <t>Solo se incluyen compromisos donde tu presencia es necesaria o relevante</t>
+        </is>
+      </c>
+    </row>
     <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="190" t="inlineStr">
-        <is>
-          <t>📅  TU PRESENCIA COMPROMETIDA</t>
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>FECHA</t>
         </is>
       </c>
       <c r="B39" s="152" t="n"/>
@@ -2574,21 +2541,24 @@
       <c r="D39" s="153" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="191" t="inlineStr">
-        <is>
-          <t>Solo se incluyen compromisos donde tu presencia es necesaria o relevante</t>
-        </is>
-      </c>
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>25 jun</t>
+        </is>
+      </c>
+      <c r="B40" s="152" t="n"/>
+      <c r="C40" s="152" t="n"/>
+      <c r="D40" s="153" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
-        <is>
-          <t>FECHA</t>
-        </is>
-      </c>
-      <c r="B41" s="192" t="inlineStr">
-        <is>
-          <t>COMPROMISO</t>
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>2-3 jul</t>
+        </is>
+      </c>
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>IBIZA — reunión deco con Sara (primera de varias)</t>
         </is>
       </c>
       <c r="C41" s="152" t="n"/>
@@ -2597,12 +2567,12 @@
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>25 jun</t>
+          <t>7-17 jul</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Visita Sevilla — Don Ramón (visita) + Hotel Sevilla (revisión) · con Marta</t>
+          <t>Pedraza — montaje (seguimiento, no presencia física necesaria)</t>
         </is>
       </c>
       <c r="C42" s="152" t="n"/>
@@ -2611,12 +2581,12 @@
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="29" t="inlineStr">
         <is>
-          <t>2-3 jul</t>
+          <t>16-17 jul</t>
         </is>
       </c>
       <c r="B43" s="34" t="inlineStr">
         <is>
-          <t>IBIZA — reunión deco con Sara (primera de varias)</t>
+          <t>Zahara — montaje · con Paula</t>
         </is>
       </c>
       <c r="C43" s="152" t="n"/>
@@ -2625,12 +2595,12 @@
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>7-17 jul</t>
+          <t>13-26 jul</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Pedraza — montaje (seguimiento, no presencia física necesaria)</t>
+          <t>Gamal RD — viaje República Dominicana · tú entras el 20 jul</t>
         </is>
       </c>
       <c r="C44" s="152" t="n"/>
@@ -2639,12 +2609,12 @@
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="29" t="inlineStr">
         <is>
-          <t>16-17 jul</t>
+          <t>21-24 jul</t>
         </is>
       </c>
       <c r="B45" s="34" t="inlineStr">
         <is>
-          <t>Zahara — montaje · con Paula</t>
+          <t>Valencia — montaje · con Sara y Andrea</t>
         </is>
       </c>
       <c r="C45" s="152" t="n"/>
@@ -2653,12 +2623,12 @@
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>13-26 jul</t>
+          <t>27 jul</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Gamal RD — viaje República Dominicana · tú entras el 20 jul</t>
+          <t>Valencia — entrega oficial · con Sara y Andrea</t>
         </is>
       </c>
       <c r="C46" s="152" t="n"/>
@@ -2667,12 +2637,12 @@
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="29" t="inlineStr">
         <is>
-          <t>21-24 jul</t>
+          <t>Ago sin fecha</t>
         </is>
       </c>
       <c r="B47" s="34" t="inlineStr">
         <is>
-          <t>Valencia — montaje · con Sara y Andrea</t>
+          <t>Bernabéu — montaje pendiente de confirmar fecha (decide 30 jun)</t>
         </is>
       </c>
       <c r="C47" s="152" t="n"/>
@@ -2681,12 +2651,12 @@
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>27 jul</t>
+          <t>Finales ago</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Valencia — entrega oficial · con Sara y Andrea</t>
+          <t>Don Ramón — montaje en Sevilla (Marta ejecuta · tú puedes pasarte)</t>
         </is>
       </c>
       <c r="C48" s="152" t="n"/>
@@ -2695,50 +2665,46 @@
     <row r="49" ht="28" customHeight="1">
       <c r="A49" s="29" t="inlineStr">
         <is>
-          <t>Ago sin fecha</t>
+          <t>3-21 ago</t>
         </is>
       </c>
       <c r="B49" s="34" t="inlineStr">
         <is>
-          <t>Bernabéu — montaje pendiente de confirmar fecha (decide 30 jun)</t>
+          <t>Vacaciones</t>
         </is>
       </c>
       <c r="C49" s="152" t="n"/>
       <c r="D49" s="153" t="n"/>
     </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="27" t="inlineStr">
-        <is>
-          <t>Finales ago</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>Don Ramón — montaje en Sevilla (Marta ejecuta · tú puedes pasarte)</t>
-        </is>
-      </c>
-      <c r="C50" s="152" t="n"/>
-      <c r="D50" s="153" t="n"/>
-    </row>
+    <row r="50" ht="28" customHeight="1"/>
     <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="29" t="inlineStr">
-        <is>
-          <t>3-21 ago</t>
-        </is>
-      </c>
-      <c r="B51" s="34" t="inlineStr">
-        <is>
-          <t>Vacaciones</t>
-        </is>
-      </c>
+      <c r="A51" s="193" t="inlineStr">
+        <is>
+          <t>🔮  PRÓXIMAS SEMANAS — TENER EN CUENTA</t>
+        </is>
+      </c>
+      <c r="B51" s="153" t="n"/>
       <c r="C51" s="152" t="n"/>
       <c r="D51" s="153" t="n"/>
     </row>
-    <row r="52"/>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>SEMANA</t>
+        </is>
+      </c>
+      <c r="B52" s="194" t="inlineStr">
+        <is>
+          <t>LO QUE VIENE</t>
+        </is>
+      </c>
+      <c r="C52" s="152" t="n"/>
+      <c r="D52" s="153" t="n"/>
+    </row>
     <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="193" t="inlineStr">
-        <is>
-          <t>🔮  PRÓXIMAS SEMANAS — TENER EN CUENTA</t>
+      <c r="A53" s="33" t="inlineStr">
+        <is>
+          <t>29 jun</t>
         </is>
       </c>
       <c r="B53" s="152" t="n"/>
@@ -2746,14 +2712,14 @@
       <c r="D53" s="153" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>SEMANA</t>
-        </is>
-      </c>
-      <c r="B54" s="194" t="inlineStr">
-        <is>
-          <t>LO QUE VIENE</t>
+      <c r="A54" s="33" t="inlineStr">
+        <is>
+          <t>6-10 jul</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>🚨 Semana densa: Pedraza montaje en curso · Viuda Aldama videocall revisión presupuestos (Natalia) · Laia ultima semana en el estudio</t>
         </is>
       </c>
       <c r="C54" s="152" t="n"/>
@@ -2762,12 +2728,12 @@
     <row r="55" ht="44" customHeight="1">
       <c r="A55" s="33" t="inlineStr">
         <is>
-          <t>29 jun</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Medir moquetas Bernabéu (Naiara) · Viuda Aldama reunión ingeniería deshumectadora MARTES 1jul · Tepeyac reunión presupuesto con Raúl + tú + Paula + PM · Santander visita 29jun (Sara+Alejandra)</t>
+          <t>13-17 jul</t>
+        </is>
+      </c>
+      <c r="B55" s="34" t="inlineStr">
+        <is>
+          <t>🚨 Laia sale · Pedraza termina 17jul · Zahara montaje 16-17jul (tú) · Gamal RD en curso (Olatz desde 13) · Jesús inicia vacaciones</t>
         </is>
       </c>
       <c r="C55" s="152" t="n"/>
@@ -2776,12 +2742,12 @@
     <row r="56" ht="44" customHeight="1">
       <c r="A56" s="33" t="inlineStr">
         <is>
-          <t>6-10 jul</t>
+          <t>20-27 jul</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>🚨 Semana densa: Pedraza montaje en curso · Viuda Aldama videocall revisión presupuestos (Natalia) · Laia ultima semana en el estudio</t>
+          <t>Gamal RD (tú entras 20jul) · Valencia montaje 21-24jul · Entrega Valencia 27jul (tú+Sara+Andrea) · One Shot Bilbao 27-30jul (Marta)</t>
         </is>
       </c>
       <c r="C56" s="152" t="n"/>
@@ -2790,53 +2756,27 @@
     <row r="57" ht="44" customHeight="1">
       <c r="A57" s="33" t="inlineStr">
         <is>
-          <t>13-17 jul</t>
+          <t>3-21 ago</t>
         </is>
       </c>
       <c r="B57" s="34" t="inlineStr">
         <is>
-          <t>🚨 Laia sale · Pedraza termina 17jul · Zahara montaje 16-17jul (tú) · Gamal RD en curso (Olatz desde 13) · Jesús inicia vacaciones</t>
+          <t>Montaje confirmado semana del 10 ago. Naiara disponible (vacaciones 6-10jul y 17-21ago). Pendiente resolver 3ª persona de apoyo.</t>
         </is>
       </c>
       <c r="C57" s="152" t="n"/>
       <c r="D57" s="153" t="n"/>
     </row>
-    <row r="58" ht="44" customHeight="1">
-      <c r="A58" s="33" t="inlineStr">
-        <is>
-          <t>20-27 jul</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>Gamal RD (tú entras 20jul) · Valencia montaje 21-24jul · Entrega Valencia 27jul (tú+Sara+Andrea) · One Shot Bilbao 27-30jul (Marta)</t>
-        </is>
-      </c>
-      <c r="C58" s="152" t="n"/>
-      <c r="D58" s="153" t="n"/>
-    </row>
+    <row r="58" ht="44" customHeight="1"/>
     <row r="59" ht="44" customHeight="1">
-      <c r="A59" s="33" t="inlineStr">
-        <is>
-          <t>3-21 ago</t>
-        </is>
-      </c>
-      <c r="B59" s="34" t="inlineStr">
-        <is>
-          <t>Estudio muy reducido · ⚠ Bernabéu sin resolver · Challan vacaciones 1-15ago · Nela disponible (no vacaciones)</t>
-        </is>
-      </c>
-      <c r="C59" s="152" t="n"/>
-      <c r="D59" s="153" t="n"/>
+      <c r="A59" s="35" t="inlineStr">
+        <is>
+          <t>Alejandra Pombo Design Studio  ·  PM Estudio  ·  25 junio 2026</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="44" customHeight="1"/>
-    <row r="61">
-      <c r="A61" s="35" t="inlineStr">
-        <is>
-          <t>Alejandra Pombo Design Studio  ·  PM Estudio  ·  25 junio 2026</t>
-        </is>
-      </c>
-    </row>
+    <row r="61"/>
     <row r="62" ht="16" customHeight="1"/>
   </sheetData>
   <mergeCells count="27">
@@ -3069,22 +3009,22 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>✅ Renders pabellón entregados · Siguiente: reunión ingeniería deshumectadora mar 1jul · videocall Natalia sem 6-10jul</t>
-        </is>
-      </c>
-      <c r="E6" s="154" t="inlineStr">
-        <is>
-          <t>Mar 1 jul</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>Natalia de vacaciones 22jun-20jul — reuniones online · Raúl valorando presupuesto</t>
+          <t>Obra en curso · presupuestos en proceso</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>HOY: Ale llama a Gaspar · enviar planos sótano y paquete a Raúl · mail a Natalia recap · presionar AUNA · cotizar lavandería (Patricia)</t>
+        </is>
+      </c>
+      <c r="F6" s="49" t="inlineStr">
+        <is>
+          <t>Hoy 1 jul</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Renders comprometidos mañana · Raúl valorando sin fecha · Natalia vacaciones 22jun-20jul y 23jul-20ago</t>
+          <t>Presupuesto Raúl pendiente · AUNA pendiente · Natalia vacaciones hasta 20jul (online) · Gaspar/Dejaje como alternativa sótano</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -3126,22 +3066,22 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Sin novedades · fecha montaje y 3ª persona sin resolver</t>
-        </is>
-      </c>
-      <c r="E7" s="155" t="inlineStr">
-        <is>
-          <t>30 jun</t>
-        </is>
-      </c>
-      <c r="F7" s="22" t="inlineStr">
-        <is>
-          <t>⚠ Fecha montaje agosto sin decidir · Naiara sola · sin 3ª persona</t>
+          <t>Pedidos en curso — montaje confirmado</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Montaje semana del 10 ago · Naiara disponible (vacaciones 6-10jul y 17-21ago)</t>
+        </is>
+      </c>
+      <c r="F7" s="49" t="inlineStr">
+        <is>
+          <t>10 ago</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>⚠ Naiara sola en montaje · sin 3ª persona</t>
+          <t>Sin 3ª persona aún · Laia ya no está · Naiara asume</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -3154,14 +3094,14 @@
           <t>PEDIDOS</t>
         </is>
       </c>
-      <c r="J7" s="44" t="inlineStr">
-        <is>
-          <t>MÁXIMA</t>
-        </is>
-      </c>
-      <c r="K7" s="44" t="inlineStr">
-        <is>
-          <t>ATENCIÓN MÁXIMA</t>
+      <c r="J7" s="53" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="K7" s="53" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3276,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="45" t="inlineStr">
         <is>
           <t>COBUE</t>
@@ -3354,22 +3294,22 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Planta rectificada recibida</t>
+          <t>Proyecto básico en desarrollo</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Arrancar 3 renders con renderista nuevo · cliente esperando</t>
-        </is>
-      </c>
-      <c r="F11" s="42" t="inlineStr">
-        <is>
-          <t>Esta semana</t>
+          <t>Revisión + coordinación con ingeniería (4-5 sem) · 3 renders con Renderista 2 (pdte nombre)</t>
+        </is>
+      </c>
+      <c r="F11" s="49" t="inlineStr">
+        <is>
+          <t>Jul-Ago 2026</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Renders con renderista nuevo (no Challan)</t>
+          <t>Renderista 2 pendiente de definir · cliente esperando renders</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -4419,7 +4359,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
+    <row r="30" ht="40" customHeight="1">
       <c r="A30" s="40" t="inlineStr">
         <is>
           <t>RUBAIYAT SP</t>
@@ -4437,22 +4377,22 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Honorarios aceptados esta sem</t>
+          <t>Kickoff confirmado</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Kickoff pendiente · 5 renders comprometidos · obra enero 2027</t>
-        </is>
-      </c>
-      <c r="F30" s="56" t="inlineStr">
-        <is>
-          <t>Ene 2027</t>
+          <t>Kickoff mié 8 jul 14h · 5 renders comprometidos · obra ene 2027 por fases</t>
+        </is>
+      </c>
+      <c r="F30" s="49" t="inlineStr">
+        <is>
+          <t>8 jul</t>
         </is>
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>Naiara asume sola · proyecto en Brasil por fases</t>
+          <t>Proyecto en Brasil · restaurante abierto · cocina cierra ~20 días</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
@@ -5985,7 +5925,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="203" t="inlineStr">
         <is>
-          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP 2026  |  30 jun 2026</t>
+          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP 2026  |  1 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -7196,9 +7136,9 @@
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="C26:T26"/>
+    <mergeCell ref="A31:T31"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C29:T29"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A31:T31"/>
     <mergeCell ref="A34:T34"/>
     <mergeCell ref="O2:R2"/>
     <mergeCell ref="A36:T36"/>
@@ -7264,7 +7204,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="220" t="inlineStr">
         <is>
-          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP 2026  |  30 jun 2026</t>
+          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP 2026  |  1 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -8018,9 +7958,9 @@
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="215" t="inlineStr">
-        <is>
-          <t>📅 PSN: reunión mié 1 jul (primera) · PE agosto · obra octubre</t>
+      <c r="A28" s="119" t="inlineStr">
+        <is>
+          <t>📅 PSN: pendientes de que el cliente comunique fecha para ir a medir · planning previsto PE agosto, obra octubre</t>
         </is>
       </c>
     </row>
@@ -8053,7 +7993,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="23">
     <mergeCell ref="B19:T19"/>
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
@@ -8077,7 +8017,6 @@
     <mergeCell ref="B23:T23"/>
     <mergeCell ref="A29:T29"/>
     <mergeCell ref="K2:N2"/>
-    <mergeCell ref="A28:T28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8117,7 +8056,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="223" t="inlineStr">
         <is>
-          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP 2026  |  30 jun 2026</t>
+          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP 2026  |  1 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -8296,6 +8235,21 @@
           <t>✅ Redistribución aplicada: Bernabéu+Hipódromo+Rubaiyat SP→Naiara · Cobue→Sofía+Naiara · Nuevo Mallorca→latente</t>
         </is>
       </c>
+      <c r="D6" s="89" t="inlineStr">
+        <is>
+          <t>RC·mié8</t>
+        </is>
+      </c>
+      <c r="I6" s="88" t="inlineStr">
+        <is>
+          <t>MONTAJE</t>
+        </is>
+      </c>
+      <c r="J6" s="88" t="inlineStr">
+        <is>
+          <t>MONTAJE</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="226" t="inlineStr">
@@ -8880,13 +8834,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
     <mergeCell ref="O2:R2"/>
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A6:T6"/>
     <mergeCell ref="A25:T25"/>
     <mergeCell ref="F2:J2"/>
     <mergeCell ref="A27:T27"/>
@@ -8981,7 +8934,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>HOY: visita Santander con Sara · PSN: reunión mié 1jul con Jesús · Tepeyac: reunión presupuesto esta semana · Ibiza: reunión deco 2-3jul con Sara · Julio muy cargado: Pedraza(seg) · Zahara(16-17jul) · Gamal(13-26jul,entra20) · Valencia(21-27jul)</t>
+          <t>HOY: visita Santander con Sara · Tepeyac: reunión presupuesto esta semana · Ibiza: reunión deco 2-3jul con Sara · Julio muy cargado: Pedraza(seg) · Zahara(16-17jul) · Gamal(13-26jul,entra20) · Valencia(21-27jul)</t>
         </is>
       </c>
       <c r="E4" s="53" t="inlineStr">
@@ -9015,7 +8968,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Tepeyac: reunión presupuesto esta semana (Raúl+Ale+Paula+PM) · PSN: reunión mié 1jul · Viuda Aldama: reunión ingeniería deshumectadora mañana mar 1jul · Bernabéu: resolver 3ª persona urgente · LAGOS 132: reunión semanal miércoles (solo PM) · jueves 2jul reunión con Alejandra+Sofía+cliente</t>
+          <t>Tepeyac: reunión presupuesto esta semana (Raúl+Ale+Paula+PM) · Viuda Aldama: pendiente reunión revisión presupuestos semana del 6 jul (videocall Natalia) · Bernabéu: resolver 3ª persona urgente · LAGOS 132: reunión semanal miércoles (solo PM) · jueves 2jul reunión con Alejandra+Sofía+cliente</t>
         </is>
       </c>
       <c r="E6" s="44" t="inlineStr">
@@ -9069,7 +9022,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>HOY: visita Santander con Alejandra · Ibiza: reunión deco 2-3jul con Alejandra · Valencia: montaje 21-24jul · Viuda Aldama: apoyo puntual a Cristina</t>
+          <t>HOY: visita Santander con Alejandra · Ibiza: reunión deco 2-3jul con Alejandra · Valencia: montaje 21-24jul · Viuda Aldama: apoyo puntual a Cristina · VIUDA ALDAMA: apoyo hoy con planos y mail recap Natalia</t>
         </is>
       </c>
       <c r="E8" s="53" t="inlineStr">
@@ -9123,7 +9076,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>VIUDA ALDAMA: reunión ingeniería deshumectadora realizada · preparar videocall Natalia sem 6-10jul · LA RINCONADA: ⚠ entregar presupuesto deco 100% semana que viene (permite pedidos) · reunión siguiente semana 13jul lo antes posible (vacaciones desde 20jul) · Camino Sur 70: montaje 7-10jul</t>
+          <t>VIUDA ALDAMA: ✅ ingeniería deshumectadora realizada · pendiente reunión revisión presupuestos semana del 6 jul (videocall Natalia) · LA RINCONADA: ⚠ entregar presupuesto deco 100% semana que viene (permite pedidos) · reunión siguiente semana 13jul lo antes posible (vacaciones desde 20jul) · Camino Sur 70: montaje 7-10jul · VIUDA ALDAMA HOY: planos sótano a Gaspar · paquete a Raúl · AUNA · cotizar lavandería (Patricia) · mail recap Natalia</t>
         </is>
       </c>
       <c r="E10" s="44" t="inlineStr">
@@ -9172,12 +9125,12 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo)</t>
+          <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo) · Viuda de Aldama (equipo)</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Camino Sur 70: montaje esta semana 7-10jul · Hermosilla+Camino Sur 35: responsable · ⚠ No coge vacaciones agosto — disponible</t>
+          <t>Camino Sur 70: montaje esta semana 7-10jul · Hermosilla+Camino Sur 35: responsable · ⚠ No coge vacaciones agosto — disponible · VIUDA ALDAMA: HOY enviar planos sótano a Gaspar + paquete a Raúl + mail a Natalia recap</t>
         </is>
       </c>
       <c r="E12" s="53" t="inlineStr">
@@ -9238,7 +9191,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>BERNABÉU: medir moquetas HOY · fecha montaje agosto pendiente resolver urgente · Hipódromo: presupuesto mobiliario en 2 semanas máx · Rubaiyat SP: asumir como responsable</t>
+          <t>BERNABÉU: medir moquetas HOY · montaje confirmado semana 10 ago ✅ · Hipódromo: presupuesto mobiliario en 2 semanas máx · Rubaiyat SP: asumir como responsable · Rubaiyat SP: kickoff mié 8jul 14h</t>
         </is>
       </c>
       <c r="E15" s="44" t="inlineStr">
@@ -9326,7 +9279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9345,7 +9298,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>RENDERS — COLA Y ESTADO  |  30 jun 2026</t>
+          <t>RENDERS — COLA Y ESTADO  |  1 jul 2026</t>
         </is>
       </c>
     </row>
@@ -9871,17 +9824,88 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="256" t="inlineStr">
+        <is>
+          <t>▸ RENDERISTA 2 — Pendiente de nombre · en proceso de incorporación</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="257" t="inlineStr">
+        <is>
+          <t>Dada la carga actual de renders, se está valorando incorporar un segundo renderista. Cuando se defina, se anotará aquí el nombre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="258" t="inlineStr">
+        <is>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="B27" s="259" t="inlineStr">
+        <is>
+          <t>RESP.</t>
+        </is>
+      </c>
+      <c r="C27" s="259" t="inlineStr">
+        <is>
+          <t>ESTADO</t>
+        </is>
+      </c>
+      <c r="D27" s="259" t="inlineStr">
+        <is>
+          <t>TIPO RENDER</t>
+        </is>
+      </c>
+      <c r="E27" s="259" t="inlineStr">
+        <is>
+          <t>NOTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>COBUE</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Sofía + Naiara</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Planta rectificada recibida · arrancar renders</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>3 renders F1→F2→F3</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>Renderista nuevo (no Challan) · cliente esperando</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="23">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="E7:H7"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="I5:K5"/>
+    <mergeCell ref="A25:K25"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A26:K26"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A23:K23"/>
@@ -9945,7 +9969,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="239" t="inlineStr">
         <is>
-          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 30 jun 2026</t>
+          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 1 jul 2026</t>
         </is>
       </c>
     </row>
@@ -10925,6 +10949,8 @@
       <c r="AE18" s="247" t="inlineStr"/>
       <c r="AF18" s="247" t="inlineStr"/>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="240" t="inlineStr">
         <is>
@@ -12252,6 +12278,8 @@
       <c r="AE36" s="248" t="inlineStr"/>
       <c r="AF36" s="247" t="inlineStr"/>
     </row>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="240" t="inlineStr">
         <is>
@@ -13022,6 +13050,8 @@
       <c r="AD54" s="247" t="inlineStr"/>
       <c r="AE54" s="247" t="inlineStr"/>
     </row>
+    <row r="55"/>
+    <row r="56"/>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="254" t="inlineStr">
         <is>
@@ -13029,6 +13059,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="139" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 02/07/2026 14:22
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="68">
+  <fonts count="69">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -428,8 +428,14 @@
       <color rgb="001C1C1C"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001C1C1C"/>
+      <sz val="7"/>
+    </font>
   </fonts>
-  <fills count="54">
+  <fills count="55">
     <fill>
       <patternFill/>
     </fill>
@@ -696,6 +702,11 @@
         <fgColor rgb="00F5B7B1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFA500"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -767,7 +778,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="260">
+  <cellXfs count="262">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1515,6 +1526,12 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="54" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1900,11 +1917,10 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="186" t="inlineStr">
         <is>
-          <t>Semana 29 jun - 3 jul 2026  ·  Actualizado 1 jul</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Semana 29 jun - 5 jul 2026  ·  Actualizado 2 jul 2026</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="187" t="inlineStr">
         <is>
@@ -2776,7 +2792,6 @@
       </c>
     </row>
     <row r="60" ht="44" customHeight="1"/>
-    <row r="61"/>
     <row r="62" ht="16" customHeight="1"/>
   </sheetData>
   <mergeCells count="27">
@@ -2837,7 +2852,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="195" t="inlineStr">
         <is>
-          <t>PM ESTUDIO — MASTER GLOBAL  |  29 junio 2026</t>
+          <t>PM ESTUDIO — MASTER GLOBAL  |  2 julio 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -3004,27 +3019,27 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Cristina(resp.) + Sara(apoyo)</t>
+          <t>Nela (resp.) · Cristina (apoyo) · Sara (puntual)</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Obra en curso · presupuestos en proceso</t>
+          <t>Presupuestos en proceso · acciones en curso hoy</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>HOY: Ale llama a Gaspar · enviar planos sótano y paquete a Raúl · mail a Natalia recap · presionar AUNA · cotizar lavandería (Patricia)</t>
+          <t>Trasladar presupuestos a Natalia · reunión revisión sem 6 jul (videocall)</t>
         </is>
       </c>
       <c r="F6" s="49" t="inlineStr">
         <is>
-          <t>Hoy 1 jul</t>
+          <t>Sem 6 jul</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Presupuesto Raúl pendiente · AUNA pendiente · Natalia vacaciones hasta 20jul (online) · Gaspar/Dejaje como alternativa sótano</t>
+          <t>Presupuesto Raúl pdte · AUNA pdte · Dejaje como alternativa sótano · Natalia vacaciones (online)</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -3219,7 +3234,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
           <t>ZAHARA</t>
@@ -3242,7 +3257,7 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Montaje retrasado al 16-17 jul · Raúl tiene que confirmar</t>
+          <t>Montaje 16-17 jul (se intenta mantener) · Raúl pendiente de confirmar</t>
         </is>
       </c>
       <c r="F10" s="49" t="inlineStr">
@@ -3252,7 +3267,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Raúl puede no terminar a tiempo · montaje muy justo 16-17 jul</t>
+          <t>Raúl tiene que confirmar que termina obra a tiempo para el 16 jul</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -3294,12 +3309,12 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Proyecto básico en desarrollo</t>
+          <t>Proyecto básico en curso · casi ejecución</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Revisión + coordinación con ingeniería (4-5 sem) · 3 renders con Renderista 2 (pdte nombre)</t>
+          <t>Avanzar en julio/agosto antes de vacaciones equipo · 3 renders con Renderista 2 (pdte)</t>
         </is>
       </c>
       <c r="F11" s="49" t="inlineStr">
@@ -3309,7 +3324,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Renderista 2 pendiente de definir · cliente esperando renders</t>
+          <t>Julio/agosto complicado (Laia sale, vacaciones Naiara y Sofía) · avanzar ya · renderista 2 sin definir</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -3732,7 +3747,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="45" t="inlineStr">
         <is>
           <t>ABUBILLA</t>
@@ -3750,22 +3765,22 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Remates/extras (3 meses)</t>
+          <t>2 temas pendientes antes de septiembre</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Poner límite al cliente</t>
-        </is>
-      </c>
-      <c r="F19" s="42" t="inlineStr">
-        <is>
-          <t>Esta semana</t>
+          <t>Cerrar tema económico con cliente + extra de mobiliario solicitado</t>
+        </is>
+      </c>
+      <c r="F19" s="49" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>3 meses desde '2 semanas para revisar'</t>
+          <t>Pendiente cerrar ambos temas · ya no es riesgo activo para Andrea</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -3778,14 +3793,14 @@
           <t>ENTREGA</t>
         </is>
       </c>
-      <c r="J19" s="53" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="K19" s="53" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
+      <c r="J19" s="59" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="K19" s="60" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO</t>
         </is>
       </c>
     </row>
@@ -3864,22 +3879,22 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Reunión presupuesto confirmada esta semana (Raúl+Alejandra+Paula+PM) · Demolición prevista agosto</t>
-        </is>
-      </c>
-      <c r="E21" s="154" t="inlineStr">
-        <is>
-          <t>Esta semana</t>
-        </is>
-      </c>
-      <c r="F21" s="47" t="inlineStr">
-        <is>
-          <t>Sem 29 jun</t>
+          <t>✅ Cliente aprueba distribución · reunión presupuesto pendiente</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Cerrar fecha reunión presupuesto (Raúl+Alejandra+Paula+PM) · demolición prevista agosto</t>
+        </is>
+      </c>
+      <c r="F21" s="49" t="inlineStr">
+        <is>
+          <t>Sin fecha concreta</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>⚠ Paula vacaciones 3-21ago — demolición agosto cruzar con disponibilidad</t>
+          <t>Reunión presupuesto sin fecha cerrada · demolición agosto condicionada a Raúl</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -4491,22 +4506,22 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>Reunión semanal miércoles (solo PM) · jueves 2jul reunión especial con Alejandra+Sofía+cliente</t>
-        </is>
-      </c>
-      <c r="E32" s="180" t="inlineStr">
-        <is>
-          <t>Jue 2 jul</t>
-        </is>
-      </c>
-      <c r="F32" s="56" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
+          <t>✅ Reunión jue 2jul muy bien · grifería/sanitarios definidos</t>
+        </is>
+      </c>
+      <c r="E32" s="179" t="inlineStr">
+        <is>
+          <t>Trasladar info grifería/sanitarios a Ferbocar · videocall domótica mar 7jul (Sandra) · visita obra mié (PM)</t>
+        </is>
+      </c>
+      <c r="F32" s="49" t="inlineStr">
+        <is>
+          <t>Mar 7 jul</t>
         </is>
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>⚠ Grifería/sanitarios sin cerrar — obra lo necesita</t>
+          <t>Trasladar definiciones a constructora esta semana</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr">
@@ -5925,7 +5940,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="203" t="inlineStr">
         <is>
-          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP 2026  |  1 jul 2026</t>
+          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP 2026  |  2 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -6513,7 +6528,11 @@
           <t>Sara+Andrea+Ale</t>
         </is>
       </c>
-      <c r="C14" s="103" t="inlineStr"/>
+      <c r="C14" s="260" t="inlineStr">
+        <is>
+          <t>⚠PRE·21jul</t>
+        </is>
+      </c>
       <c r="D14" s="103" t="inlineStr"/>
       <c r="E14" s="103" t="inlineStr"/>
       <c r="F14" s="103" t="inlineStr"/>
@@ -6945,7 +6964,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="207" t="inlineStr">
         <is>
@@ -7021,7 +7039,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="14" customHeight="1">
       <c r="A31" s="211" t="inlineStr">
         <is>
@@ -7204,7 +7221,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="220" t="inlineStr">
         <is>
-          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP 2026  |  1 jul 2026</t>
+          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP 2026  |  2 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -7451,7 +7468,11 @@
       </c>
       <c r="D7" s="104" t="inlineStr"/>
       <c r="E7" s="103" t="inlineStr"/>
-      <c r="F7" s="103" t="inlineStr"/>
+      <c r="F7" s="260" t="inlineStr">
+        <is>
+          <t>⚠PRE·ago</t>
+        </is>
+      </c>
       <c r="G7" s="103" t="inlineStr"/>
       <c r="H7" s="103" t="inlineStr"/>
       <c r="I7" s="103" t="inlineStr"/>
@@ -7857,7 +7878,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="207" t="inlineStr">
         <is>
@@ -7949,7 +7969,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="211" t="inlineStr">
         <is>
@@ -7993,7 +8012,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="22">
     <mergeCell ref="B19:T19"/>
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
@@ -8009,7 +8028,6 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A18:T18"/>
     <mergeCell ref="B22:T22"/>
-    <mergeCell ref="J7:K7"/>
     <mergeCell ref="B21:T21"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:T5"/>
@@ -8056,7 +8074,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="223" t="inlineStr">
         <is>
-          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP 2026  |  1 jul 2026</t>
+          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP 2026  |  2 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -8235,6 +8253,11 @@
           <t>✅ Redistribución aplicada: Bernabéu+Hipódromo+Rubaiyat SP→Naiara · Cobue→Sofía+Naiara · Nuevo Mallorca→latente</t>
         </is>
       </c>
+      <c r="C6" s="261" t="inlineStr">
+        <is>
+          <t>⚠NOW·8jul</t>
+        </is>
+      </c>
       <c r="D6" s="89" t="inlineStr">
         <is>
           <t>RC·mié8</t>
@@ -8364,7 +8387,11 @@
           <t>RC·jue2</t>
         </is>
       </c>
-      <c r="D9" s="103" t="inlineStr"/>
+      <c r="D9" s="89" t="inlineStr">
+        <is>
+          <t>RC·mar7</t>
+        </is>
+      </c>
       <c r="E9" s="103" t="inlineStr"/>
       <c r="F9" s="103" t="inlineStr"/>
       <c r="G9" s="103" t="inlineStr"/>
@@ -8739,7 +8766,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="207" t="inlineStr">
         <is>
@@ -8783,7 +8809,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="211" t="inlineStr">
         <is>
@@ -8878,7 +8903,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>FOCO POR PERSONA — SEMANA 29 JUN - 3 JUL 2026  |  29 jun</t>
+          <t>FOCO POR PERSONA — SEMANA 29 JUN - 5 JUL 2026  |  2 jul 2026</t>
         </is>
       </c>
     </row>
@@ -8968,7 +8993,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Tepeyac: reunión presupuesto esta semana (Raúl+Ale+Paula+PM) · Viuda Aldama: pendiente reunión revisión presupuestos semana del 6 jul (videocall Natalia) · Bernabéu: resolver 3ª persona urgente · LAGOS 132: reunión semanal miércoles (solo PM) · jueves 2jul reunión con Alejandra+Sofía+cliente</t>
+          <t>Tepeyac: reunión presupuesto esta semana (Raúl+Ale+Paula+PM) · Viuda Aldama: pendiente reunión revisión presupuestos semana del 6 jul (videocall Natalia) · Bernabéu: resolver 3ª persona urgente · LAGOS 132: reunión semanal miércoles (solo PM) · jueves 2jul reunión con Alejandra+Sofía+cliente · LAGOS 132: trasladar info grifería/sanitarios a Ferbocar · videocall domótica mar 7jul (Sandra)</t>
         </is>
       </c>
       <c r="E6" s="44" t="inlineStr">
@@ -9125,7 +9150,7 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo) · Viuda de Aldama (equipo)</t>
+          <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo) ·  · Viuda de Aldama (RESP.)</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -9164,7 +9189,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>JOANN: render semanal (cumpliendo bien) · LAGOS 132: reunión miércoles con clientes · COBUE: arrancar renders con renderista nuevo · Puerto Rico: coordinar reunión cliente · LAGOS 132: reunión especial jueves 2jul con Alejandra y cliente</t>
+          <t>JOANN: render semanal (cumpliendo bien) · LAGOS 132: reunión miércoles con clientes · COBUE: arrancar renders con renderista nuevo · Puerto Rico: coordinar reunión cliente · LAGOS 132: reunión especial jueves 2jul con Alejandra y cliente · LAGOS 132: ✅ reunión 2jul bien · videocall domótica mar 7jul con Sandra</t>
         </is>
       </c>
       <c r="E14" s="44" t="inlineStr">
@@ -9298,7 +9323,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>RENDERS — COLA Y ESTADO  |  1 jul 2026</t>
+          <t>RENDERS — COLA Y ESTADO  |  2 jul 2026</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9799,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="236" t="inlineStr">
         <is>
@@ -9824,7 +9848,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="256" t="inlineStr">
         <is>
@@ -9969,11 +9992,10 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="239" t="inlineStr">
         <is>
-          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 1 jul 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 2 jul 2026</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="240" t="inlineStr">
         <is>
@@ -10949,8 +10971,6 @@
       <c r="AE18" s="247" t="inlineStr"/>
       <c r="AF18" s="247" t="inlineStr"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="240" t="inlineStr">
         <is>
@@ -12278,8 +12298,6 @@
       <c r="AE36" s="248" t="inlineStr"/>
       <c r="AF36" s="247" t="inlineStr"/>
     </row>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="240" t="inlineStr">
         <is>
@@ -13050,8 +13068,6 @@
       <c r="AD54" s="247" t="inlineStr"/>
       <c r="AE54" s="247" t="inlineStr"/>
     </row>
-    <row r="55"/>
-    <row r="56"/>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="254" t="inlineStr">
         <is>
@@ -13059,7 +13075,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="139" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 02/07/2026 15:39
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="69">
+  <fonts count="73">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -434,6 +434,30 @@
       <color rgb="001C1C1C"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A5276"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007D4E00"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007D6608"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="004A4A4A"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="55">
     <fill>
@@ -778,7 +802,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="262">
+  <cellXfs count="267">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1531,6 +1555,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="32" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5965,43 +6004,36 @@
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="73" t="inlineStr"/>
-      <c r="B2" s="153" t="n"/>
-      <c r="C2" s="74" t="inlineStr">
+      <c r="C2" s="262" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="D2" s="152" t="n"/>
-      <c r="E2" s="153" t="n"/>
-      <c r="F2" s="75" t="inlineStr">
+      <c r="D2" s="153" t="n"/>
+      <c r="E2" s="263" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="G2" s="152" t="n"/>
-      <c r="H2" s="152" t="n"/>
-      <c r="I2" s="152" t="n"/>
-      <c r="J2" s="153" t="n"/>
-      <c r="K2" s="76" t="inlineStr">
+      <c r="I2" s="264" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="L2" s="152" t="n"/>
-      <c r="M2" s="152" t="n"/>
-      <c r="N2" s="153" t="n"/>
-      <c r="O2" s="77" t="inlineStr">
+      <c r="M2" s="265" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
-      <c r="P2" s="152" t="n"/>
-      <c r="Q2" s="152" t="n"/>
-      <c r="R2" s="153" t="n"/>
+      <c r="R2" s="266" t="inlineStr">
+        <is>
+          <t>OCTUBRE</t>
+        </is>
+      </c>
       <c r="S2" s="78" t="inlineStr"/>
       <c r="T2" s="78" t="inlineStr"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="79" t="inlineStr">
         <is>
           <t>PROYECTO</t>
@@ -6089,7 +6121,7 @@
       </c>
       <c r="R3" s="81" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>6-10</t>
         </is>
       </c>
       <c r="S3" s="81" t="inlineStr">
@@ -7151,24 +7183,23 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="29">
     <mergeCell ref="C26:T26"/>
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C29:T29"/>
     <mergeCell ref="A34:T34"/>
-    <mergeCell ref="O2:R2"/>
     <mergeCell ref="A36:T36"/>
     <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C2:E2"/>
     <mergeCell ref="C10:D10"/>
+    <mergeCell ref="M2:Q2"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="C27:T27"/>
     <mergeCell ref="A25:T25"/>
-    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="I2:L2"/>
     <mergeCell ref="A37:T37"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C2:D2"/>
     <mergeCell ref="M23:R23"/>
     <mergeCell ref="C28:T28"/>
     <mergeCell ref="A33:T33"/>
@@ -7181,7 +7212,7 @@
     <mergeCell ref="A35:T35"/>
     <mergeCell ref="K19:R19"/>
     <mergeCell ref="A38:T38"/>
-    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="E2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7246,43 +7277,36 @@
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="78" t="inlineStr"/>
-      <c r="B2" s="153" t="n"/>
-      <c r="C2" s="74" t="inlineStr">
+      <c r="C2" s="262" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="D2" s="152" t="n"/>
-      <c r="E2" s="153" t="n"/>
-      <c r="F2" s="75" t="inlineStr">
+      <c r="D2" s="153" t="n"/>
+      <c r="E2" s="263" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="G2" s="152" t="n"/>
-      <c r="H2" s="152" t="n"/>
-      <c r="I2" s="152" t="n"/>
-      <c r="J2" s="153" t="n"/>
-      <c r="K2" s="76" t="inlineStr">
+      <c r="I2" s="264" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="L2" s="152" t="n"/>
-      <c r="M2" s="152" t="n"/>
-      <c r="N2" s="153" t="n"/>
-      <c r="O2" s="77" t="inlineStr">
+      <c r="M2" s="265" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
-      <c r="P2" s="152" t="n"/>
-      <c r="Q2" s="152" t="n"/>
-      <c r="R2" s="153" t="n"/>
+      <c r="R2" s="266" t="inlineStr">
+        <is>
+          <t>OCTUBRE</t>
+        </is>
+      </c>
       <c r="S2" s="78" t="inlineStr"/>
       <c r="T2" s="78" t="inlineStr"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="79" t="inlineStr">
         <is>
           <t>PROYECTO</t>
@@ -7370,7 +7394,7 @@
       </c>
       <c r="R3" s="81" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>6-10</t>
         </is>
       </c>
       <c r="S3" s="81" t="inlineStr">
@@ -8012,20 +8036,19 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="21">
     <mergeCell ref="B19:T19"/>
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
-    <mergeCell ref="O2:R2"/>
     <mergeCell ref="B24:T24"/>
     <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C2:E2"/>
     <mergeCell ref="B20:T20"/>
+    <mergeCell ref="M2:Q2"/>
     <mergeCell ref="O10:R10"/>
-    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="I2:L2"/>
     <mergeCell ref="B25:T25"/>
     <mergeCell ref="A27:T27"/>
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
     <mergeCell ref="A18:T18"/>
     <mergeCell ref="B22:T22"/>
     <mergeCell ref="B21:T21"/>
@@ -8034,7 +8057,7 @@
     <mergeCell ref="A32:T32"/>
     <mergeCell ref="B23:T23"/>
     <mergeCell ref="A29:T29"/>
-    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="E2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8099,43 +8122,36 @@
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="78" t="inlineStr"/>
-      <c r="B2" s="153" t="n"/>
-      <c r="C2" s="74" t="inlineStr">
+      <c r="C2" s="262" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="D2" s="152" t="n"/>
-      <c r="E2" s="153" t="n"/>
-      <c r="F2" s="75" t="inlineStr">
+      <c r="D2" s="153" t="n"/>
+      <c r="E2" s="263" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="G2" s="152" t="n"/>
-      <c r="H2" s="152" t="n"/>
-      <c r="I2" s="152" t="n"/>
-      <c r="J2" s="153" t="n"/>
-      <c r="K2" s="76" t="inlineStr">
+      <c r="I2" s="264" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="L2" s="152" t="n"/>
-      <c r="M2" s="152" t="n"/>
-      <c r="N2" s="153" t="n"/>
-      <c r="O2" s="77" t="inlineStr">
+      <c r="M2" s="265" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
-      <c r="P2" s="152" t="n"/>
-      <c r="Q2" s="152" t="n"/>
-      <c r="R2" s="153" t="n"/>
+      <c r="R2" s="266" t="inlineStr">
+        <is>
+          <t>OCTUBRE</t>
+        </is>
+      </c>
       <c r="S2" s="78" t="inlineStr"/>
       <c r="T2" s="78" t="inlineStr"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="79" t="inlineStr">
         <is>
           <t>PROYECTO</t>
@@ -8223,7 +8239,7 @@
       </c>
       <c r="R3" s="81" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>6-10</t>
         </is>
       </c>
       <c r="S3" s="81" t="inlineStr">
@@ -8859,16 +8875,15 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="18">
     <mergeCell ref="A31:T31"/>
     <mergeCell ref="A30:T30"/>
-    <mergeCell ref="O2:R2"/>
     <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="M2:Q2"/>
     <mergeCell ref="A25:T25"/>
-    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="I2:L2"/>
     <mergeCell ref="A27:T27"/>
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
     <mergeCell ref="B22:T22"/>
     <mergeCell ref="A26:T26"/>
     <mergeCell ref="B21:T21"/>
@@ -8877,8 +8892,8 @@
     <mergeCell ref="B23:T23"/>
     <mergeCell ref="A29:T29"/>
     <mergeCell ref="A20:T20"/>
-    <mergeCell ref="K2:N2"/>
     <mergeCell ref="A28:T28"/>
+    <mergeCell ref="E2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 03/07/2026 12:27
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="73">
+  <fonts count="74">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -458,6 +458,12 @@
       <color rgb="004A4A4A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A5276"/>
+      <sz val="7"/>
+    </font>
   </fonts>
   <fills count="55">
     <fill>
@@ -802,7 +808,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="267">
+  <cellXfs count="268">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1570,6 +1576,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1956,7 +1965,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="186" t="inlineStr">
         <is>
-          <t>Semana 29 jun - 5 jul 2026  ·  Actualizado 2 jul 2026</t>
+          <t>Semana 29 jun - 5 jul 2026  ·  Actualizado 3 jul 2026</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2900,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="195" t="inlineStr">
         <is>
-          <t>PM ESTUDIO — MASTER GLOBAL  |  2 julio 2026</t>
+          <t>PM ESTUDIO — MASTER GLOBAL  |  3 julio 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -2988,7 +2997,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
           <t>MONTESQUINZA</t>
@@ -3006,22 +3015,22 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Entregando a Constructora</t>
+          <t>En demolición · planos actualizados</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Entrega proyecto Consultores esta semana</t>
-        </is>
-      </c>
-      <c r="F5" s="42" t="inlineStr">
-        <is>
-          <t>Esta semana</t>
+          <t>Videollamada clientes lunes 6 jul · sin presupuesto de obra cerrado todavía</t>
+        </is>
+      </c>
+      <c r="F5" s="49" t="inlineStr">
+        <is>
+          <t>Lun 6 jul</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Presupuesto de obra pendiente de cerrar · Consultores Proyectos</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
@@ -3034,18 +3043,18 @@
           <t>OBRA</t>
         </is>
       </c>
-      <c r="J5" s="44" t="inlineStr">
-        <is>
-          <t>MÁXIMA</t>
-        </is>
-      </c>
-      <c r="K5" s="44" t="inlineStr">
-        <is>
-          <t>ATENCIÓN MÁXIMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+      <c r="J5" s="53" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="K5" s="53" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
           <t>VIUDA ALDAMA</t>
@@ -3058,27 +3067,27 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Nela (resp.) · Cristina (apoyo) · Sara (puntual)</t>
+          <t>Nela(resp.) · Cristina(apoyo) · Sara(puntual)</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Presupuestos en proceso · acciones en curso hoy</t>
+          <t>Presupuestos en proceso · reunión clienta lunes 6 jul</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Trasladar presupuestos a Natalia · reunión revisión sem 6 jul (videocall)</t>
+          <t>Reunión clienta lunes 6 jul · mail hoy (recap) · AUNA sin precios todavía</t>
         </is>
       </c>
       <c r="F6" s="49" t="inlineStr">
         <is>
-          <t>Sem 6 jul</t>
+          <t>Lun 6 jul</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Presupuesto Raúl pdte · AUNA pdte · Dejaje como alternativa sótano · Natalia vacaciones (online)</t>
+          <t>AUNA sin precios · Raúl valorando · Natalia online (vacaciones)</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -3159,7 +3168,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="45" t="inlineStr">
         <is>
           <t>PEDRAZA</t>
@@ -3177,22 +3186,22 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Prep. montaje</t>
+          <t>Montaje en curso</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Montaje 7-17 jul · del 13 entran tapiceros y cortinas</t>
+          <t>Montaje 6-9 jul (aloj. 7-8) + 13-14 jul · Casa invitados sin montar (sin fecha)</t>
         </is>
       </c>
       <c r="F8" s="49" t="inlineStr">
         <is>
-          <t>7 jul</t>
+          <t>6 jul</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Sin becarias tras 31 jul · conflicto Olatz resuelto si Zahara se retrasa</t>
+          <t>Casa de invitados pendiente de programar · sin fecha concreta aún</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -3273,7 +3282,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
           <t>ZAHARA</t>
@@ -3291,22 +3300,22 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Obra en ejecución</t>
+          <t>Obra en curso · ⚠ serias dudas de que llegue a tiempo</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Montaje 16-17 jul (se intenta mantener) · Raúl pendiente de confirmar</t>
+          <t>Montaje emplazado 14-16 jul · ⚠ serias dudas avance Raúl</t>
         </is>
       </c>
       <c r="F10" s="49" t="inlineStr">
         <is>
-          <t>16 jul</t>
+          <t>14 jul</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Raúl tiene que confirmar que termina obra a tiempo para el 16 jul</t>
+          <t>⚠ Raúl puede no llegar a tiempo · si no hay avance esta semana hay que decidir ya</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -3729,7 +3738,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
+    <row r="18" ht="44" customHeight="1">
       <c r="A18" s="40" t="inlineStr">
         <is>
           <t>SANTANDER VIV</t>
@@ -3747,22 +3756,22 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Obra en curso</t>
+          <t>Presupuestos deco enviados</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Visita HOY 25 jun (Sara+Alejandra) · Deco se habla en sep</t>
-        </is>
-      </c>
-      <c r="F18" s="42" t="inlineStr">
-        <is>
-          <t>Hoy 25 jun</t>
+          <t>Pendiente feedback clientes + cerrar fecha visita</t>
+        </is>
+      </c>
+      <c r="F18" s="49" t="inlineStr">
+        <is>
+          <t>Sin fecha</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>⚠ Deco coincide con Ibiza (ambas Sara)</t>
+          <t>Feedback clientes pendiente · visita sin cerrar</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
@@ -3786,7 +3795,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
+    <row r="19" ht="44" customHeight="1">
       <c r="A19" s="45" t="inlineStr">
         <is>
           <t>ABUBILLA</t>
@@ -3804,12 +3813,12 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>2 temas pendientes antes de septiembre</t>
+          <t>Pendiente aprobación cliente · retomar septiembre</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Cerrar tema económico con cliente + extra de mobiliario solicitado</t>
+          <t>Septiembre: sofá + pendientes de aprobación cliente</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
@@ -3819,7 +3828,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Pendiente cerrar ambos temas · ya no es riesgo activo para Andrea</t>
+          <t>Cliente debe aprobar pendientes · sofá y extras sin cerrar</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -3900,7 +3909,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
+    <row r="21" ht="44" customHeight="1">
       <c r="A21" s="45" t="inlineStr">
         <is>
           <t>TEPEYAC</t>
@@ -3918,22 +3927,22 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>✅ Cliente aprueba distribución · reunión presupuesto pendiente</t>
+          <t>✅ Distribución aprobada · reunión presupuesto pendiente</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Cerrar fecha reunión presupuesto (Raúl+Alejandra+Paula+PM) · demolición prevista agosto</t>
+          <t>Intentar reunión presupuesto viernes 10 jul (pdte cliente y Raúl) · demolición agosto</t>
         </is>
       </c>
       <c r="F21" s="49" t="inlineStr">
         <is>
-          <t>Sin fecha concreta</t>
+          <t>10 jul</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Reunión presupuesto sin fecha cerrada · demolición agosto condicionada a Raúl</t>
+          <t>Cliente y Raúl deben confirmar disponibilidad viernes 10 jul</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -4014,7 +4023,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="40" customHeight="1">
+    <row r="23" ht="44" customHeight="1">
       <c r="A23" s="45" t="inlineStr">
         <is>
           <t>IBIZA</t>
@@ -4032,22 +4041,22 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Obra — parón jul/ago</t>
+          <t>Reunión bien · carpintería actualizada</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Reunión deco 2-3 jul (Sara+Alejandra)</t>
+          <t>Valorar + aceptación carpintería actualizada · montaje 1: hab. ppal 1ª sem oct · montaje 2: resto 7 dic</t>
         </is>
       </c>
       <c r="F23" s="49" t="inlineStr">
         <is>
-          <t>2 jul</t>
+          <t>Oct 2026</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Jul-ago sin obra · ⚠ Deco coincide con Santander (ambas Sara)</t>
+          <t>Carpintería actualizada pdte valoración y aceptación cliente · 2 montajes: oct y dic</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -4060,18 +4069,18 @@
           <t>OBRA</t>
         </is>
       </c>
-      <c r="J23" s="53" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="K23" s="53" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="26" customHeight="1">
+      <c r="J23" s="59" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="K23" s="60" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
       <c r="A24" s="40" t="inlineStr">
         <is>
           <t>CAMINO SUR 70</t>
@@ -4084,27 +4093,27 @@
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Cristina+Nela+becarias</t>
+          <t>Cristina + Nela (sem 20 jul)</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Prep. montaje</t>
+          <t>Montaje en curso por fases</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>Montaje 7-10jul + 16-17jul</t>
+          <t>Sem 6jul: librería+mueble bar+mueble aseo · Sem 13jul: sala TV+isla vestidor · Sem 20jul: Nela cubre (Cristina vacaciones)</t>
         </is>
       </c>
       <c r="F24" s="49" t="inlineStr">
         <is>
-          <t>7 jul</t>
+          <t>6 jul</t>
         </is>
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>Cerrar luminarias · Pedir exterior</t>
+          <t>⚠ Semana 20 jul: Cristina de vacaciones · Nela cubre · pendiente coordinar</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
@@ -4242,7 +4251,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="26" customHeight="1">
+    <row r="27" ht="44" customHeight="1">
       <c r="A27" s="45" t="inlineStr">
         <is>
           <t>VALENCIA</t>
@@ -4260,17 +4269,17 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Obra avanzando</t>
+          <t>Obra en curso · montaje según previsto</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Montaje 21-24jul · Entrega oficial 27jul (Alejandra+Sara+Andrea)</t>
+          <t>Visita semana 13 jul · montaje 21-24 jul · entrega Alejandra martes 28 jul</t>
         </is>
       </c>
       <c r="F27" s="49" t="inlineStr">
         <is>
-          <t>21 jul</t>
+          <t>28 jul</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -4356,7 +4365,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
+    <row r="29" ht="44" customHeight="1">
       <c r="A29" s="45" t="inlineStr">
         <is>
           <t>CAMINO SUR 35</t>
@@ -4369,27 +4378,27 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Nela(resp.)/Olatz</t>
+          <t>Nela (responsable)</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Obra en estructura</t>
+          <t>Modificaciones distribución recibidas hoy</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Reuniones cliente pdte confirmar</t>
-        </is>
-      </c>
-      <c r="F29" s="57" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
+          <t>Reunión 13 jul para ver modificaciones de distribución</t>
+        </is>
+      </c>
+      <c r="F29" s="49" t="inlineStr">
+        <is>
+          <t>13 jul</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Nela asumiendo</t>
+          <t>Modificaciones distribución recibidas 3 jul · pendiente reunión 13 jul</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
@@ -4755,7 +4764,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="26" customHeight="1">
+    <row r="36" ht="44" customHeight="1">
       <c r="A36" s="40" t="inlineStr">
         <is>
           <t>TORRE VALENCIA</t>
@@ -4773,22 +4782,22 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Proyecto</t>
+          <t>Distribución definida · diseños baños pendientes de elección mármoles</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>Actualizar timing Ecobuild · proyecto deco septiembre</t>
-        </is>
-      </c>
-      <c r="F36" s="56" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
+          <t>Checklist capítulos definidos / pendientes (Paula sem que viene) · mármoles → griferías → carpintería</t>
+        </is>
+      </c>
+      <c r="F36" s="49" t="inlineStr">
+        <is>
+          <t>Sem 6 jul</t>
         </is>
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>Ecobuild sin planning cerrado · deco sin empezar</t>
+          <t>Cliente cierra capítulos despacio · mármoles sin decidir · griferías y carpintería en espera · domótica pendiente</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr">
@@ -4801,18 +4810,18 @@
           <t>PROYECTO</t>
         </is>
       </c>
-      <c r="J36" s="59" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="K36" s="60" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1">
+      <c r="J36" s="53" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="K36" s="53" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1">
       <c r="A37" s="45" t="inlineStr">
         <is>
           <t>LA FLORIDA</t>
@@ -4830,22 +4839,22 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Presupuesto+feedback</t>
+          <t>Obra arranca sem 27 jul · termina antes 10 sep</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>Montaje ppios septiembre</t>
-        </is>
-      </c>
-      <c r="F37" s="57" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
+          <t>Obra arranca sem 27 jul · termina antes 10 sep · montaje acto seguido (sep)</t>
+        </is>
+      </c>
+      <c r="F37" s="49" t="inlineStr">
+        <is>
+          <t>27 jul</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Proyecto 'amigo'</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr">
@@ -4858,18 +4867,18 @@
           <t>PROYECTO</t>
         </is>
       </c>
-      <c r="J37" s="59" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="K37" s="60" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="40" customHeight="1">
+      <c r="J37" s="53" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="K37" s="53" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1">
       <c r="A38" s="40" t="inlineStr">
         <is>
           <t>LA RINCONADA</t>
@@ -4887,22 +4896,22 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>✅ Parte presupuesto deco aceptado · compromiso 100% semana que viene</t>
-        </is>
-      </c>
-      <c r="E38" s="180" t="inlineStr">
-        <is>
-          <t>Sem 6 jul</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="inlineStr">
-        <is>
-          <t>⚠ Reunión siguiente semana 13jul lo antes posible — Cristina vacaciones desde 20jul, cerrar lo máximo antes</t>
+          <t>Deco aceptada · revisar pedidos antes de cerrar</t>
+        </is>
+      </c>
+      <c r="E38" s="179" t="inlineStr">
+        <is>
+          <t>Revisar con Olatz + Ale mié 8 jul antes de cerrar pedidos · cosas que no llegan hasta sep</t>
+        </is>
+      </c>
+      <c r="F38" s="49" t="inlineStr">
+        <is>
+          <t>8 jul</t>
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠ Cristina vacaciones desde 20 jul — pedidos deben quedar cerrados antes · algunas entregas hasta finales sep</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr">
@@ -4915,14 +4924,14 @@
           <t>PROYECTO</t>
         </is>
       </c>
-      <c r="J38" s="59" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="K38" s="60" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
+      <c r="J38" s="53" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="K38" s="53" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5049,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="26" customHeight="1">
+    <row r="41" ht="44" customHeight="1">
       <c r="A41" s="45" t="inlineStr">
         <is>
           <t>HERMOSILLA</t>
@@ -5058,22 +5067,22 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Raumplan sin presupuesto</t>
+          <t>Cliente sin prisa · quiere avanzar con Consultores</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>Presionar Raumplan para presupuesto · deco ya presupuestada</t>
-        </is>
-      </c>
-      <c r="F41" s="57" t="inlineStr">
+          <t>⚠ Sin mediciones · cliente debe pagar para hacerlas · pendiente decisión</t>
+        </is>
+      </c>
+      <c r="F41" s="49" t="inlineStr">
         <is>
           <t>Sin fecha</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>Cliente respondió · Raumplan sin presupuesto aún</t>
+          <t>⚠ Sin mediciones (cliente debe pagarlas) · sin eso no se puede avanzar con Consultores</t>
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr">
@@ -5268,7 +5277,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="19" customHeight="1">
+    <row r="45" ht="44" customHeight="1">
       <c r="A45" s="45" t="inlineStr">
         <is>
           <t>VIV PALOMA RD</t>
@@ -5286,22 +5295,22 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Obra en curso</t>
+          <t>Obra retrasada ~6 meses · entrega julio 2027</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Fin obra mar2027 · hablar deco oct/nov</t>
-        </is>
-      </c>
-      <c r="F45" s="57" t="inlineStr">
-        <is>
-          <t>Mar 2027</t>
+          <t>⚠ Arrancar proyecto deco sep/oct 2026 · cadena: deco sep → pedidos ene 2027 → montaje jul 2027</t>
+        </is>
+      </c>
+      <c r="F45" s="49" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>Sin equipo propio allí</t>
+          <t>⚠ Hay que ponerse con deco en sep/oct 2026 · cliente fuera y reuniones difíciles de cuadrar · Olatz responsable</t>
         </is>
       </c>
       <c r="H45" s="8" t="inlineStr">
@@ -5314,14 +5323,14 @@
           <t>ESPERA</t>
         </is>
       </c>
-      <c r="J45" s="59" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="K45" s="59" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
+      <c r="J45" s="53" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="K45" s="53" t="inlineStr">
+        <is>
+          <t>ATENCIÓN ALTA</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5988,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="203" t="inlineStr">
         <is>
-          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP 2026  |  2 jul 2026</t>
+          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP 2026  | 3 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -6015,16 +6024,26 @@
           <t>JULIO</t>
         </is>
       </c>
+      <c r="F2" s="152" t="n"/>
+      <c r="G2" s="152" t="n"/>
+      <c r="H2" s="153" t="n"/>
       <c r="I2" s="264" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
+      <c r="J2" s="152" t="n"/>
+      <c r="K2" s="152" t="n"/>
+      <c r="L2" s="153" t="n"/>
       <c r="M2" s="265" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
+      <c r="N2" s="152" t="n"/>
+      <c r="O2" s="152" t="n"/>
+      <c r="P2" s="152" t="n"/>
+      <c r="Q2" s="153" t="n"/>
       <c r="R2" s="266" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
@@ -6227,14 +6246,19 @@
           <t>Olatz+Paula+becaria</t>
         </is>
       </c>
-      <c r="C6" s="87" t="inlineStr">
-        <is>
-          <t>PEDIDOS</t>
+      <c r="C6" s="88" t="inlineStr">
+        <is>
+          <t>MON·6-9</t>
+        </is>
+      </c>
+      <c r="D6" s="88" t="inlineStr">
+        <is>
+          <t>MON·13-14</t>
         </is>
       </c>
       <c r="E6" s="88" t="inlineStr">
         <is>
-          <t>MONTAJE</t>
+          <t>MONT·13-14</t>
         </is>
       </c>
       <c r="G6" s="101" t="inlineStr"/>
@@ -6271,9 +6295,21 @@
           <t>Paula+Alejandra</t>
         </is>
       </c>
-      <c r="C7" s="103" t="inlineStr"/>
-      <c r="D7" s="103" t="inlineStr"/>
-      <c r="E7" s="103" t="inlineStr"/>
+      <c r="C7" s="260" t="inlineStr">
+        <is>
+          <t>⚠PRE</t>
+        </is>
+      </c>
+      <c r="D7" s="88" t="inlineStr">
+        <is>
+          <t>⚠MON·14-16</t>
+        </is>
+      </c>
+      <c r="E7" s="88" t="inlineStr">
+        <is>
+          <t>MONT·14-16?</t>
+        </is>
+      </c>
       <c r="F7" s="103" t="inlineStr"/>
       <c r="G7" s="88" t="inlineStr">
         <is>
@@ -6317,12 +6353,16 @@
           <t>Sara/Andrea/Nela</t>
         </is>
       </c>
-      <c r="C8" s="90" t="inlineStr">
-        <is>
-          <t>ENTREGA</t>
-        </is>
-      </c>
-      <c r="D8" s="103" t="inlineStr"/>
+      <c r="C8" s="89" t="inlineStr">
+        <is>
+          <t>RC·lun6</t>
+        </is>
+      </c>
+      <c r="D8" s="89" t="inlineStr">
+        <is>
+          <t>RC·lun6</t>
+        </is>
+      </c>
       <c r="E8" s="103" t="inlineStr"/>
       <c r="F8" s="103" t="inlineStr"/>
       <c r="G8" s="103" t="inlineStr"/>
@@ -6357,8 +6397,16 @@
           <t>Cristina(resp.)+Sara</t>
         </is>
       </c>
-      <c r="C9" s="103" t="inlineStr"/>
-      <c r="D9" s="103" t="inlineStr"/>
+      <c r="C9" s="89" t="inlineStr">
+        <is>
+          <t>RC·lun6</t>
+        </is>
+      </c>
+      <c r="D9" s="89" t="inlineStr">
+        <is>
+          <t>RC·lun6</t>
+        </is>
+      </c>
       <c r="E9" s="103" t="inlineStr"/>
       <c r="F9" s="103" t="inlineStr"/>
       <c r="G9" s="103" t="inlineStr"/>
@@ -6394,14 +6442,24 @@
           <t>Cristina+Nela+becarias</t>
         </is>
       </c>
-      <c r="C10" s="87" t="inlineStr">
-        <is>
-          <t>PEDIDOS</t>
-        </is>
-      </c>
-      <c r="E10" s="88" t="inlineStr">
-        <is>
-          <t>MONTAJE</t>
+      <c r="C10" s="88" t="inlineStr">
+        <is>
+          <t>MON·sem6</t>
+        </is>
+      </c>
+      <c r="D10" s="88" t="inlineStr">
+        <is>
+          <t>MON·sem13</t>
+        </is>
+      </c>
+      <c r="E10" s="260" t="inlineStr">
+        <is>
+          <t>MON·sem20</t>
+        </is>
+      </c>
+      <c r="F10" s="88" t="inlineStr">
+        <is>
+          <t>MONT·Nela</t>
         </is>
       </c>
       <c r="G10" s="101" t="inlineStr"/>
@@ -6409,7 +6467,11 @@
       <c r="I10" s="101" t="inlineStr"/>
       <c r="J10" s="101" t="inlineStr"/>
       <c r="K10" s="101" t="inlineStr"/>
-      <c r="L10" s="101" t="inlineStr"/>
+      <c r="L10" s="86" t="inlineStr">
+        <is>
+          <t>EXT+CINE</t>
+        </is>
+      </c>
       <c r="M10" s="101" t="inlineStr"/>
       <c r="N10" s="101" t="inlineStr"/>
       <c r="O10" s="101" t="inlineStr"/>
@@ -6439,8 +6501,16 @@
         </is>
       </c>
       <c r="C11" s="103" t="inlineStr"/>
-      <c r="D11" s="103" t="inlineStr"/>
-      <c r="E11" s="103" t="inlineStr"/>
+      <c r="D11" s="89" t="inlineStr">
+        <is>
+          <t>RC·13jul</t>
+        </is>
+      </c>
+      <c r="E11" s="89" t="inlineStr">
+        <is>
+          <t>RC·13jul</t>
+        </is>
+      </c>
       <c r="F11" s="103" t="inlineStr"/>
       <c r="G11" s="103" t="inlineStr"/>
       <c r="H11" s="103" t="inlineStr"/>
@@ -6478,11 +6548,15 @@
       </c>
       <c r="C12" s="89" t="inlineStr">
         <is>
-          <t>REUNIÓN</t>
+          <t>RC?·10jul</t>
         </is>
       </c>
       <c r="D12" s="103" t="inlineStr"/>
-      <c r="E12" s="103" t="inlineStr"/>
+      <c r="E12" s="89" t="inlineStr">
+        <is>
+          <t>RC?·10jul</t>
+        </is>
+      </c>
       <c r="F12" s="103" t="inlineStr"/>
       <c r="G12" s="103" t="inlineStr"/>
       <c r="H12" s="103" t="inlineStr"/>
@@ -6565,12 +6639,24 @@
           <t>⚠PRE·21jul</t>
         </is>
       </c>
-      <c r="D14" s="103" t="inlineStr"/>
-      <c r="E14" s="103" t="inlineStr"/>
-      <c r="F14" s="103" t="inlineStr"/>
-      <c r="G14" s="88" t="inlineStr">
+      <c r="D14" s="89" t="inlineStr">
+        <is>
+          <t>VISITA</t>
+        </is>
+      </c>
+      <c r="E14" s="267" t="inlineStr">
+        <is>
+          <t>VISITA</t>
+        </is>
+      </c>
+      <c r="F14" s="88" t="inlineStr">
         <is>
           <t>MONTAJE</t>
+        </is>
+      </c>
+      <c r="G14" s="90" t="inlineStr">
+        <is>
+          <t>ENTREGA·28</t>
         </is>
       </c>
       <c r="H14" s="91" t="inlineStr">
@@ -6820,11 +6906,31 @@
       </c>
       <c r="D20" s="103" t="inlineStr"/>
       <c r="E20" s="103" t="inlineStr"/>
-      <c r="F20" s="103" t="inlineStr"/>
-      <c r="G20" s="103" t="inlineStr"/>
-      <c r="H20" s="103" t="inlineStr"/>
-      <c r="I20" s="104" t="inlineStr"/>
-      <c r="J20" s="104" t="inlineStr"/>
+      <c r="F20" s="86" t="inlineStr">
+        <is>
+          <t>OBRA</t>
+        </is>
+      </c>
+      <c r="G20" s="86" t="inlineStr">
+        <is>
+          <t>OBRA</t>
+        </is>
+      </c>
+      <c r="H20" s="86" t="inlineStr">
+        <is>
+          <t>OBRA</t>
+        </is>
+      </c>
+      <c r="I20" s="86" t="inlineStr">
+        <is>
+          <t>OBRA</t>
+        </is>
+      </c>
+      <c r="J20" s="88" t="inlineStr">
+        <is>
+          <t>MONTAJE</t>
+        </is>
+      </c>
       <c r="K20" s="88" t="inlineStr">
         <is>
           <t>MONTAJE</t>
@@ -6863,14 +6969,14 @@
           <t>Cristina</t>
         </is>
       </c>
-      <c r="C21" s="85" t="inlineStr">
-        <is>
-          <t>PROY DECO</t>
-        </is>
-      </c>
-      <c r="D21" s="90" t="inlineStr">
-        <is>
-          <t>ENTREGA·100%</t>
+      <c r="C21" s="89" t="inlineStr">
+        <is>
+          <t>RC·mié8</t>
+        </is>
+      </c>
+      <c r="D21" s="260" t="inlineStr">
+        <is>
+          <t>⚠PED</t>
         </is>
       </c>
       <c r="E21" s="103" t="inlineStr"/>
@@ -7183,22 +7289,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="23">
     <mergeCell ref="C26:T26"/>
+    <mergeCell ref="C29:T29"/>
     <mergeCell ref="A31:T31"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C29:T29"/>
     <mergeCell ref="A34:T34"/>
     <mergeCell ref="A36:T36"/>
     <mergeCell ref="A1:T1"/>
-    <mergeCell ref="C10:D10"/>
     <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="E10:F10"/>
     <mergeCell ref="C27:T27"/>
     <mergeCell ref="A25:T25"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="A37:T37"/>
-    <mergeCell ref="E6:F6"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="M23:R23"/>
     <mergeCell ref="C28:T28"/>
@@ -7207,8 +7309,6 @@
     <mergeCell ref="L18:R18"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:T5"/>
-    <mergeCell ref="L8:R8"/>
-    <mergeCell ref="M9:R9"/>
     <mergeCell ref="A35:T35"/>
     <mergeCell ref="K19:R19"/>
     <mergeCell ref="A38:T38"/>
@@ -7252,7 +7352,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="220" t="inlineStr">
         <is>
-          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP 2026  |  2 jul 2026</t>
+          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP 2026  | 3 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -7288,16 +7388,26 @@
           <t>JULIO</t>
         </is>
       </c>
+      <c r="F2" s="152" t="n"/>
+      <c r="G2" s="152" t="n"/>
+      <c r="H2" s="153" t="n"/>
       <c r="I2" s="264" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
+      <c r="J2" s="152" t="n"/>
+      <c r="K2" s="152" t="n"/>
+      <c r="L2" s="153" t="n"/>
       <c r="M2" s="265" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
+      <c r="N2" s="152" t="n"/>
+      <c r="O2" s="152" t="n"/>
+      <c r="P2" s="152" t="n"/>
+      <c r="Q2" s="153" t="n"/>
       <c r="R2" s="266" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
@@ -8097,7 +8207,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="223" t="inlineStr">
         <is>
-          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP 2026  |  2 jul 2026</t>
+          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP 2026  | 3 jul 2026</t>
         </is>
       </c>
       <c r="B1" s="152" t="n"/>
@@ -8133,16 +8243,26 @@
           <t>JULIO</t>
         </is>
       </c>
+      <c r="F2" s="152" t="n"/>
+      <c r="G2" s="152" t="n"/>
+      <c r="H2" s="153" t="n"/>
       <c r="I2" s="264" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
+      <c r="J2" s="152" t="n"/>
+      <c r="K2" s="152" t="n"/>
+      <c r="L2" s="153" t="n"/>
       <c r="M2" s="265" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
+      <c r="N2" s="152" t="n"/>
+      <c r="O2" s="152" t="n"/>
+      <c r="P2" s="152" t="n"/>
+      <c r="Q2" s="153" t="n"/>
       <c r="R2" s="266" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
@@ -8876,22 +8996,22 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:T5"/>
+    <mergeCell ref="A27:T27"/>
     <mergeCell ref="A31:T31"/>
-    <mergeCell ref="A30:T30"/>
-    <mergeCell ref="A1:T1"/>
     <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="A25:T25"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="A27:T27"/>
     <mergeCell ref="C2:D2"/>
+    <mergeCell ref="B23:T23"/>
     <mergeCell ref="B22:T22"/>
     <mergeCell ref="A26:T26"/>
+    <mergeCell ref="A30:T30"/>
+    <mergeCell ref="A29:T29"/>
+    <mergeCell ref="A25:T25"/>
+    <mergeCell ref="A20:T20"/>
     <mergeCell ref="B21:T21"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:T5"/>
-    <mergeCell ref="B23:T23"/>
-    <mergeCell ref="A29:T29"/>
-    <mergeCell ref="A20:T20"/>
+    <mergeCell ref="I2:L2"/>
     <mergeCell ref="A28:T28"/>
     <mergeCell ref="E2:H2"/>
   </mergeCells>
@@ -8918,7 +9038,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>FOCO POR PERSONA — SEMANA 29 JUN - 5 JUL 2026  |  2 jul 2026</t>
+          <t>FOCO POR PERSONA — SEMANA 29 JUN - 5 JUL 2026  | 3 jul 2026</t>
         </is>
       </c>
     </row>
@@ -9003,12 +9123,12 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Lagos 132 · Alcalá 58 · Supervisión general · Challan · Carbon (gestiona)</t>
+          <t>Lagos 132 · Alcalá 58 · Supervisión general · Challan · Carbon</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Tepeyac: reunión presupuesto esta semana (Raúl+Ale+Paula+PM) · Viuda Aldama: pendiente reunión revisión presupuestos semana del 6 jul (videocall Natalia) · Bernabéu: resolver 3ª persona urgente · LAGOS 132: reunión semanal miércoles (solo PM) · jueves 2jul reunión con Alejandra+Sofía+cliente · LAGOS 132: trasladar info grifería/sanitarios a Ferbocar · videocall domótica mar 7jul (Sandra)</t>
+          <t>ZAHARA: confirmar con Raúl esta semana si llega para 14-16jul · CAMINO SUR 35: reunión 13jul · RINCONADA: revisión con Olatz+Ale mié 8jul · TEPEYAC: intentar viernes 10jul · VIV PALOMA RD: llamar al cliente antes de agosto para arrancar deco sep/oct</t>
         </is>
       </c>
       <c r="E6" s="44" t="inlineStr">
@@ -9035,7 +9155,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Tepeyac: reunión presupuesto esta semana · Pedraza: montaje arranca 7jul · Zahara: montaje 16-17jul · 🏖 Vacaciones 3-21 ago</t>
+          <t>PEDRAZA: montaje 6-9jul (aloj 7-8) + 13-14jul · ZAHARA: emplazado 14-16jul con serias dudas Raúl — confirmar esta semana · TORRE VALENCIA: checklist capítulos sem que viene · TEPEYAC: intentar reunión presupuesto viernes 10jul · LA FLORIDA: obra arranca sem 27jul</t>
         </is>
       </c>
       <c r="E7" s="53" t="inlineStr">
@@ -9057,12 +9177,12 @@
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Montesquinza · Valencia · Santander Viv · Ibiza · Viuda Aldama (apoyo)</t>
+          <t>Montesquinza · Valencia · Santander Viv · Ibiza · Viuda Aldama (puntual)</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>HOY: visita Santander con Alejandra · Ibiza: reunión deco 2-3jul con Alejandra · Valencia: montaje 21-24jul · Viuda Aldama: apoyo puntual a Cristina · VIUDA ALDAMA: apoyo hoy con planos y mail recap Natalia</t>
+          <t>VALENCIA: visita semana 13jul · montaje 21-24jul · entrega Alejandra 28jul · IBIZA: carpintería actualizada pdte valoración · montaje oct y dic · SANTANDER: presupuestos deco enviados pdte feedback+visita</t>
         </is>
       </c>
       <c r="E8" s="53" t="inlineStr">
@@ -9089,7 +9209,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Lagos 105: revisando proyecto · Abubilla: poner límite al cliente · preparar montajes Zahara(16-17jul) y Valencia(21-24jul)</t>
+          <t>LAGOS 105: pendiente 2º presu Jamena + ver con Alejandra · ABUBILLA: sep (sofá + pendientes cliente) · preparar montajes Zahara(14-16jul) y Valencia(21-24jul)</t>
         </is>
       </c>
       <c r="E9" s="53" t="inlineStr">
@@ -9111,12 +9231,12 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Camino Sur 70 · La Rinconada · Viuda de Aldama (responsable)</t>
+          <t>Camino Sur 70 · La Rinconada · Viuda de Aldama (apoyo)</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>VIUDA ALDAMA: ✅ ingeniería deshumectadora realizada · pendiente reunión revisión presupuestos semana del 6 jul (videocall Natalia) · LA RINCONADA: ⚠ entregar presupuesto deco 100% semana que viene (permite pedidos) · reunión siguiente semana 13jul lo antes posible (vacaciones desde 20jul) · Camino Sur 70: montaje 7-10jul · VIUDA ALDAMA HOY: planos sótano a Gaspar · paquete a Raúl · AUNA · cotizar lavandería (Patricia) · mail recap Natalia</t>
+          <t>CAMINO SUR 70: montaje sem6jul + sem13jul · ⚠ sem 20jul Nela cubre (vac Cristina) · LA RINCONADA: ⚠ revisar con Olatz+Ale mié 8jul · cerrar pedidos antes 20jul · VIUDA ALDAMA: apoyo puntual</t>
         </is>
       </c>
       <c r="E10" s="44" t="inlineStr">
@@ -9143,7 +9263,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Pedraza: montaje arranca 7jul · Gamal RD: preparar viaje RD (entra 15jul) · Hermosilla: apoyo a Nela · Camino Sur 35: asumir con Nela</t>
+          <t>PEDRAZA: montaje 6-9jul + 13-14jul · GAMAL RD: preparar viaje RD (arranca 13jul) · HERMOSILLA+CAMINO SUR 35: apoyo a Nela · VIV PALOMA RD: ⚠ arrancar proyecto deco sep/oct — cliente hay que llamarlo pronto</t>
         </is>
       </c>
       <c r="E11" s="53" t="inlineStr">
@@ -9165,12 +9285,12 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Camino Sur 70 (apoyo) ·  · Viuda de Aldama (RESP.)</t>
+          <t>Montesquinza · Camino Sur 35 (resp.) · Hermosilla (resp.) · Viuda Aldama (resp.) · Camino Sur 70 (cubre sem 20jul)</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Camino Sur 70: montaje esta semana 7-10jul · Hermosilla+Camino Sur 35: responsable · ⚠ No coge vacaciones agosto — disponible · VIUDA ALDAMA: HOY enviar planos sótano a Gaspar + paquete a Raúl + mail a Natalia recap</t>
+          <t>VIUDA ALDAMA: reunión clienta lunes 6jul · pendiente AUNA · CAMINO SUR 35: reunión 13jul (modificaciones distribución recibidas hoy) · RINCONADA: revisión con Cristina+Ale mié 8jul · CAMINO SUR 70: cubrir semana del 20jul (Cristina vacaciones)</t>
         </is>
       </c>
       <c r="E12" s="53" t="inlineStr">
@@ -9338,7 +9458,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>RENDERS — COLA Y ESTADO  |  2 jul 2026</t>
+          <t>RENDERS — COLA Y ESTADO  | 3 jul 2026</t>
         </is>
       </c>
     </row>
@@ -10007,7 +10127,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="239" t="inlineStr">
         <is>
-          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 2 jul 2026</t>
+          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 3 jul 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 07/07/2026 15:48
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -7100,8 +7100,16 @@
           <t>MON·13-14</t>
         </is>
       </c>
-      <c r="G6" s="293" t="inlineStr"/>
-      <c r="H6" s="293" t="inlineStr"/>
+      <c r="G6" s="88" t="inlineStr">
+        <is>
+          <t>MON·Paula+Olatz</t>
+        </is>
+      </c>
+      <c r="H6" s="87" t="inlineStr">
+        <is>
+          <t>REMATES·Olatz</t>
+        </is>
+      </c>
       <c r="I6" s="293" t="inlineStr"/>
       <c r="J6" s="293" t="inlineStr"/>
       <c r="K6" s="293" t="inlineStr"/>
@@ -7142,12 +7150,12 @@
       </c>
       <c r="E7" s="88" t="inlineStr">
         <is>
-          <t>MON·16-17</t>
-        </is>
-      </c>
-      <c r="F7" s="91" t="inlineStr">
-        <is>
-          <t>ALE·24</t>
+          <t>MON·16-17·Ale+Paula</t>
+        </is>
+      </c>
+      <c r="F7" s="88" t="inlineStr">
+        <is>
+          <t>MON·23-27·Ale+Paula→Ale</t>
         </is>
       </c>
       <c r="G7" s="293" t="inlineStr"/>
@@ -7430,12 +7438,12 @@
       </c>
       <c r="F14" s="88" t="inlineStr">
         <is>
-          <t>MONTAJE</t>
-        </is>
-      </c>
-      <c r="G14" s="91" t="inlineStr">
-        <is>
-          <t>ALE·27</t>
+          <t>MON·21-24·Sara+Andrea</t>
+        </is>
+      </c>
+      <c r="G14" s="90" t="inlineStr">
+        <is>
+          <t>PRES·28jul</t>
         </is>
       </c>
       <c r="H14" s="299" t="inlineStr">
@@ -8021,12 +8029,12 @@
       </c>
       <c r="E35" s="88" t="inlineStr">
         <is>
-          <t>MON·16-17</t>
-        </is>
-      </c>
-      <c r="F35" s="91" t="inlineStr">
-        <is>
-          <t>ALE·24</t>
+          <t>MON·16-17·Ale+Paula</t>
+        </is>
+      </c>
+      <c r="F35" s="88" t="inlineStr">
+        <is>
+          <t>MON·23-27·Ale+Paula→Ale</t>
         </is>
       </c>
     </row>
@@ -8044,6 +8052,16 @@
       <c r="E36" s="88" t="inlineStr">
         <is>
           <t>MON·13-14</t>
+        </is>
+      </c>
+      <c r="G36" s="88" t="inlineStr">
+        <is>
+          <t>MON·Paula+Olatz</t>
+        </is>
+      </c>
+      <c r="H36" s="87" t="inlineStr">
+        <is>
+          <t>REMATES·Olatz</t>
         </is>
       </c>
     </row>
@@ -8825,7 +8843,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="108" t="inlineStr">
         <is>
@@ -8917,7 +8934,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="113" t="inlineStr">
         <is>
@@ -8972,7 +8988,6 @@
       <c r="S27" s="117" t="inlineStr"/>
       <c r="T27" s="117" t="inlineStr"/>
     </row>
-    <row r="28"/>
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="112" t="inlineStr">
         <is>
@@ -9123,12 +9138,12 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Supervisión todos · Joann (compromiso renders) · Zahara · Gamal RD · Valencia · entregas finales</t>
+          <t>Supervisión todos · Zahara · Gamal RD · Valencia · Ibiza</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>GAMAL RD: 15-23jul (viaje RD con Olatz y Sofía) · ZAHARA: visita 24jul (fin de semana) · VALENCIA: entrega oficial 27jul (martes) · ⚠ Riesgo menor: vuelo internacional 23 + desplazamiento 24 + entrega 27</t>
+          <t>ZAHARA: 16-17jul (con Paula) + 18-23jul GAMAL RD + 24jul vuelta Zahara (con Paula) + 25-27jul sola en Zahara · VALENCIA: presentación oficial 28jul · Agenda muy comprimida 16-28jul — sin margen</t>
         </is>
       </c>
       <c r="E4" s="53" t="inlineStr">
@@ -9184,12 +9199,12 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Pedraza · Zahara · La Florida · Tepeyac · Torre Valencia</t>
+          <t>Pedraza · Zahara · Valencia(montaje) · Tepeyac</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>PEDRAZA: montaje 13-14jul (con Olatz) + 15jul sola · ZAHARA: montaje 16-17jul con Andrea · ⚠ tránsito directo Pedraza→Zahara — un día de margen el 15</t>
+          <t>ZAHARA: montaje 16-17jul (con Ale) + 23-24jul (con Ale) · PEDRAZA: montaje 27-31jul con Olatz · VALENCIA: montaje 21-24jul con Sara+Andrea · Vacaciones 3-21ago</t>
         </is>
       </c>
       <c r="E7" s="53" t="inlineStr">
@@ -9238,12 +9253,12 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Lagos 105 · Zahara(montaje) · Valencia(montaje) · Abubilla</t>
+          <t>Lagos 105 · Valencia(montaje) · Abubilla</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>ZAHARA: montaje 16-17jul con Paula · VALENCIA: montaje 21-24jul con Sara · margen 18-20 entre ambos</t>
+          <t>VALENCIA: montaje 21-24jul con Sara · Lagos 105: actualizando proyecto · Vacaciones 3-21ago</t>
         </is>
       </c>
       <c r="E9" s="53" t="inlineStr">
@@ -9297,7 +9312,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>PEDRAZA: montaje 13-14jul con Paula · GAMAL RD: entra 15jul viaje RD (hasta 23jul) · ⚠ sale directo de Pedraza a Gamal</t>
+          <t>GAMAL RD: viaje RD 15-23jul · PEDRAZA: montaje 27-31jul con Paula · remates deco 1ª sem ago (sola) · Vacaciones 17-28ago</t>
         </is>
       </c>
       <c r="E11" s="53" t="inlineStr">
@@ -9517,7 +9532,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="240" t="inlineStr">
         <is>
@@ -10493,8 +10507,6 @@
       <c r="AE18" s="247" t="inlineStr"/>
       <c r="AF18" s="247" t="inlineStr"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="240" t="inlineStr">
         <is>
@@ -11822,8 +11834,6 @@
       <c r="AE36" s="248" t="inlineStr"/>
       <c r="AF36" s="247" t="inlineStr"/>
     </row>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="240" t="inlineStr">
         <is>
@@ -12594,8 +12604,6 @@
       <c r="AD54" s="247" t="inlineStr"/>
       <c r="AE54" s="247" t="inlineStr"/>
     </row>
-    <row r="55"/>
-    <row r="56"/>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="254" t="inlineStr">
         <is>
@@ -12603,7 +12611,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="139" t="inlineStr">
         <is>
@@ -13034,7 +13041,7 @@
       </c>
       <c r="B9" s="98" t="inlineStr">
         <is>
-          <t>Sofía+Olatz+Ale</t>
+          <t>Sofía(13)+Olatz(15)+Ale(18)</t>
         </is>
       </c>
       <c r="C9" s="292" t="inlineStr"/>
@@ -13380,7 +13387,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="108" t="inlineStr">
         <is>
@@ -13424,7 +13430,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="113" t="inlineStr">
         <is>
@@ -13475,7 +13480,6 @@
       <c r="S24" s="117" t="inlineStr"/>
       <c r="T24" s="117" t="inlineStr"/>
     </row>
-    <row r="25"/>
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="112" t="inlineStr">
         <is>
@@ -14057,7 +14061,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="236" t="inlineStr">
         <is>
@@ -14107,7 +14110,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="256" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel actualizado automaticamente — 07/07/2026 16:06
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -2127,11 +2127,10 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="186" t="inlineStr">
         <is>
-          <t>Semana 29 jun - 6 jul 2026  ·  Actualizado 6 jul 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Semana 29 jun - 7 jul 2026  ·  Actualizado 7 jul 2026</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="187" t="inlineStr">
         <is>
@@ -3003,7 +3002,6 @@
       </c>
     </row>
     <row r="60" ht="44" customHeight="1"/>
-    <row r="61"/>
     <row r="62" ht="16" customHeight="1"/>
   </sheetData>
   <mergeCells count="27">
@@ -6200,7 +6198,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="62" t="inlineStr">
         <is>
@@ -6800,7 +6797,6 @@
       <c r="N65" s="285" t="inlineStr"/>
       <c r="O65" s="285" t="inlineStr"/>
     </row>
-    <row r="66"/>
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="269" t="inlineStr">
         <is>
@@ -6855,7 +6851,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="286" t="inlineStr">
         <is>
-          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP·OCT 2026  |  6 jul 2026</t>
+          <t>PLANNING VIVIENDA — JUN·JUL·AGO·SEP·OCT 2026  |  7 jul 2026</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7859,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="108" t="inlineStr">
         <is>
@@ -7939,7 +7934,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="14" customHeight="1">
       <c r="A31" s="112" t="inlineStr">
         <is>
@@ -8013,7 +8007,6 @@
       <c r="S32" s="117" t="inlineStr"/>
       <c r="T32" s="117" t="inlineStr"/>
     </row>
-    <row r="33"/>
     <row r="34" ht="14" customHeight="1">
       <c r="A34" s="112" t="inlineStr">
         <is>
@@ -8184,7 +8177,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="301" t="inlineStr">
         <is>
-          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP·OCT 2026  |  6 jul 2026</t>
+          <t>PLANNING HOTELES — JUN·JUL·AGO·SEP·OCT 2026  |  7 jul 2026</t>
         </is>
       </c>
     </row>
@@ -9087,7 +9080,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>FOCO POR PERSONA — SEMANA 29 JUN - 5 JUL 2026  | 6 jul 2026</t>
+          <t>FOCO POR PERSONA — SEMANA 29 JUN - 5 JUL 2026  | 7 jul 2026</t>
         </is>
       </c>
     </row>
@@ -9528,10 +9521,11 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="239" t="inlineStr">
         <is>
-          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 6 jul 2026</t>
-        </is>
-      </c>
-    </row>
+          <t>VACACIONES EQUIPO — VERANO 2026  |  Actualizado 7 jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="240" t="inlineStr">
         <is>
@@ -12673,7 +12667,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="304" t="inlineStr">
         <is>
-          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP·OCT 2026  |  6 jul 2026</t>
+          <t>PLANNING RESTAURANTES — JUN·JUL·AGO·SEP·OCT 2026  |  7 jul 2026</t>
         </is>
       </c>
     </row>
@@ -13585,7 +13579,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="228" t="inlineStr">
         <is>
-          <t>RENDERS — COLA Y ESTADO  | 6 jul 2026</t>
+          <t>RENDERS — COLA Y ESTADO  | 7 jul 2026</t>
         </is>
       </c>
     </row>

</xml_diff>